<commit_message>
Publish EconSheet 261015 (October 15, 2026)
</commit_message>
<xml_diff>
--- a/files/EconSheet.xlsx
+++ b/files/EconSheet.xlsx
@@ -8,44 +8,44 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.0.130\Documents\Business\EconSheet\FREDData\ToDistribute\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A9C3DE64-25FF-4B30-9977-F30D16B0E1DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{CD806712-3D06-4078-8015-90D422AA8E9A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5295" windowWidth="29040" windowHeight="15720" xr2:uid="{626B6F87-D248-4394-AE80-16238AEFE6A8}"/>
+    <workbookView xWindow="-28920" yWindow="5295" windowWidth="29040" windowHeight="15720" xr2:uid="{0AFC93D1-2EB9-43FD-BE55-A1659D96EA6D}"/>
   </bookViews>
   <sheets>
-    <sheet name="261010 EconSheet" sheetId="1" r:id="rId1"/>
+    <sheet name="261015 EconSheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId2"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'261010 EconSheet'!$A$28:$AF$33</definedName>
-    <definedName name="Conditions" localSheetId="0">'261010 EconSheet'!$AH$3:$AH$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'261015 EconSheet'!$A$28:$AF$33</definedName>
+    <definedName name="Conditions" localSheetId="0">'261015 EconSheet'!$AH$3:$AH$96</definedName>
     <definedName name="CurrDates">[1]Currencies!$A$8:$A$14337</definedName>
     <definedName name="DataStart">'[1]Retrieved Data'!$A$1</definedName>
-    <definedName name="DataTable" localSheetId="0">'261010 EconSheet'!$G$4:$AD$96</definedName>
-    <definedName name="DataTableStart" localSheetId="0">'261010 EconSheet'!$G$4</definedName>
-    <definedName name="DatesAndSeries" localSheetId="0">'261010 EconSheet'!$E$4:$F$96</definedName>
+    <definedName name="DataTable" localSheetId="0">'261015 EconSheet'!$G$4:$AD$96</definedName>
+    <definedName name="DataTableStart" localSheetId="0">'261015 EconSheet'!$G$4</definedName>
+    <definedName name="DatesAndSeries" localSheetId="0">'261015 EconSheet'!$E$4:$F$96</definedName>
     <definedName name="DatesAndSeries">[1]EconSheet!$E$4:$F$96</definedName>
-    <definedName name="DatesCol" localSheetId="0">'261010 EconSheet'!$E$4:$E$96</definedName>
+    <definedName name="DatesCol" localSheetId="0">'261015 EconSheet'!$E$4:$E$96</definedName>
     <definedName name="DatesCol">[1]EconSheet!$E$4:$E$96</definedName>
-    <definedName name="ESSeries" localSheetId="0">'261010 EconSheet'!$B$4:$B$103</definedName>
-    <definedName name="ForceAll" localSheetId="0">'261010 EconSheet'!#REF!</definedName>
+    <definedName name="ESSeries" localSheetId="0">'261015 EconSheet'!$B$4:$B$103</definedName>
+    <definedName name="ForceAll" localSheetId="0">'261015 EconSheet'!#REF!</definedName>
     <definedName name="FormatOptions">[1]Calculations!$U$3:$U$14</definedName>
-    <definedName name="FormatTable" localSheetId="0">'261010 EconSheet'!$A$1:$AD$96</definedName>
+    <definedName name="FormatTable" localSheetId="0">'261015 EconSheet'!$A$1:$AD$96</definedName>
     <definedName name="PPIGreen">'[1]Producer Price Archive'!$AB$8:$AD$1023</definedName>
     <definedName name="PPIRaw">'[1]Producer Price Archive'!$B$7:$F$1023</definedName>
     <definedName name="PPIRed">'[1]Producer Price Archive'!$AF$8:$AH$1023</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'261010 EconSheet'!$F$1:$AD$54,'261010 EconSheet'!$F$56:$AD$96</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'261015 EconSheet'!$F$1:$AD$54,'261015 EconSheet'!$F$56:$AD$96</definedName>
     <definedName name="ReleaseData">[1]ReleaseDates!$A$2:$E$1882</definedName>
     <definedName name="ReleaseDates">[1]ReleaseDates!$A$2:$A$1898</definedName>
     <definedName name="SDSeries">[1]SeriesData!$A$2:$A$76</definedName>
     <definedName name="SeriesLookup">'[1]Retrieved Data'!$A$1:$ET$1</definedName>
-    <definedName name="SpFormat1" localSheetId="0">'261010 EconSheet'!$AH$131</definedName>
-    <definedName name="SpFormat2" localSheetId="0">'261010 EconSheet'!$AH$136</definedName>
-    <definedName name="TrueFalse" localSheetId="0">'261010 EconSheet'!#REF!</definedName>
+    <definedName name="SpFormat1" localSheetId="0">'261015 EconSheet'!$AH$131</definedName>
+    <definedName name="SpFormat2" localSheetId="0">'261015 EconSheet'!$AH$136</definedName>
+    <definedName name="TrueFalse" localSheetId="0">'261015 EconSheet'!#REF!</definedName>
     <definedName name="TrueFalse">[1]EconSheet!$AU$1:$AU$2</definedName>
-    <definedName name="WholeTable" localSheetId="0">'261010 EconSheet'!$F$1:$AD$96</definedName>
+    <definedName name="WholeTable" localSheetId="0">'261015 EconSheet'!$F$1:$AD$96</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -68,6 +68,55 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Ron Levin</author>
+  </authors>
+  <commentList>
+    <comment ref="AD42" authorId="0" shapeId="0" xr:uid="{4AE5D1B4-1B5F-423B-B86F-2013EC0A88C8}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>New Value</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AD43" authorId="0" shapeId="0" xr:uid="{12674E6F-628F-4207-BB1C-6FB294A48C89}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>New Value</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AD45" authorId="0" shapeId="0" xr:uid="{FB9E791C-7FD0-4AD2-96FB-5382E7D7349D}">
+      <text>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>New Value</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -631,7 +680,7 @@
     <t>Green if</t>
   </si>
   <si>
-    <t>Next Update: 10/13/26</t>
+    <t>Next Update: 10/15/26</t>
   </si>
   <si>
     <t>Next Update</t>
@@ -657,7 +706,7 @@
     <numFmt numFmtId="167" formatCode="mmm"/>
     <numFmt numFmtId="168" formatCode="m/d/yyyy\ h:mm\ AM/PM"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -751,6 +800,12 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -778,7 +833,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -804,17 +859,45 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top style="thick">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thick">
+        <color indexed="64"/>
+      </left>
+      <right style="thick">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="71">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="4" fillId="2" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -886,7 +969,9 @@
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -906,7 +991,7 @@
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{2CDF5CA3-93E2-44C1-BA1E-DE369082333B}"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{0FD409DF-9518-4606-9E86-0965EEF01158}"/>
   </cellStyles>
   <dxfs count="237">
     <dxf>
@@ -2091,7 +2176,24 @@
       <font>
         <b/>
         <i val="0"/>
+        <color rgb="FF711204"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
         <color rgb="FF10651B"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
       </font>
     </dxf>
     <dxf>
@@ -2103,7 +2205,21 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF10651B"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF711204"/>
       </font>
     </dxf>
     <dxf>
@@ -2115,14 +2231,14 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF711204"/>
+        <color theme="0"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <color theme="0"/>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF711204"/>
       </font>
     </dxf>
     <dxf>
@@ -2134,46 +2250,20 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF711204"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF10651B"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF711204"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <color theme="0"/>
       </font>
     </dxf>
     <dxf>
       <border>
         <left style="thin">
-          <color indexed="17"/>
+          <color indexed="10"/>
         </left>
       </border>
     </dxf>
     <dxf>
       <border>
         <left style="thin">
-          <color indexed="10"/>
+          <color indexed="17"/>
         </left>
       </border>
     </dxf>
@@ -2186,7 +2276,19 @@
       <font>
         <b/>
         <i val="0"/>
+        <color rgb="FF711204"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
         <color rgb="FF10651B"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
       </font>
     </dxf>
     <dxf>
@@ -2198,7 +2300,21 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF10651B"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF711204"/>
       </font>
     </dxf>
     <dxf>
@@ -2210,9 +2326,21 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
         <color rgb="FF711204"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF10651B"/>
       </font>
     </dxf>
     <dxf>
@@ -2224,7 +2352,19 @@
       <font>
         <b/>
         <i val="0"/>
+        <color rgb="FF711204"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
         <color rgb="FF10651B"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
       </font>
     </dxf>
     <dxf>
@@ -2236,7 +2376,21 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF10651B"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF711204"/>
       </font>
     </dxf>
     <dxf>
@@ -2248,9 +2402,21 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
         <color rgb="FF711204"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF10651B"/>
       </font>
     </dxf>
     <dxf>
@@ -2262,19 +2428,7 @@
       <font>
         <b/>
         <i val="0"/>
-        <color rgb="FF10651B"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
         <color rgb="FF711204"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
       </font>
     </dxf>
     <dxf>
@@ -2282,75 +2436,6 @@
         <b/>
         <i val="0"/>
         <color rgb="FF10651B"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF711204"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF10651B"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF711204"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF10651B"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF711204"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF10651B"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF711204"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
       </font>
     </dxf>
     <dxf>
@@ -2542,7 +2627,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{E94B10F3-F016-48B4-8E42-A5B2D2DD8B9F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B18524DF-E19E-490F-BDC0-0A4874637349}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2587,7 +2672,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0791CA5-2F17-4FD3-9DE2-AF8496D411F5}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{90AE3F45-D422-4FBE-A976-CF156A3676E4}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2912,7 +2997,7 @@
         </row>
         <row r="42">
           <cell r="E42">
-            <v>46309.401261574065</v>
+            <v>46336.380891203706</v>
           </cell>
           <cell r="F42" t="str">
             <v>Consumer Price Index (% Δ YoY)</v>
@@ -2920,7 +3005,7 @@
         </row>
         <row r="43">
           <cell r="E43">
-            <v>46309.401180555549</v>
+            <v>46336.380891203706</v>
           </cell>
           <cell r="F43" t="str">
             <v>Food (% Δ YoY)</v>
@@ -2928,7 +3013,7 @@
         </row>
         <row r="44">
           <cell r="E44">
-            <v>46309.401284722233</v>
+            <v>46336.380891203706</v>
           </cell>
           <cell r="F44" t="str">
             <v>Energy (% Δ YoY)</v>
@@ -2936,7 +3021,7 @@
         </row>
         <row r="45">
           <cell r="E45">
-            <v>46309.401307870372</v>
+            <v>46336.380891203706</v>
           </cell>
           <cell r="F45" t="str">
             <v>All Items Less Food &amp; Energy (% Δ YoY)</v>
@@ -3132,7 +3217,7 @@
         </row>
         <row r="74">
           <cell r="E74">
-            <v>46308.678148148145</v>
+            <v>46311.678611111114</v>
           </cell>
           <cell r="F74" t="str">
             <v>3-Month Treasury Bills, Secondary market (%)</v>
@@ -3140,7 +3225,7 @@
         </row>
         <row r="75">
           <cell r="E75">
-            <v>46308.678460648138</v>
+            <v>46311.678460648138</v>
           </cell>
           <cell r="F75" t="str">
             <v>Bank Prime Rate (%)</v>
@@ -3148,7 +3233,7 @@
         </row>
         <row r="76">
           <cell r="E76">
-            <v>46308.678194444452</v>
+            <v>46311.678576388891</v>
           </cell>
           <cell r="F76" t="str">
             <v>2-yr. Treasury Bond Yield at Constant Maturity (%)</v>
@@ -3156,7 +3241,7 @@
         </row>
         <row r="77">
           <cell r="E77">
-            <v>46308.678171296298</v>
+            <v>46311.678483796306</v>
           </cell>
           <cell r="F77" t="str">
             <v>10-yr. Treasury Bond Yield at Constant Maturity (%)</v>
@@ -3164,7 +3249,7 @@
         </row>
         <row r="78">
           <cell r="E78">
-            <v>46308.710868055554</v>
+            <v>46311.710868055554</v>
           </cell>
           <cell r="F78" t="str">
             <v>10 Yr - 2 Yr Treasury Spread - Const Maturity %</v>
@@ -3172,7 +3257,7 @@
         </row>
         <row r="79">
           <cell r="E79">
-            <v>46308.678171296298</v>
+            <v>46311.678437499999</v>
           </cell>
           <cell r="F79" t="str">
             <v>10-yr. Treasury Bond Yield at Const. Mat. Inflation Indexed (%)</v>
@@ -3180,7 +3265,7 @@
         </row>
         <row r="80">
           <cell r="E80">
-            <v>46308.678217592591</v>
+            <v>46311.678587962961</v>
           </cell>
           <cell r="F80" t="str">
             <v>30-yr. Treasury Bond Yield at Constant Maturity (%)</v>
@@ -3188,7 +3273,7 @@
         </row>
         <row r="81">
           <cell r="E81">
-            <v>46308.710856481484</v>
+            <v>46311.710844907415</v>
           </cell>
           <cell r="F81" t="str">
             <v>10 Yr - 3 Month Treasury Spread - Const Maturity %</v>
@@ -3196,7 +3281,7 @@
         </row>
         <row r="82">
           <cell r="E82">
-            <v>46308.678252314814</v>
+            <v>46314.678506944445</v>
           </cell>
           <cell r="F82" t="str">
             <v>USD/EUR Exchange Rate - Last Day of Month</v>
@@ -3204,7 +3289,7 @@
         </row>
         <row r="83">
           <cell r="E83">
-            <v>46308.678391203706</v>
+            <v>46314.67859953703</v>
           </cell>
           <cell r="F83" t="str">
             <v>Nominal Broad USD Index - Last Day of Month</v>
@@ -45592,10 +45677,10 @@
             <v>46309</v>
           </cell>
           <cell r="C162" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D162">
-            <v>46309</v>
+            <v>0</v>
           </cell>
           <cell r="E162">
             <v>162</v>
@@ -48431,10 +48516,10 @@
             <v>46308</v>
           </cell>
           <cell r="C329" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D329">
-            <v>46308</v>
+            <v>0</v>
           </cell>
           <cell r="E329">
             <v>329</v>
@@ -53208,10 +53293,10 @@
             <v>46308</v>
           </cell>
           <cell r="C610" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D610">
-            <v>46308</v>
+            <v>0</v>
           </cell>
           <cell r="E610">
             <v>610</v>
@@ -53225,10 +53310,10 @@
             <v>46309</v>
           </cell>
           <cell r="C611" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D611">
-            <v>46309</v>
+            <v>0</v>
           </cell>
           <cell r="E611">
             <v>611</v>
@@ -53242,10 +53327,10 @@
             <v>46310</v>
           </cell>
           <cell r="C612" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D612">
-            <v>46310</v>
+            <v>0</v>
           </cell>
           <cell r="E612">
             <v>612</v>
@@ -58733,10 +58818,10 @@
             <v>46308</v>
           </cell>
           <cell r="C935" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D935">
-            <v>46308</v>
+            <v>0</v>
           </cell>
           <cell r="E935">
             <v>935</v>
@@ -58750,10 +58835,10 @@
             <v>46309</v>
           </cell>
           <cell r="C936" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D936">
-            <v>46309</v>
+            <v>0</v>
           </cell>
           <cell r="E936">
             <v>936</v>
@@ -58767,10 +58852,10 @@
             <v>46310</v>
           </cell>
           <cell r="C937" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D937">
-            <v>46310</v>
+            <v>0</v>
           </cell>
           <cell r="E937">
             <v>937</v>
@@ -68304,10 +68389,10 @@
             <v>46307</v>
           </cell>
           <cell r="C1498" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1498">
-            <v>46307</v>
+            <v>0</v>
           </cell>
           <cell r="E1498">
             <v>1498</v>
@@ -68321,10 +68406,10 @@
             <v>46308</v>
           </cell>
           <cell r="C1499" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1499">
-            <v>46308</v>
+            <v>0</v>
           </cell>
           <cell r="E1499">
             <v>1499</v>
@@ -68338,10 +68423,10 @@
             <v>46309</v>
           </cell>
           <cell r="C1500" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1500">
-            <v>46309</v>
+            <v>0</v>
           </cell>
           <cell r="E1500">
             <v>1500</v>
@@ -68355,10 +68440,10 @@
             <v>46310</v>
           </cell>
           <cell r="C1501" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1501">
-            <v>46310</v>
+            <v>0</v>
           </cell>
           <cell r="E1501">
             <v>1501</v>
@@ -73914,10 +73999,10 @@
             <v>46308</v>
           </cell>
           <cell r="C1828" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1828">
-            <v>46308</v>
+            <v>0</v>
           </cell>
           <cell r="E1828">
             <v>1828</v>
@@ -73931,10 +74016,10 @@
             <v>46309</v>
           </cell>
           <cell r="C1829" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1829">
-            <v>46309</v>
+            <v>0</v>
           </cell>
           <cell r="E1829">
             <v>1829</v>
@@ -73948,10 +74033,10 @@
             <v>46310</v>
           </cell>
           <cell r="C1830" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1830">
-            <v>46310</v>
+            <v>0</v>
           </cell>
           <cell r="E1830">
             <v>1830</v>
@@ -75244,19 +75329,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9CBDDA8C-B250-47A1-9A47-3E7656BE6E44}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98B26542-9572-4EB5-BC42-710A3C09049A}">
   <sheetPr codeName="Sheet22">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:AH144"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15.75" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:AU145"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.28515625" style="1" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="2" max="2" width="28.140625" style="1" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="3" max="3" width="77.140625" style="1" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="4" max="4" width="17.42578125" style="2" hidden="1" customWidth="1" outlineLevel="1"/>
-    <col min="5" max="5" width="21" style="2" bestFit="1" customWidth="1" collapsed="1"/>
-    <col min="6" max="6" width="61.42578125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="8.28515625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="2" max="2" width="28.140625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="3" max="3" width="77.140625" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="4" max="4" width="17.42578125" hidden="1" customWidth="1" outlineLevel="1"/>
+    <col min="5" max="5" width="21" bestFit="1" customWidth="1" collapsed="1"/>
+    <col min="6" max="6" width="61.42578125" customWidth="1"/>
     <col min="7" max="8" width="10.28515625" hidden="1" customWidth="1" outlineLevel="1"/>
     <col min="9" max="9" width="9.28515625" hidden="1" customWidth="1" outlineLevel="1"/>
     <col min="10" max="16" width="10.28515625" hidden="1" customWidth="1" outlineLevel="1"/>
@@ -75271,13 +75356,13 @@
     <col min="34" max="34" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" s="68" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="70"/>
-      <c r="B1" s="70"/>
-      <c r="C1" s="70"/>
+    <row r="1" spans="1:34" s="70" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="72"/>
+      <c r="B1" s="72"/>
+      <c r="C1" s="72"/>
       <c r="D1" s="37"/>
       <c r="E1" s="37"/>
-      <c r="F1" s="70" t="s">
+      <c r="F1" s="72" t="s">
         <v>190</v>
       </c>
       <c r="G1" s="34">
@@ -75353,7 +75438,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:34" s="68" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:34" s="70" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="25"/>
       <c r="B2" s="25"/>
       <c r="C2" s="25" t="s">
@@ -75368,93 +75453,93 @@
       <c r="F2" s="25" t="s">
         <v>186</v>
       </c>
-      <c r="G2" s="69">
+      <c r="G2" s="71">
         <v>45566</v>
       </c>
-      <c r="H2" s="69">
+      <c r="H2" s="71">
         <v>45597</v>
       </c>
-      <c r="I2" s="69">
+      <c r="I2" s="71">
         <v>45627</v>
       </c>
-      <c r="J2" s="69">
+      <c r="J2" s="71">
         <v>45658</v>
       </c>
-      <c r="K2" s="69">
+      <c r="K2" s="71">
         <v>45689</v>
       </c>
-      <c r="L2" s="69">
+      <c r="L2" s="71">
         <v>45717</v>
       </c>
-      <c r="M2" s="69">
+      <c r="M2" s="71">
         <v>45748</v>
       </c>
-      <c r="N2" s="69">
+      <c r="N2" s="71">
         <v>45778</v>
       </c>
-      <c r="O2" s="69">
+      <c r="O2" s="71">
         <v>45809</v>
       </c>
-      <c r="P2" s="69">
+      <c r="P2" s="71">
         <v>45839</v>
       </c>
-      <c r="Q2" s="69">
+      <c r="Q2" s="71">
         <v>45870</v>
       </c>
-      <c r="R2" s="69">
+      <c r="R2" s="71">
         <v>45901</v>
       </c>
-      <c r="S2" s="69">
+      <c r="S2" s="71">
         <v>45931</v>
       </c>
-      <c r="T2" s="69">
+      <c r="T2" s="71">
         <v>45962</v>
       </c>
-      <c r="U2" s="69">
+      <c r="U2" s="71">
         <v>45992</v>
       </c>
-      <c r="V2" s="69">
+      <c r="V2" s="71">
         <v>46023</v>
       </c>
-      <c r="W2" s="69">
+      <c r="W2" s="71">
         <v>46054</v>
       </c>
-      <c r="X2" s="69">
+      <c r="X2" s="71">
         <v>46082</v>
       </c>
-      <c r="Y2" s="69">
+      <c r="Y2" s="71">
         <v>46113</v>
       </c>
-      <c r="Z2" s="69">
+      <c r="Z2" s="71">
         <v>46143</v>
       </c>
-      <c r="AA2" s="69">
+      <c r="AA2" s="71">
         <v>46174</v>
       </c>
-      <c r="AB2" s="69">
+      <c r="AB2" s="71">
         <v>46204</v>
       </c>
-      <c r="AC2" s="69">
+      <c r="AC2" s="71">
         <v>46235</v>
       </c>
-      <c r="AD2" s="69">
+      <c r="AD2" s="71">
         <v>46266</v>
       </c>
-      <c r="AH2" s="68" t="s">
+      <c r="AH2" s="70" t="s">
         <v>185</v>
       </c>
     </row>
-    <row r="3" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A3" s="10"/>
       <c r="B3" s="10" t="s">
         <v>184</v>
       </c>
       <c r="C3" s="10"/>
-      <c r="D3" s="67">
-        <v>46304.710856481484</v>
-      </c>
-      <c r="E3" s="66">
-        <v>46308.678148148145</v>
+      <c r="D3" s="69">
+        <v>46309.380891203706</v>
+      </c>
+      <c r="E3" s="68">
+        <v>46310.418414351851</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>183</v>
@@ -75487,7 +75572,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="4" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>3</v>
       </c>
@@ -75578,14 +75663,14 @@
       <c r="AD4" s="7" t="e">
         <v>#N/A</v>
       </c>
-      <c r="AE4" s="65" t="s">
+      <c r="AE4" s="67" t="s">
         <v>35</v>
       </c>
       <c r="AH4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>129</v>
       </c>
@@ -75680,7 +75765,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A6" s="6">
         <v>5</v>
       </c>
@@ -75775,7 +75860,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A7" s="25">
         <v>1</v>
       </c>
@@ -75870,7 +75955,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>9</v>
       </c>
@@ -75965,7 +76050,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="6">
         <v>7</v>
       </c>
@@ -76060,7 +76145,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="25"/>
       <c r="B10" s="25"/>
       <c r="C10" s="16" t="s">
@@ -76145,7 +76230,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>131</v>
       </c>
@@ -76224,13 +76309,13 @@
       <c r="Z11" s="13">
         <v>1252</v>
       </c>
-      <c r="AA11" s="63">
+      <c r="AA11" s="65">
         <v>1256</v>
       </c>
-      <c r="AB11" s="63">
+      <c r="AB11" s="65">
         <v>1267</v>
       </c>
-      <c r="AC11" s="63">
+      <c r="AC11" s="65">
         <v>1271</v>
       </c>
       <c r="AD11" s="13" t="e">
@@ -76240,7 +76325,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="6">
         <v>133</v>
       </c>
@@ -76325,7 +76410,7 @@
       <c r="AB12" s="4">
         <v>4.2940300000000002</v>
       </c>
-      <c r="AC12" s="59">
+      <c r="AC12" s="60">
         <v>-2.0935100000000002</v>
       </c>
       <c r="AD12" s="4" t="e">
@@ -76335,7 +76420,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="25">
         <v>13</v>
       </c>
@@ -76430,7 +76515,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="25"/>
       <c r="B14" s="25"/>
       <c r="C14" s="25"/>
@@ -76452,10 +76537,10 @@
       <c r="S14" s="36"/>
       <c r="T14" s="36"/>
       <c r="U14" s="36"/>
-      <c r="V14" s="64"/>
-      <c r="W14" s="64"/>
-      <c r="X14" s="64"/>
-      <c r="Y14" s="64"/>
+      <c r="V14" s="66"/>
+      <c r="W14" s="66"/>
+      <c r="X14" s="66"/>
+      <c r="Y14" s="66"/>
       <c r="Z14" s="36"/>
       <c r="AA14" s="36"/>
       <c r="AB14" s="36"/>
@@ -76465,7 +76550,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="15" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A15" s="10"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
@@ -76502,7 +76587,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="16" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>19</v>
       </c>
@@ -76597,7 +76682,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>127</v>
       </c>
@@ -76693,7 +76778,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="18" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A18" s="6">
         <v>17</v>
       </c>
@@ -76775,10 +76860,10 @@
       <c r="AA18" s="4">
         <v>1.867</v>
       </c>
-      <c r="AB18" s="59">
+      <c r="AB18" s="60">
         <v>1.837</v>
       </c>
-      <c r="AC18" s="59">
+      <c r="AC18" s="60">
         <v>1.8080000000000001</v>
       </c>
       <c r="AD18" s="4" t="e">
@@ -76788,7 +76873,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A19" s="25">
         <v>15</v>
       </c>
@@ -76883,7 +76968,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A20" s="25"/>
       <c r="B20" s="25"/>
       <c r="C20" s="25"/>
@@ -76918,7 +77003,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="21" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A21" s="10"/>
       <c r="B21" s="10"/>
       <c r="C21" s="10" t="s">
@@ -76957,7 +77042,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="22" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>47</v>
       </c>
@@ -77042,17 +77127,17 @@
       <c r="AB22" s="13">
         <v>-10</v>
       </c>
-      <c r="AC22" s="63">
+      <c r="AC22" s="65">
         <v>133</v>
       </c>
-      <c r="AD22" s="62">
+      <c r="AD22" s="64">
         <v>29</v>
       </c>
       <c r="AH22" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>49</v>
       </c>
@@ -77140,14 +77225,14 @@
       <c r="AC23" s="12">
         <v>115</v>
       </c>
-      <c r="AD23" s="61">
+      <c r="AD23" s="63">
         <v>78</v>
       </c>
       <c r="AH23" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A24" s="6">
         <v>135</v>
       </c>
@@ -77232,17 +77317,17 @@
       <c r="AB24" s="4">
         <v>4.0999999999999996</v>
       </c>
-      <c r="AC24" s="59">
+      <c r="AC24" s="60">
         <v>4.0999999999999996</v>
       </c>
-      <c r="AD24" s="59">
+      <c r="AD24" s="60">
         <v>4.2</v>
       </c>
       <c r="AH24" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="25" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A25" s="25">
         <v>53</v>
       </c>
@@ -77337,7 +77422,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="26" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>51</v>
       </c>
@@ -77432,7 +77517,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="27" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A27" s="25"/>
       <c r="B27" s="25"/>
       <c r="C27" s="25"/>
@@ -77467,7 +77552,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
@@ -77504,7 +77589,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="29" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>101</v>
       </c>
@@ -77599,7 +77684,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>111</v>
       </c>
@@ -77700,7 +77785,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="6">
         <v>109</v>
       </c>
@@ -77795,7 +77880,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A32" s="25">
         <v>105</v>
       </c>
@@ -77890,7 +77975,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>103</v>
       </c>
@@ -77985,7 +78070,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A34" s="25"/>
       <c r="B34" s="25"/>
       <c r="C34" s="25"/>
@@ -78020,7 +78105,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="10"/>
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
@@ -78057,7 +78142,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>55</v>
       </c>
@@ -78152,7 +78237,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="37" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>59</v>
       </c>
@@ -78247,7 +78332,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="6">
         <v>139</v>
       </c>
@@ -78329,7 +78414,7 @@
       <c r="AA38" s="4">
         <v>-0.2</v>
       </c>
-      <c r="AB38" s="59">
+      <c r="AB38" s="60">
         <v>0.8</v>
       </c>
       <c r="AC38" s="4" t="e">
@@ -78342,7 +78427,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="39" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="25">
         <v>57</v>
       </c>
@@ -78437,42 +78522,42 @@
         <v>18</v>
       </c>
     </row>
-    <row r="40" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A40" s="25"/>
       <c r="B40" s="25"/>
       <c r="C40" s="25"/>
       <c r="D40" s="37"/>
       <c r="E40" s="14"/>
       <c r="F40" s="25"/>
-      <c r="G40" s="60"/>
-      <c r="H40" s="60"/>
-      <c r="I40" s="60"/>
-      <c r="J40" s="60"/>
-      <c r="K40" s="60"/>
-      <c r="L40" s="60"/>
-      <c r="M40" s="60"/>
-      <c r="N40" s="60"/>
-      <c r="O40" s="60"/>
-      <c r="P40" s="60"/>
-      <c r="Q40" s="60"/>
-      <c r="R40" s="60"/>
-      <c r="S40" s="60"/>
-      <c r="T40" s="60"/>
-      <c r="U40" s="60"/>
-      <c r="V40" s="60"/>
-      <c r="W40" s="60"/>
-      <c r="X40" s="60"/>
-      <c r="Y40" s="60"/>
-      <c r="Z40" s="60"/>
-      <c r="AA40" s="60"/>
-      <c r="AB40" s="60"/>
-      <c r="AC40" s="60"/>
-      <c r="AD40" s="60"/>
+      <c r="G40" s="62"/>
+      <c r="H40" s="62"/>
+      <c r="I40" s="62"/>
+      <c r="J40" s="62"/>
+      <c r="K40" s="62"/>
+      <c r="L40" s="62"/>
+      <c r="M40" s="62"/>
+      <c r="N40" s="62"/>
+      <c r="O40" s="62"/>
+      <c r="P40" s="62"/>
+      <c r="Q40" s="62"/>
+      <c r="R40" s="62"/>
+      <c r="S40" s="62"/>
+      <c r="T40" s="62"/>
+      <c r="U40" s="62"/>
+      <c r="V40" s="62"/>
+      <c r="W40" s="62"/>
+      <c r="X40" s="62"/>
+      <c r="Y40" s="62"/>
+      <c r="Z40" s="62"/>
+      <c r="AA40" s="62"/>
+      <c r="AB40" s="62"/>
+      <c r="AC40" s="62"/>
+      <c r="AD40" s="62"/>
       <c r="AH40" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="41" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:34" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A41" s="10"/>
       <c r="B41" s="10"/>
       <c r="C41" s="10"/>
@@ -78504,12 +78589,12 @@
       <c r="AA41" s="9"/>
       <c r="AB41" s="9"/>
       <c r="AC41" s="9"/>
-      <c r="AD41" s="9"/>
+      <c r="AD41" s="36"/>
       <c r="AH41" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="42" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A42" s="1">
         <v>25</v>
       </c>
@@ -78520,10 +78605,10 @@
         <v>103</v>
       </c>
       <c r="D42" s="24">
-        <v>46276.401261574072</v>
+        <v>46309.380891203706</v>
       </c>
       <c r="E42" s="23">
-        <v>46309.401261574065</v>
+        <v>46336.380891203706</v>
       </c>
       <c r="F42" s="1" t="s">
         <v>117</v>
@@ -78597,14 +78682,14 @@
       <c r="AC42" s="54">
         <v>3.3530199999999999</v>
       </c>
-      <c r="AD42" s="7" t="e">
-        <v>#N/A</v>
+      <c r="AD42" s="59">
+        <v>3.7172499999999999</v>
       </c>
       <c r="AH42" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="43" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A43" s="1">
         <v>23</v>
       </c>
@@ -78615,10 +78700,10 @@
         <v>103</v>
       </c>
       <c r="D43" s="24">
-        <v>46276.401180555556</v>
+        <v>46309.380891203706</v>
       </c>
       <c r="E43" s="23">
-        <v>46309.401180555549</v>
+        <v>46336.380891203706</v>
       </c>
       <c r="F43" s="1" t="s">
         <v>115</v>
@@ -78662,44 +78747,44 @@
       <c r="S43" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="T43" s="54">
+      <c r="T43" s="7">
         <v>2.5808499999999999</v>
       </c>
-      <c r="U43" s="54">
+      <c r="U43" s="7">
         <v>2.9889899999999998</v>
       </c>
-      <c r="V43" s="54">
+      <c r="V43" s="7">
         <v>2.8765000000000001</v>
       </c>
-      <c r="W43" s="54">
+      <c r="W43" s="7">
         <v>3.0527899999999999</v>
       </c>
-      <c r="X43" s="54">
+      <c r="X43" s="7">
         <v>2.6852800000000001</v>
       </c>
-      <c r="Y43" s="54">
+      <c r="Y43" s="7">
         <v>3.1423999999999999</v>
       </c>
-      <c r="Z43" s="54">
+      <c r="Z43" s="7">
         <v>3.02291</v>
       </c>
-      <c r="AA43" s="54">
+      <c r="AA43" s="7">
         <v>2.9311199999999999</v>
       </c>
-      <c r="AB43" s="54">
+      <c r="AB43" s="7">
         <v>2.8907099999999999</v>
       </c>
-      <c r="AC43" s="54">
+      <c r="AC43" s="7">
         <v>2.5751400000000002</v>
       </c>
-      <c r="AD43" s="7" t="e">
-        <v>#N/A</v>
+      <c r="AD43" s="61">
+        <v>2.39337</v>
       </c>
       <c r="AH43" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="44" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A44" s="6">
         <v>21</v>
       </c>
@@ -78710,10 +78795,10 @@
         <v>103</v>
       </c>
       <c r="D44" s="21">
-        <v>46276.401284722226</v>
+        <v>46309.380891203706</v>
       </c>
       <c r="E44" s="20">
-        <v>46309.401284722233</v>
+        <v>46336.380891203706</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>113</v>
@@ -78766,35 +78851,35 @@
       <c r="V44" s="4">
         <v>-0.29616999999999999</v>
       </c>
-      <c r="W44" s="59">
+      <c r="W44" s="60">
         <v>0.39950999999999998</v>
       </c>
-      <c r="X44" s="59">
+      <c r="X44" s="60">
         <v>12.589549999999999</v>
       </c>
-      <c r="Y44" s="59">
+      <c r="Y44" s="60">
         <v>17.536049999999999</v>
       </c>
-      <c r="Z44" s="59">
+      <c r="Z44" s="60">
         <v>22.97287</v>
       </c>
-      <c r="AA44" s="59">
+      <c r="AA44" s="60">
         <v>15.451370000000001</v>
       </c>
-      <c r="AB44" s="59">
+      <c r="AB44" s="60">
         <v>14.44533</v>
       </c>
-      <c r="AC44" s="59">
+      <c r="AC44" s="60">
         <v>16.04935</v>
       </c>
-      <c r="AD44" s="4" t="e">
-        <v>#N/A</v>
+      <c r="AD44" s="54">
+        <v>20.354109999999999</v>
       </c>
       <c r="AH44" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="45" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="1">
         <v>27</v>
       </c>
@@ -78805,10 +78890,10 @@
         <v>103</v>
       </c>
       <c r="D45" s="24">
-        <v>46276.401307870372</v>
+        <v>46309.380891203706</v>
       </c>
       <c r="E45" s="23">
-        <v>46309.401307870372</v>
+        <v>46336.380891203706</v>
       </c>
       <c r="F45" s="1" t="s">
         <v>111</v>
@@ -78876,20 +78961,20 @@
       <c r="AA45" s="7">
         <v>2.5657899999999998</v>
       </c>
-      <c r="AB45" s="28">
+      <c r="AB45" s="7">
         <v>2.46652</v>
       </c>
-      <c r="AC45" s="28">
+      <c r="AC45" s="7">
         <v>2.4461599999999999</v>
       </c>
-      <c r="AD45" s="7" t="e">
-        <v>#N/A</v>
+      <c r="AD45" s="59">
+        <v>2.5658400000000001</v>
       </c>
       <c r="AH45" t="s">
         <v>110</v>
       </c>
     </row>
-    <row r="46" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:34" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A46" s="25"/>
       <c r="B46" s="25"/>
       <c r="C46" s="25"/>
@@ -78924,7 +79009,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="47" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="10"/>
       <c r="B47" s="10"/>
       <c r="C47" s="10"/>
@@ -78961,7 +79046,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="48" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>123</v>
       </c>
@@ -79056,7 +79141,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="49" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>119</v>
       </c>
@@ -79151,7 +79236,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="50" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="6">
         <v>121</v>
       </c>
@@ -79246,7 +79331,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="51" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="47">
         <v>115</v>
       </c>
@@ -79341,7 +79426,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="52" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A52" s="25">
         <v>113</v>
       </c>
@@ -79436,7 +79521,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="53" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A53" s="6">
         <v>125</v>
       </c>
@@ -79531,7 +79616,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="54" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A54" s="57">
         <v>117</v>
       </c>
@@ -79626,7 +79711,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="55" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A55" s="25"/>
       <c r="B55" s="25"/>
       <c r="C55" s="25"/>
@@ -79661,7 +79746,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="56" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A56" s="25"/>
       <c r="B56" s="25"/>
       <c r="C56" s="25"/>
@@ -79746,7 +79831,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="57" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A57" s="10"/>
       <c r="B57" s="10"/>
       <c r="C57" s="10"/>
@@ -79831,7 +79916,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="58" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A58" s="1">
         <v>141</v>
       </c>
@@ -79926,7 +80011,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="59" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A59" s="1">
         <v>41</v>
       </c>
@@ -80021,7 +80106,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="60" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A60" s="6">
         <v>45</v>
       </c>
@@ -80116,7 +80201,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="61" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A61" s="25">
         <v>43</v>
       </c>
@@ -80211,7 +80296,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="62" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A62" s="1">
         <v>39</v>
       </c>
@@ -80306,7 +80391,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="63" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A63" s="6">
         <v>35</v>
       </c>
@@ -80401,7 +80486,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="64" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" s="25">
         <v>37</v>
       </c>
@@ -80496,7 +80581,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="65" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>137</v>
       </c>
@@ -80591,7 +80676,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="66" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A66" s="6">
         <v>29</v>
       </c>
@@ -80686,7 +80771,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="67" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A67" s="25">
         <v>31</v>
       </c>
@@ -80781,7 +80866,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="68" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A68" s="1">
         <v>33</v>
       </c>
@@ -80876,7 +80961,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A69" s="25"/>
       <c r="B69" s="25"/>
       <c r="C69" s="25"/>
@@ -80911,7 +80996,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="70" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A70" s="10"/>
       <c r="B70" s="10"/>
       <c r="C70" s="10"/>
@@ -80948,7 +81033,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="71" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A71" s="1">
         <v>61</v>
       </c>
@@ -81043,7 +81128,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="72" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A72" s="1">
         <v>63</v>
       </c>
@@ -81138,7 +81223,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="73" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A73" s="6">
         <v>83</v>
       </c>
@@ -81233,7 +81318,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="74" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A74" s="1">
         <v>81</v>
       </c>
@@ -81244,10 +81329,10 @@
         <v>37</v>
       </c>
       <c r="D74" s="24">
-        <v>46304.678148148145</v>
+        <v>46308.678611111114</v>
       </c>
       <c r="E74" s="48">
-        <v>46308.678148148145</v>
+        <v>46311.678611111114</v>
       </c>
       <c r="F74" s="47" t="s">
         <v>57</v>
@@ -81328,7 +81413,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="75" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A75" s="25">
         <v>79</v>
       </c>
@@ -81342,7 +81427,7 @@
         <v>46300.678460648145</v>
       </c>
       <c r="E75" s="52">
-        <v>46308.678460648138</v>
+        <v>46311.678460648138</v>
       </c>
       <c r="F75" s="42" t="s">
         <v>55</v>
@@ -81423,7 +81508,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="76" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A76" s="6">
         <v>149</v>
       </c>
@@ -81434,10 +81519,10 @@
         <v>37</v>
       </c>
       <c r="D76" s="21">
-        <v>46304.678194444445</v>
+        <v>46308.678576388891</v>
       </c>
       <c r="E76" s="53">
-        <v>46308.678194444452</v>
+        <v>46311.678576388891</v>
       </c>
       <c r="F76" s="45" t="s">
         <v>53</v>
@@ -81518,7 +81603,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="77" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A77" s="1">
         <v>73</v>
       </c>
@@ -81529,10 +81614,10 @@
         <v>37</v>
       </c>
       <c r="D77" s="24">
-        <v>46304.678171296298</v>
+        <v>46308.678483796299</v>
       </c>
       <c r="E77" s="52">
-        <v>46308.678171296298</v>
+        <v>46311.678483796306</v>
       </c>
       <c r="F77" s="47" t="s">
         <v>51</v>
@@ -81613,7 +81698,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="78" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A78" s="42">
         <v>145</v>
       </c>
@@ -81627,7 +81712,7 @@
         <v>46296.710868055554</v>
       </c>
       <c r="E78" s="52">
-        <v>46308.710868055554</v>
+        <v>46311.710868055554</v>
       </c>
       <c r="F78" s="42" t="s">
         <v>49</v>
@@ -81709,7 +81794,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A79" s="6">
         <v>75</v>
       </c>
@@ -81720,10 +81805,10 @@
         <v>37</v>
       </c>
       <c r="D79" s="21">
-        <v>46304.678171296298</v>
+        <v>46308.678437499999</v>
       </c>
       <c r="E79" s="50">
-        <v>46308.678171296298</v>
+        <v>46311.678437499999</v>
       </c>
       <c r="F79" s="45" t="s">
         <v>47</v>
@@ -81804,7 +81889,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="80" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A80" s="1">
         <v>77</v>
       </c>
@@ -81815,10 +81900,10 @@
         <v>37</v>
       </c>
       <c r="D80" s="24">
-        <v>46304.678217592591</v>
+        <v>46308.678587962961</v>
       </c>
       <c r="E80" s="48">
-        <v>46308.678217592591</v>
+        <v>46311.678587962961</v>
       </c>
       <c r="F80" s="47" t="s">
         <v>45</v>
@@ -81899,7 +81984,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="81" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A81" s="25">
         <v>147</v>
       </c>
@@ -81910,10 +81995,10 @@
         <v>42</v>
       </c>
       <c r="D81" s="15">
-        <v>46304.710856481484</v>
+        <v>46308.710844907408</v>
       </c>
       <c r="E81" s="14">
-        <v>46308.710856481484</v>
+        <v>46311.710844907415</v>
       </c>
       <c r="F81" s="42" t="s">
         <v>41</v>
@@ -81994,7 +82079,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="82" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A82" s="6">
         <v>67</v>
       </c>
@@ -82005,10 +82090,10 @@
         <v>37</v>
       </c>
       <c r="D82" s="21">
-        <v>46300.678252314814</v>
+        <v>46308.678506944445</v>
       </c>
       <c r="E82" s="20">
-        <v>46308.678252314814</v>
+        <v>46314.678506944445</v>
       </c>
       <c r="F82" s="45" t="s">
         <v>39</v>
@@ -82089,7 +82174,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="83" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A83" s="25">
         <v>65</v>
       </c>
@@ -82100,10 +82185,10 @@
         <v>37</v>
       </c>
       <c r="D83" s="15">
-        <v>46300.678391203706</v>
+        <v>46308.678599537037</v>
       </c>
       <c r="E83" s="23">
-        <v>46308.678391203706</v>
+        <v>46314.67859953703</v>
       </c>
       <c r="F83" s="42" t="s">
         <v>36</v>
@@ -82184,7 +82269,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="84" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A84" s="25"/>
       <c r="B84" s="25"/>
       <c r="C84" s="25"/>
@@ -82268,7 +82353,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="85" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A85" s="25"/>
       <c r="B85" s="25"/>
       <c r="C85" s="25"/>
@@ -82352,7 +82437,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="86" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A86" s="10"/>
       <c r="B86" s="10"/>
       <c r="C86" s="10"/>
@@ -82438,7 +82523,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="87" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A87" s="1">
         <v>97</v>
       </c>
@@ -82533,7 +82618,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="88" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A88" s="1">
         <v>99</v>
       </c>
@@ -82628,7 +82713,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="89" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A89" s="6">
         <v>107</v>
       </c>
@@ -82723,7 +82808,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="90" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A90" s="25">
         <v>95</v>
       </c>
@@ -82818,7 +82903,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="91" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A91" s="1">
         <v>93</v>
       </c>
@@ -82913,7 +82998,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="92" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A92" s="6">
         <v>91</v>
       </c>
@@ -83008,7 +83093,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="93" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A93" s="25">
         <v>89</v>
       </c>
@@ -83103,7 +83188,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="94" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A94" s="1">
         <v>85</v>
       </c>
@@ -83198,7 +83283,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="95" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A95" s="19">
         <v>87</v>
       </c>
@@ -83293,7 +83378,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="96" spans="1:34" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A96" s="1">
         <v>11</v>
       </c>
@@ -83391,10 +83476,12 @@
     <row r="98" spans="17:17" x14ac:dyDescent="0.25">
       <c r="Q98" s="11"/>
     </row>
-    <row r="118" spans="1:30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:30" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A118" s="10"/>
       <c r="B118" s="10"/>
       <c r="C118" s="10"/>
+      <c r="D118" s="3"/>
+      <c r="E118" s="3"/>
       <c r="F118" s="10" t="s">
         <v>5</v>
       </c>
@@ -83423,7 +83510,12 @@
       <c r="AC118" s="9"/>
       <c r="AD118" s="9"/>
     </row>
-    <row r="119" spans="1:30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:30" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A119" s="1"/>
+      <c r="B119" s="1"/>
+      <c r="C119" s="1"/>
+      <c r="D119" s="3"/>
+      <c r="E119" s="3"/>
       <c r="F119" s="1" t="s">
         <v>2</v>
       </c>
@@ -83500,7 +83592,12 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="120" spans="1:30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:30" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A120" s="1"/>
+      <c r="B120" s="1"/>
+      <c r="C120" s="1"/>
+      <c r="D120" s="3"/>
+      <c r="E120" s="3"/>
       <c r="F120" s="1" t="s">
         <v>1</v>
       </c>
@@ -83577,10 +83674,12 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="121" spans="1:30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:30" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="A121" s="6"/>
       <c r="B121" s="6"/>
       <c r="C121" s="6"/>
+      <c r="D121" s="3"/>
+      <c r="E121" s="3"/>
       <c r="F121" s="6" t="s">
         <v>0</v>
       </c>
@@ -83657,12 +83756,22 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="122" spans="1:30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:30" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A122" s="1"/>
+      <c r="B122" s="1"/>
+      <c r="C122" s="1"/>
+      <c r="D122" s="3"/>
+      <c r="E122" s="3"/>
       <c r="F122" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="123" spans="1:30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:30" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A123" s="1"/>
+      <c r="B123" s="1"/>
+      <c r="C123" s="1"/>
+      <c r="D123" s="3"/>
+      <c r="E123" s="3"/>
       <c r="F123" s="1" t="s">
         <v>2</v>
       </c>
@@ -83739,7 +83848,12 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="124" spans="1:30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:30" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A124" s="1"/>
+      <c r="B124" s="1"/>
+      <c r="C124" s="1"/>
+      <c r="D124" s="3"/>
+      <c r="E124" s="3"/>
       <c r="F124" s="1" t="s">
         <v>1</v>
       </c>
@@ -83816,7 +83930,12 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="125" spans="1:30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:30" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A125" s="1"/>
+      <c r="B125" s="1"/>
+      <c r="C125" s="1"/>
+      <c r="D125" s="3"/>
+      <c r="E125" s="3"/>
       <c r="F125" s="1" t="s">
         <v>0</v>
       </c>
@@ -83893,12 +84012,22 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="126" spans="1:30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:30" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A126" s="1"/>
+      <c r="B126" s="1"/>
+      <c r="C126" s="1"/>
+      <c r="D126" s="3"/>
+      <c r="E126" s="3"/>
       <c r="F126" s="1" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="127" spans="1:30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:30" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A127" s="1"/>
+      <c r="B127" s="1"/>
+      <c r="C127" s="1"/>
+      <c r="D127" s="3"/>
+      <c r="E127" s="3"/>
       <c r="F127" s="1" t="s">
         <v>2</v>
       </c>
@@ -83975,7 +84104,12 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="128" spans="1:30" hidden="1" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:30" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="A128" s="1"/>
+      <c r="B128" s="1"/>
+      <c r="C128" s="1"/>
+      <c r="D128" s="3"/>
+      <c r="E128" s="3"/>
       <c r="F128" s="1" t="s">
         <v>1</v>
       </c>
@@ -84052,7 +84186,7 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="129" spans="6:34" hidden="1" x14ac:dyDescent="0.25">
+    <row r="129" spans="6:34" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="F129" s="1" t="s">
         <v>0</v>
       </c>
@@ -84129,510 +84263,513 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="130" spans="6:34" hidden="1" x14ac:dyDescent="0.25">
+    <row r="130" spans="6:34" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="F130" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="131" spans="6:34" hidden="1" x14ac:dyDescent="0.25">
+    <row r="131" spans="6:34" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="F131" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G131" s="3">
+      <c r="G131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="H131" s="3">
+      <c r="H131" s="2">
         <v>2.00332</v>
       </c>
-      <c r="I131" s="3">
+      <c r="I131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="J131" s="3">
+      <c r="J131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="K131" s="3">
+      <c r="K131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="L131" s="3">
+      <c r="L131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="M131" s="3">
+      <c r="M131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="N131" s="3">
+      <c r="N131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="O131" s="3">
+      <c r="O131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="P131" s="3">
+      <c r="P131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="Q131" s="3">
+      <c r="Q131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="R131" s="3">
+      <c r="R131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="S131" s="3">
+      <c r="S131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="T131" s="3">
+      <c r="T131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="U131" s="3">
+      <c r="U131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="V131" s="3">
+      <c r="V131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="W131" s="3">
+      <c r="W131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="X131" s="3">
+      <c r="X131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="Y131" s="3">
+      <c r="Y131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="Z131" s="3">
+      <c r="Z131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="AA131" s="3">
+      <c r="AA131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="AB131" s="3">
+      <c r="AB131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="AC131" s="3">
+      <c r="AC131" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="AD131" s="3" t="e">
+      <c r="AD131" s="2" t="e">
         <v>#N/A</v>
       </c>
       <c r="AH131">
         <v>83</v>
       </c>
     </row>
-    <row r="132" spans="6:34" hidden="1" x14ac:dyDescent="0.25">
+    <row r="132" spans="6:34" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="F132" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G132" s="3">
+      <c r="G132" s="2">
         <v>-1.32026</v>
       </c>
-      <c r="H132" s="3">
+      <c r="H132" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="I132" s="3">
+      <c r="I132" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="J132" s="3">
+      <c r="J132" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="K132" s="3">
+      <c r="K132" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="L132" s="3">
+      <c r="L132" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="M132" s="3">
+      <c r="M132" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="N132" s="3">
+      <c r="N132" s="2">
         <v>1.8177700000000001</v>
       </c>
-      <c r="O132" s="3">
+      <c r="O132" s="2">
         <v>1.82314</v>
       </c>
-      <c r="P132" s="3">
+      <c r="P132" s="2">
         <v>2.1143399999999999</v>
       </c>
-      <c r="Q132" s="3">
+      <c r="Q132" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="R132" s="3">
+      <c r="R132" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="S132" s="3">
+      <c r="S132" s="2">
         <v>3.1039699999999999</v>
       </c>
-      <c r="T132" s="3">
+      <c r="T132" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="U132" s="3">
+      <c r="U132" s="2">
         <v>3.4494099999999999</v>
       </c>
-      <c r="V132" s="3">
+      <c r="V132" s="2">
         <v>2.7845900000000001</v>
       </c>
-      <c r="W132" s="3">
+      <c r="W132" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="X132" s="3">
+      <c r="X132" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="Y132" s="3">
+      <c r="Y132" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="Z132" s="3">
+      <c r="Z132" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="AA132" s="3">
+      <c r="AA132" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="AB132" s="3">
+      <c r="AB132" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="AC132" s="3">
+      <c r="AC132" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="AD132" s="3" t="e">
+      <c r="AD132" s="2" t="e">
         <v>#N/A</v>
       </c>
     </row>
-    <row r="133" spans="6:34" hidden="1" x14ac:dyDescent="0.25">
+    <row r="133" spans="6:34" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="F133" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G133" s="3">
+      <c r="G133" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="H133" s="3">
+      <c r="H133" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="I133" s="3">
+      <c r="I133" s="2">
         <v>4.7821400000000001</v>
       </c>
-      <c r="J133" s="3">
+      <c r="J133" s="2">
         <v>8.6400299999999994</v>
       </c>
-      <c r="K133" s="3">
+      <c r="K133" s="2">
         <v>9.3640600000000003</v>
       </c>
-      <c r="L133" s="3">
+      <c r="L133" s="2">
         <v>6.5289299999999999</v>
       </c>
-      <c r="M133" s="3">
+      <c r="M133" s="2">
         <v>0.27726000000000001</v>
       </c>
-      <c r="N133" s="3">
+      <c r="N133" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="O133" s="3">
+      <c r="O133" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="P133" s="3">
+      <c r="P133" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="Q133" s="3">
+      <c r="Q133" s="2">
         <v>1.4526600000000001</v>
       </c>
-      <c r="R133" s="3">
+      <c r="R133" s="2">
         <v>3.4353099999999999</v>
       </c>
-      <c r="S133" s="3">
+      <c r="S133" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="T133" s="3">
+      <c r="T133" s="2">
         <v>1.89177</v>
       </c>
-      <c r="U133" s="3">
+      <c r="U133" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="V133" s="3">
+      <c r="V133" s="2">
         <v>-10000000000</v>
       </c>
-      <c r="W133" s="3">
+      <c r="W133" s="2">
         <v>5.3440700000000003</v>
       </c>
-      <c r="X133" s="3">
+      <c r="X133" s="2">
         <v>9.3355499999999996</v>
       </c>
-      <c r="Y133" s="3">
+      <c r="Y133" s="2">
         <v>15.40253</v>
       </c>
-      <c r="Z133" s="3">
+      <c r="Z133" s="2">
         <v>20.728020000000001</v>
       </c>
-      <c r="AA133" s="3">
+      <c r="AA133" s="2">
         <v>10.44711</v>
       </c>
-      <c r="AB133" s="3">
+      <c r="AB133" s="2">
         <v>9.8271599999999992</v>
       </c>
-      <c r="AC133" s="3">
+      <c r="AC133" s="2">
         <v>13.063190000000001</v>
       </c>
-      <c r="AD133" s="3" t="e">
+      <c r="AD133" s="2" t="e">
         <v>#N/A</v>
       </c>
     </row>
-    <row r="134" spans="6:34" hidden="1" x14ac:dyDescent="0.25">
+    <row r="134" spans="6:34" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="F134" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G134" s="3"/>
-      <c r="H134" s="3"/>
-      <c r="I134" s="3"/>
-      <c r="J134" s="3"/>
-      <c r="K134" s="3"/>
-      <c r="L134" s="3"/>
-      <c r="M134" s="3"/>
-      <c r="N134" s="3"/>
-      <c r="O134" s="3"/>
-      <c r="P134" s="3"/>
-      <c r="Q134" s="3"/>
-      <c r="R134" s="3"/>
-      <c r="S134" s="3"/>
-      <c r="T134" s="3"/>
-      <c r="U134" s="3"/>
-      <c r="V134" s="3"/>
-      <c r="W134" s="3"/>
-      <c r="X134" s="3"/>
-      <c r="Y134" s="3"/>
-      <c r="Z134" s="3"/>
-      <c r="AA134" s="3"/>
-      <c r="AB134" s="3"/>
-      <c r="AC134" s="3"/>
-      <c r="AD134" s="3"/>
+      <c r="G134" s="2"/>
+      <c r="H134" s="2"/>
+      <c r="I134" s="2"/>
+      <c r="J134" s="2"/>
+      <c r="K134" s="2"/>
+      <c r="L134" s="2"/>
+      <c r="M134" s="2"/>
+      <c r="N134" s="2"/>
+      <c r="O134" s="2"/>
+      <c r="P134" s="2"/>
+      <c r="Q134" s="2"/>
+      <c r="R134" s="2"/>
+      <c r="S134" s="2"/>
+      <c r="T134" s="2"/>
+      <c r="U134" s="2"/>
+      <c r="V134" s="2"/>
+      <c r="W134" s="2"/>
+      <c r="X134" s="2"/>
+      <c r="Y134" s="2"/>
+      <c r="Z134" s="2"/>
+      <c r="AA134" s="2"/>
+      <c r="AB134" s="2"/>
+      <c r="AC134" s="2"/>
+      <c r="AD134" s="2"/>
     </row>
-    <row r="135" spans="6:34" hidden="1" x14ac:dyDescent="0.25">
+    <row r="135" spans="6:34" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="F135" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="G135" s="3">
+      <c r="G135" s="2">
         <v>10000000000</v>
       </c>
-      <c r="H135" s="3">
+      <c r="H135" s="2">
         <v>10000000000</v>
       </c>
-      <c r="I135" s="3">
+      <c r="I135" s="2">
         <v>10000000000</v>
       </c>
-      <c r="J135" s="3">
+      <c r="J135" s="2">
         <v>10000000000</v>
       </c>
-      <c r="K135" s="3">
+      <c r="K135" s="2">
         <v>10000000000</v>
       </c>
-      <c r="L135" s="3">
+      <c r="L135" s="2">
         <v>10000000000</v>
       </c>
-      <c r="M135" s="3">
+      <c r="M135" s="2">
         <v>0.29111999999999999</v>
       </c>
-      <c r="N135" s="3">
+      <c r="N135" s="2">
         <v>10000000000</v>
       </c>
-      <c r="O135" s="3">
+      <c r="O135" s="2">
         <v>1.8916599999999999</v>
       </c>
-      <c r="P135" s="3">
+      <c r="P135" s="2">
         <v>1.9171</v>
       </c>
-      <c r="Q135" s="3">
+      <c r="Q135" s="2">
         <v>1.9361200000000001</v>
       </c>
-      <c r="R135" s="3">
+      <c r="R135" s="2">
         <v>3.10771</v>
       </c>
-      <c r="S135" s="3">
+      <c r="S135" s="2">
         <v>10000000000</v>
       </c>
-      <c r="T135" s="3">
+      <c r="T135" s="2">
         <v>2.7689699999999999</v>
       </c>
-      <c r="U135" s="3">
+      <c r="U135" s="2">
         <v>2.15889</v>
       </c>
-      <c r="V135" s="3">
+      <c r="V135" s="2">
         <v>1.11154</v>
       </c>
-      <c r="W135" s="3">
+      <c r="W135" s="2">
         <v>1.6553800000000001</v>
       </c>
-      <c r="X135" s="3">
+      <c r="X135" s="2">
         <v>10000000000</v>
       </c>
-      <c r="Y135" s="3">
+      <c r="Y135" s="2">
         <v>10000000000</v>
       </c>
-      <c r="Z135" s="3">
+      <c r="Z135" s="2">
         <v>10000000000</v>
       </c>
-      <c r="AA135" s="3">
+      <c r="AA135" s="2">
         <v>6.55274</v>
       </c>
-      <c r="AB135" s="3">
+      <c r="AB135" s="2">
         <v>5.7949400000000004</v>
       </c>
-      <c r="AC135" s="3">
+      <c r="AC135" s="2">
         <v>6.5589300000000001</v>
       </c>
-      <c r="AD135" s="3" t="e">
+      <c r="AD135" s="2" t="e">
         <v>#N/A</v>
       </c>
     </row>
-    <row r="136" spans="6:34" hidden="1" x14ac:dyDescent="0.25">
+    <row r="136" spans="6:34" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="F136" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G136" s="3">
+      <c r="G136" s="2">
         <v>10000000000</v>
       </c>
-      <c r="H136" s="3">
+      <c r="H136" s="2">
         <v>10000000000</v>
       </c>
-      <c r="I136" s="3">
+      <c r="I136" s="2">
         <v>9.7409999999999997E-2</v>
       </c>
-      <c r="J136" s="3">
+      <c r="J136" s="2">
         <v>0.96982999999999997</v>
       </c>
-      <c r="K136" s="3">
+      <c r="K136" s="2">
         <v>0.28866000000000003</v>
       </c>
-      <c r="L136" s="3">
+      <c r="L136" s="2">
         <v>0.69299999999999995</v>
       </c>
-      <c r="M136" s="3">
+      <c r="M136" s="2">
         <v>10000000000</v>
       </c>
-      <c r="N136" s="3">
+      <c r="N136" s="2">
         <v>10000000000</v>
       </c>
-      <c r="O136" s="3">
+      <c r="O136" s="2">
         <v>10000000000</v>
       </c>
-      <c r="P136" s="3">
+      <c r="P136" s="2">
         <v>10000000000</v>
       </c>
-      <c r="Q136" s="3">
+      <c r="Q136" s="2">
         <v>10000000000</v>
       </c>
-      <c r="R136" s="3">
+      <c r="R136" s="2">
         <v>10000000000</v>
       </c>
-      <c r="S136" s="3">
+      <c r="S136" s="2">
         <v>10000000000</v>
       </c>
-      <c r="T136" s="3">
+      <c r="T136" s="2">
         <v>10000000000</v>
       </c>
-      <c r="U136" s="3">
+      <c r="U136" s="2">
         <v>10000000000</v>
       </c>
-      <c r="V136" s="3">
+      <c r="V136" s="2">
         <v>10000000000</v>
       </c>
-      <c r="W136" s="3">
+      <c r="W136" s="2">
         <v>10000000000</v>
       </c>
-      <c r="X136" s="3">
+      <c r="X136" s="2">
         <v>6.9090499999999997</v>
       </c>
-      <c r="Y136" s="3">
+      <c r="Y136" s="2">
         <v>9.4268000000000001</v>
       </c>
-      <c r="Z136" s="3">
+      <c r="Z136" s="2">
         <v>12.209860000000001</v>
       </c>
-      <c r="AA136" s="3">
+      <c r="AA136" s="2">
         <v>10000000000</v>
       </c>
-      <c r="AB136" s="3">
+      <c r="AB136" s="2">
         <v>10000000000</v>
       </c>
-      <c r="AC136" s="3">
+      <c r="AC136" s="2">
         <v>10000000000</v>
       </c>
-      <c r="AD136" s="3" t="e">
+      <c r="AD136" s="2" t="e">
         <v>#N/A</v>
       </c>
       <c r="AH136">
         <v>87</v>
       </c>
     </row>
-    <row r="137" spans="6:34" hidden="1" x14ac:dyDescent="0.25">
+    <row r="137" spans="6:34" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
       <c r="F137" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="G137" s="3">
+      <c r="G137" s="2">
         <v>-4.3331</v>
       </c>
-      <c r="H137" s="3">
+      <c r="H137" s="2">
         <v>-2.0904600000000002</v>
       </c>
-      <c r="I137" s="3">
+      <c r="I137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="J137" s="3">
+      <c r="J137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="K137" s="3">
+      <c r="K137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="L137" s="3">
+      <c r="L137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="M137" s="3">
+      <c r="M137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="N137" s="3">
+      <c r="N137" s="2">
         <v>-1.1279399999999999</v>
       </c>
-      <c r="O137" s="3">
+      <c r="O137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="P137" s="3">
+      <c r="P137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="Q137" s="3">
+      <c r="Q137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="R137" s="3">
+      <c r="R137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="S137" s="3">
+      <c r="S137" s="2">
         <v>-0.64237999999999995</v>
       </c>
-      <c r="T137" s="3">
+      <c r="T137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="U137" s="3">
+      <c r="U137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="V137" s="3">
+      <c r="V137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="W137" s="3">
+      <c r="W137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="X137" s="3">
+      <c r="X137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="Y137" s="3">
+      <c r="Y137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="Z137" s="3">
+      <c r="Z137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="AA137" s="3">
+      <c r="AA137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="AB137" s="3">
+      <c r="AB137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="AC137" s="3">
+      <c r="AC137" s="2">
         <v>10000000000</v>
       </c>
-      <c r="AD137" s="3" t="e">
+      <c r="AD137" s="2" t="e">
         <v>#N/A</v>
       </c>
     </row>
-    <row r="138" spans="6:34" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="138" spans="6:34" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F138" s="1"/>
+    </row>
     <row r="139" spans="6:34" ht="16.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F139" s="1"/>
       <c r="G139" t="b">
         <v>0</v>
       </c>
@@ -84706,7 +84843,8 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="140" spans="6:34" hidden="1" x14ac:dyDescent="0.25">
+    <row r="140" spans="6:34" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F140" s="1"/>
       <c r="G140" t="b">
         <v>1</v>
       </c>
@@ -84780,10 +84918,33 @@
         <v>#N/A</v>
       </c>
     </row>
-    <row r="141" spans="6:34" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="142" spans="6:34" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="143" spans="6:34" hidden="1" x14ac:dyDescent="0.25"/>
-    <row r="144" spans="6:34" hidden="1" x14ac:dyDescent="0.25"/>
+    <row r="141" spans="6:34" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F141" s="1"/>
+    </row>
+    <row r="142" spans="6:34" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F142" s="1"/>
+    </row>
+    <row r="143" spans="6:34" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F143" s="1"/>
+    </row>
+    <row r="144" spans="6:34" ht="15.75" hidden="1" x14ac:dyDescent="0.25">
+      <c r="F144" s="1"/>
+    </row>
+    <row r="145" spans="35:47" s="1" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="AI145"/>
+      <c r="AJ145"/>
+      <c r="AK145"/>
+      <c r="AL145"/>
+      <c r="AM145"/>
+      <c r="AN145"/>
+      <c r="AO145"/>
+      <c r="AP145"/>
+      <c r="AQ145"/>
+      <c r="AR145"/>
+      <c r="AS145"/>
+      <c r="AT145"/>
+      <c r="AU145"/>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="E3:E96">
     <cfRule type="cellIs" priority="238" stopIfTrue="1" operator="equal">
@@ -84876,156 +85037,210 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G4:AD4">
-    <cfRule type="expression" dxfId="221" priority="220">
-      <formula>ISERROR(G4)</formula>
+    <cfRule type="cellIs" dxfId="221" priority="222" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>0</formula>
     </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4:AD4">
     <cfRule type="cellIs" dxfId="220" priority="221" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="219" priority="222" stopIfTrue="1" operator="greaterThanOrEqual">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G4:AD4">
+    <cfRule type="expression" dxfId="219" priority="220">
+      <formula>ISERROR(G4)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G5:AD5">
+    <cfRule type="cellIs" dxfId="218" priority="219" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:AD5">
-    <cfRule type="expression" dxfId="218" priority="217">
-      <formula>ISERROR(G5)</formula>
-    </cfRule>
     <cfRule type="cellIs" dxfId="217" priority="218" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="216" priority="219" stopIfTrue="1" operator="greaterThanOrEqual">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G5:AD5">
+    <cfRule type="expression" dxfId="216" priority="217">
+      <formula>ISERROR(G5)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G6:AD6">
+    <cfRule type="cellIs" dxfId="215" priority="216" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G6:AD6">
-    <cfRule type="expression" dxfId="215" priority="214">
-      <formula>ISERROR(G6)</formula>
-    </cfRule>
     <cfRule type="cellIs" dxfId="214" priority="215" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="213" priority="216" stopIfTrue="1" operator="greaterThanOrEqual">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G6:AD6">
+    <cfRule type="expression" dxfId="213" priority="214">
+      <formula>ISERROR(G6)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G7:AD7">
+    <cfRule type="cellIs" dxfId="212" priority="213" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:AD7">
-    <cfRule type="expression" dxfId="212" priority="211">
-      <formula>ISERROR(G7)</formula>
-    </cfRule>
     <cfRule type="cellIs" dxfId="211" priority="212" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="210" priority="213" stopIfTrue="1" operator="greaterThanOrEqual">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G7:AD7">
+    <cfRule type="expression" dxfId="210" priority="211">
+      <formula>ISERROR(G7)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G8:AD8">
+    <cfRule type="cellIs" dxfId="209" priority="210" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G8:AD8">
-    <cfRule type="expression" dxfId="209" priority="208">
-      <formula>ISERROR(G8)</formula>
-    </cfRule>
     <cfRule type="cellIs" dxfId="208" priority="209" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="207" priority="210" stopIfTrue="1" operator="greaterThanOrEqual">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G8:AD8">
+    <cfRule type="expression" dxfId="207" priority="208">
+      <formula>ISERROR(G8)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9:AD9">
+    <cfRule type="cellIs" dxfId="206" priority="207" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>F9</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9:AD9">
+    <cfRule type="cellIs" dxfId="205" priority="206" stopIfTrue="1" operator="lessThan">
+      <formula>F9</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G9:AD9">
+    <cfRule type="expression" dxfId="204" priority="205">
+      <formula>ISERROR(G9)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G10:AD10">
+    <cfRule type="cellIs" dxfId="203" priority="204" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G9:AD9">
-    <cfRule type="expression" dxfId="206" priority="205">
-      <formula>ISERROR(G9)</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="205" priority="206" stopIfTrue="1" operator="lessThan">
-      <formula>F9</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="204" priority="207" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>F9</formula>
+  <conditionalFormatting sqref="G10:AD10">
+    <cfRule type="cellIs" dxfId="202" priority="203" stopIfTrue="1" operator="lessThan">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G10:AD10">
-    <cfRule type="expression" dxfId="203" priority="202">
+    <cfRule type="expression" dxfId="201" priority="202">
       <formula>ISERROR(G10)</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="202" priority="203" stopIfTrue="1" operator="lessThan">
-      <formula>0</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G11:AD11">
+    <cfRule type="cellIs" dxfId="200" priority="201" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>F11</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="201" priority="204" stopIfTrue="1" operator="greaterThanOrEqual">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G11:AD11">
+    <cfRule type="cellIs" dxfId="199" priority="200" stopIfTrue="1" operator="lessThan">
+      <formula>F11</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G11:AD11">
+    <cfRule type="expression" dxfId="198" priority="199">
+      <formula>ISERROR(G11)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G12:AD12">
+    <cfRule type="cellIs" dxfId="197" priority="198" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G11:AD11">
-    <cfRule type="expression" dxfId="200" priority="199">
-      <formula>ISERROR(G11)</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="199" priority="200" stopIfTrue="1" operator="lessThan">
-      <formula>F11</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="198" priority="201" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>F11</formula>
+  <conditionalFormatting sqref="G12:AD12">
+    <cfRule type="cellIs" dxfId="196" priority="197" stopIfTrue="1" operator="lessThan">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G12:AD12">
-    <cfRule type="expression" dxfId="197" priority="196">
+    <cfRule type="expression" dxfId="195" priority="196">
       <formula>ISERROR(G12)</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="196" priority="197" stopIfTrue="1" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="195" priority="198" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G13:AD13">
-    <cfRule type="expression" dxfId="194" priority="193">
-      <formula>ISERROR(G13)</formula>
+    <cfRule type="cellIs" dxfId="194" priority="195" stopIfTrue="1" operator="lessThanOrEqual">
+      <formula>F13</formula>
     </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G13:AD13">
     <cfRule type="cellIs" dxfId="193" priority="194" stopIfTrue="1" operator="greaterThan">
       <formula>F13</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="192" priority="195" stopIfTrue="1" operator="lessThanOrEqual">
-      <formula>F13</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G13:AD13">
+    <cfRule type="expression" dxfId="192" priority="193">
+      <formula>ISERROR(G13)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G16:AD16">
-    <cfRule type="expression" dxfId="191" priority="190">
-      <formula>ISERROR(G16)</formula>
+    <cfRule type="cellIs" dxfId="191" priority="192" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>F16</formula>
     </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G16:AD16">
     <cfRule type="cellIs" dxfId="190" priority="191" stopIfTrue="1" operator="lessThan">
       <formula>F16</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="189" priority="192" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>F16</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G16:AD16">
+    <cfRule type="expression" dxfId="189" priority="190">
+      <formula>ISERROR(G16)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G17:AD17">
-    <cfRule type="expression" dxfId="188" priority="187">
-      <formula>ISERROR(G17)</formula>
+    <cfRule type="cellIs" dxfId="188" priority="189" stopIfTrue="1" operator="lessThanOrEqual">
+      <formula>F17</formula>
     </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17:AD17">
     <cfRule type="cellIs" dxfId="187" priority="188" stopIfTrue="1" operator="greaterThan">
       <formula>F17</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="186" priority="189" stopIfTrue="1" operator="lessThanOrEqual">
-      <formula>F17</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G17:AD17">
+    <cfRule type="expression" dxfId="186" priority="187">
+      <formula>ISERROR(G17)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G18:AD18">
-    <cfRule type="expression" dxfId="185" priority="184">
-      <formula>ISERROR(G18)</formula>
+    <cfRule type="cellIs" dxfId="185" priority="186" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>F18</formula>
     </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G18:AD18">
     <cfRule type="cellIs" dxfId="184" priority="185" stopIfTrue="1" operator="lessThan">
       <formula>F18</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="183" priority="186" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>F18</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G18:AD18">
+    <cfRule type="expression" dxfId="183" priority="184">
+      <formula>ISERROR(G18)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G19:AD19">
-    <cfRule type="expression" dxfId="182" priority="181">
+    <cfRule type="expression" dxfId="182" priority="182">
       <formula>ISERROR(G19)</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="181" priority="182" stopIfTrue="1" operator="lessThan">
+    <cfRule type="cellIs" dxfId="181" priority="183" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>F19</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="180" priority="183" stopIfTrue="1" operator="greaterThanOrEqual">
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G19:AD19">
+    <cfRule type="cellIs" dxfId="180" priority="181" stopIfTrue="1" operator="lessThan">
       <formula>F19</formula>
     </cfRule>
   </conditionalFormatting>
@@ -85913,86 +86128,87 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="AH3:AH96" xr:uid="{59570CE4-F1A7-4DEB-BEF1-9189FC5F643B}">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="AH3:AH96" xr:uid="{AF63E834-3B73-4010-83D4-3865E120A78E}">
       <formula1>FormatOptions</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" display="https://fred.stlouisfed.org/series/MPCTXXXXS" xr:uid="{88492EB0-DAFC-43DA-AA6E-8ABFACDF74DA}"/>
-    <hyperlink ref="C5" r:id="rId2" display="https://fred.stlouisfed.org/series/TLPRVCONS" xr:uid="{51ED0711-A4A6-4EC0-87CD-768952C59674}"/>
-    <hyperlink ref="C6" r:id="rId3" display="https://fred.stlouisfed.org/series/TLRESCONS" xr:uid="{A6E57FC2-44A8-4D77-8BE4-1588F7A4FB82}"/>
-    <hyperlink ref="C7" r:id="rId4" display="https://fred.stlouisfed.org/series/TLHWYCONS" xr:uid="{E342A80F-5D09-43A4-A607-108DA69F5250}"/>
-    <hyperlink ref="C8" r:id="rId5" display="https://fred.stlouisfed.org/series/HSN1F" xr:uid="{4CAC796E-C454-48BC-AF5D-7E487E64DBF8}"/>
-    <hyperlink ref="C9" r:id="rId6" display="https://fred.stlouisfed.org/series/HOUST" xr:uid="{4C50C442-CEB4-464C-A8B4-698DA3C83E77}"/>
-    <hyperlink ref="C11" r:id="rId7" display="https://fred.stlouisfed.org/series/UNDCONTSA" xr:uid="{0F260AED-6919-40F9-9FA9-A03647350B4D}"/>
-    <hyperlink ref="C12" r:id="rId8" display="https://fred.stlouisfed.org/series/PERMIT" xr:uid="{2B84BD33-2999-44E3-8621-426775320981}"/>
-    <hyperlink ref="C13" r:id="rId9" display="https://fred.stlouisfed.org/series/MORTGAGE30US" xr:uid="{0C2ED4C5-488A-4BBE-B4EA-1B363F96129E}"/>
-    <hyperlink ref="C16" r:id="rId10" display="https://fred.stlouisfed.org/series/ALTSALES" xr:uid="{29943286-2182-46B4-97CE-C4CAA8FB7BA2}"/>
-    <hyperlink ref="C17" r:id="rId11" display="https://fred.stlouisfed.org/series/AISRSA" xr:uid="{4103B93B-1544-4C95-82DF-D24BA8BC1267}"/>
-    <hyperlink ref="C18" r:id="rId12" display="https://fred.stlouisfed.org/series/DAUTOSAAR" xr:uid="{E2C40C17-B823-4590-A2F0-D99B1E4BC214}"/>
-    <hyperlink ref="C19" r:id="rId13" display="https://fred.stlouisfed.org/series/DAUPSA" xr:uid="{02184A29-46CE-4577-906C-BA2DEC01002C}"/>
-    <hyperlink ref="C23" r:id="rId14" display="https://fred.stlouisfed.org/series/UNEMPLOY" xr:uid="{BA2E6E8F-FC3F-481F-9213-80A99F0C1C73}"/>
-    <hyperlink ref="C24" r:id="rId15" display="https://fred.stlouisfed.org/series/UNRATE" xr:uid="{381059A2-79C3-4DCF-B9BD-B20984340AAB}"/>
-    <hyperlink ref="C25" r:id="rId16" display="https://fred.stlouisfed.org/series/AWHNONAG" xr:uid="{BB856BE4-5360-486E-82EA-14FA7C8FC7A1}"/>
-    <hyperlink ref="C26" r:id="rId17" display="https://fred.stlouisfed.org/series/CLF16OV" xr:uid="{480742D5-D142-4908-8C6C-D31527FEA5D2}"/>
-    <hyperlink ref="C29" r:id="rId18" display="https://fred.stlouisfed.org/series/INDPRO" xr:uid="{390EB9FD-4F2A-4C45-800A-919FE9BD7FEF}"/>
-    <hyperlink ref="C30" r:id="rId19" display="https://fred.stlouisfed.org/series/TCU" xr:uid="{8183AACC-1A78-4FC7-97E8-AABE9E09E1DF}"/>
-    <hyperlink ref="C31" r:id="rId20" display="https://fred.stlouisfed.org/series/AMTMNO" xr:uid="{38FA034D-65D2-4523-A5A8-5240DF6B26F0}"/>
-    <hyperlink ref="C32" r:id="rId21" display="https://fred.stlouisfed.org/series/DGORDER" xr:uid="{7FFC5C59-24F5-47E2-B40A-0F347501A82B}"/>
-    <hyperlink ref="C33" r:id="rId22" display="https://fred.stlouisfed.org/series/ANXAVS" xr:uid="{CF941BB3-EEF8-4DC1-ADB0-6882150A6C4B}"/>
-    <hyperlink ref="C36" r:id="rId23" display="https://fred.stlouisfed.org/series/BUSINV" xr:uid="{E9FB583A-0D83-4091-A98A-8690479AF6EC}"/>
-    <hyperlink ref="C37" r:id="rId24" display="https://fred.stlouisfed.org/series/ISRATIO" xr:uid="{C666B7C2-6CEE-46B1-B571-8EDBB9FD7C4F}"/>
-    <hyperlink ref="C38" r:id="rId25" display="https://fred.stlouisfed.org/series/RETAILMPCIMSA" xr:uid="{D3A86B1A-98E7-4167-BF41-DBE652B682B9}"/>
-    <hyperlink ref="C39" r:id="rId26" display="https://fred.stlouisfed.org/series/ACNGTI" xr:uid="{A35BC242-06E8-4D6F-A8F7-F426E6559583}"/>
-    <hyperlink ref="C42" r:id="rId27" display="https://fred.stlouisfed.org/series/CPIAUCSL" xr:uid="{6CAED720-D0B9-4D5D-89A9-391B538440FA}"/>
-    <hyperlink ref="C43" r:id="rId28" display="https://fred.stlouisfed.org/series/CPIFABSL" xr:uid="{DE84378F-AE11-4685-8846-B5B5103B4C3F}"/>
-    <hyperlink ref="C44" r:id="rId29" display="https://fred.stlouisfed.org/series/CPIENGSL" xr:uid="{E0181EC3-C708-465E-821D-95277897B72C}"/>
-    <hyperlink ref="C45" r:id="rId30" display="https://fred.stlouisfed.org/series/CPILFESL" xr:uid="{F9A83B9D-71DE-43F7-ADB5-BCDF2CDDA9E4}"/>
-    <hyperlink ref="C48" r:id="rId31" display="https://fred.stlouisfed.org/series/WPUFD49207" xr:uid="{45871092-8FC4-40F6-8492-8E5DD0961E1E}"/>
-    <hyperlink ref="C49" r:id="rId32" display="https://fred.stlouisfed.org/series/WPSID61" xr:uid="{12F56867-DE78-444C-8FE0-7C48B7F74FDF}"/>
-    <hyperlink ref="C50" r:id="rId33" display="https://fred.stlouisfed.org/series/PRAWMINDEXM" xr:uid="{DECC3A48-9115-4F9A-ACDB-BC793C9F6794}"/>
-    <hyperlink ref="C52" r:id="rId34" display="https://fred.stlouisfed.org/series/DCOILWTICO" xr:uid="{AF0D0BB8-32D2-40AD-A94C-2653CB33784A}"/>
-    <hyperlink ref="C53" r:id="rId35" display="https://fred.stlouisfed.org/series/DCOILBRENTEU" xr:uid="{467B1EE6-8799-4E3C-9B0D-4707E5945CDB}"/>
-    <hyperlink ref="C54" r:id="rId36" display="https://fred.stlouisfed.org/series/DHHNGSP" xr:uid="{1F895757-63B9-494F-A4FF-F6080DFB290D}"/>
-    <hyperlink ref="C58" r:id="rId37" display="https://fred.stlouisfed.org/series/DHHNGSP" xr:uid="{A89B5976-1F8F-4ECE-B907-2428BAFE699B}"/>
-    <hyperlink ref="C59" r:id="rId38" display="https://fred.stlouisfed.org/series/PI" xr:uid="{4F0D0A91-9D7B-4767-B4DB-2ED9BC2AF842}"/>
-    <hyperlink ref="C60" r:id="rId39" display="https://fred.stlouisfed.org/series/DSPI" xr:uid="{1AC8416C-8AAD-4627-A04C-E7157DB4F40B}"/>
-    <hyperlink ref="C61" r:id="rId40" display="https://fred.stlouisfed.org/series/A229RX0" xr:uid="{72DA8C32-A6A0-4B5E-A0F0-71B88D192ECC}"/>
-    <hyperlink ref="C62" r:id="rId41" display="https://fred.stlouisfed.org/series/PSAVERT" xr:uid="{321E91F4-5E3B-4FDD-94DD-8CDB479205DF}"/>
-    <hyperlink ref="C63" r:id="rId42" display="https://fred.stlouisfed.org/series/PCE" xr:uid="{6B08D37A-82E1-476D-B243-DAD6A5812006}"/>
-    <hyperlink ref="C64" r:id="rId43" display="https://fred.stlouisfed.org/series/PCEC96" xr:uid="{690EE849-E3CF-4FBC-B09B-6A42B5FA4074}"/>
-    <hyperlink ref="C65" r:id="rId44" display="https://fred.stlouisfed.org/series/MRTSMPCSM44X72USS" xr:uid="{0161B883-9F92-490D-B7B7-23697DC57532}"/>
-    <hyperlink ref="C66" r:id="rId45" display="https://fred.stlouisfed.org/series/TOTALSL" xr:uid="{2AB2F327-11E4-4BA3-B1A9-6540C7B9BFD0}"/>
-    <hyperlink ref="C67" r:id="rId46" display="https://fred.stlouisfed.org/series/PCEND" xr:uid="{56A85A3A-23F6-4421-8AA5-7C2450E4FE09}"/>
-    <hyperlink ref="C68" r:id="rId47" display="https://fred.stlouisfed.org/series/A22BVS" xr:uid="{E6EE3BD4-804A-46F1-A048-0C5F8C03F0F3}"/>
-    <hyperlink ref="C71" r:id="rId48" display="https://fred.stlouisfed.org/series/M1SL" xr:uid="{9E9F5E70-7074-419D-B9C1-3D43045B4F67}"/>
-    <hyperlink ref="C72" r:id="rId49" display="https://fred.stlouisfed.org/series/M2SL" xr:uid="{79D018E4-63A0-4779-911B-85E67FA26776}"/>
-    <hyperlink ref="C74" r:id="rId50" display="https://fred.stlouisfed.org/series/DTB3" xr:uid="{DD3AE14C-BC47-4CD2-9CC5-0FD9F277BAA1}"/>
-    <hyperlink ref="C75" r:id="rId51" display="https://fred.stlouisfed.org/series/DPRIME" xr:uid="{58055FE9-5E72-4B60-B5A4-93A160022241}"/>
-    <hyperlink ref="C76" r:id="rId52" display="https://fred.stlouisfed.org/series/DGS10" xr:uid="{38BD90B9-DB91-445C-B6EB-FC4203135E9B}"/>
-    <hyperlink ref="C79" r:id="rId53" display="https://fred.stlouisfed.org/series/DFII10" xr:uid="{64A044AA-484E-4D65-84C0-B04E92E37CA9}"/>
-    <hyperlink ref="C80" r:id="rId54" display="https://fred.stlouisfed.org/series/DGS30" xr:uid="{47BD0F7F-EAF5-4B4F-AD96-8A68085225E3}"/>
-    <hyperlink ref="C82" r:id="rId55" display="https://fred.stlouisfed.org/series/DEXUSEU" xr:uid="{6CE12038-E30E-4370-941D-15E93C227966}"/>
-    <hyperlink ref="C83" r:id="rId56" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{B394A429-564E-481A-AFF6-BFEAE5177221}"/>
-    <hyperlink ref="C87" r:id="rId57" display="https://fred.stlouisfed.org/series/GDPC1" xr:uid="{4034F284-75B4-4569-9E76-4B32421526E3}"/>
-    <hyperlink ref="C88" r:id="rId58" display="https://fred.stlouisfed.org/series/GDP" xr:uid="{588DED00-9B68-4F1C-8F32-8C4D21136C50}"/>
-    <hyperlink ref="C89" r:id="rId59" display="https://fred.stlouisfed.org/series/PCEDG" xr:uid="{564F3239-EBC9-4EF7-84D7-3ACD7B166BF1}"/>
-    <hyperlink ref="C90" r:id="rId60" display="https://fred.stlouisfed.org/series/PNFIC1" xr:uid="{11DC3ED1-F2D4-4744-9260-2A1220A68388}"/>
-    <hyperlink ref="C91" r:id="rId61" display="https://fred.stlouisfed.org/series/PRFIC1" xr:uid="{C14B1D11-3EB3-4303-A4E0-961C355CB636}"/>
-    <hyperlink ref="C92" r:id="rId62" display="https://fred.stlouisfed.org/series/CBI" xr:uid="{45429FC9-3AA3-4A0D-A103-B6DCBDFB02E3}"/>
-    <hyperlink ref="C93" r:id="rId63" display="https://fred.stlouisfed.org/series/NETEXC" xr:uid="{623792BD-5A1A-45A7-9D65-4FFE3FAED79A}"/>
-    <hyperlink ref="C94" r:id="rId64" display="https://fred.stlouisfed.org/series/IEABC" xr:uid="{CDF709E8-2580-4B9D-A34F-9D4E79C83A96}"/>
-    <hyperlink ref="C73" r:id="rId65" display="https://fred.stlouisfed.org/series/BOPGSTB" xr:uid="{C430C1FD-32E0-4CF6-8DD9-A1BAE4550003}"/>
-    <hyperlink ref="C95" r:id="rId66" display="https://fred.stlouisfed.org/series/GCEC1" xr:uid="{582D6B52-63D9-4D4B-955C-669DDDE74A70}"/>
-    <hyperlink ref="C96" r:id="rId67" display="https://fred.stlouisfed.org/series/EVACANTUSQ176N" xr:uid="{6212F3CD-E92F-4CE2-8E6E-CBBF5D8AE27E}"/>
-    <hyperlink ref="C81" r:id="rId68" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{D48A420B-44AA-4745-B5B8-7E8DFE64327C}"/>
-    <hyperlink ref="C78" r:id="rId69" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{12C20E0D-844F-477E-B275-824D512F1252}"/>
-    <hyperlink ref="C77" r:id="rId70" display="https://fred.stlouisfed.org/series/DGS10" xr:uid="{A17D4AF5-3A65-4E13-8B7F-487D054CD9B7}"/>
-    <hyperlink ref="C51" r:id="rId71" display="https://fred.stlouisfed.org/series/PRAWMINDEXM" xr:uid="{D148DAA5-1E60-4666-8AB7-856546DB8AF7}"/>
-    <hyperlink ref="C22" r:id="rId72" display="https://fred.stlouisfed.org/series/PAYEMS" xr:uid="{8FA511F7-8A6D-45CA-9397-57D9EA0A8D79}"/>
+    <hyperlink ref="C4" r:id="rId1" display="https://fred.stlouisfed.org/series/MPCTXXXXS" xr:uid="{CD39BC6D-9D78-4490-9FBB-D1C56712D8FE}"/>
+    <hyperlink ref="C5" r:id="rId2" display="https://fred.stlouisfed.org/series/TLPRVCONS" xr:uid="{1C84536D-F29F-4E79-B65A-B7779466C2E6}"/>
+    <hyperlink ref="C6" r:id="rId3" display="https://fred.stlouisfed.org/series/TLRESCONS" xr:uid="{9D611DD8-81FA-4EBB-808D-95725C24D5DD}"/>
+    <hyperlink ref="C7" r:id="rId4" display="https://fred.stlouisfed.org/series/TLHWYCONS" xr:uid="{81E4D87D-67D2-4A64-B95C-E75BF7E9D8DE}"/>
+    <hyperlink ref="C8" r:id="rId5" display="https://fred.stlouisfed.org/series/HSN1F" xr:uid="{82F2BFEA-71A0-42E8-8771-4F8D8D7C1271}"/>
+    <hyperlink ref="C9" r:id="rId6" display="https://fred.stlouisfed.org/series/HOUST" xr:uid="{F89DB7FE-D506-4565-8661-6ED5581FF450}"/>
+    <hyperlink ref="C11" r:id="rId7" display="https://fred.stlouisfed.org/series/UNDCONTSA" xr:uid="{C374F2D1-9E8D-4982-AEFA-8C97D15044ED}"/>
+    <hyperlink ref="C12" r:id="rId8" display="https://fred.stlouisfed.org/series/PERMIT" xr:uid="{DAC9D067-CF54-4034-AAAB-042066987EA3}"/>
+    <hyperlink ref="C13" r:id="rId9" display="https://fred.stlouisfed.org/series/MORTGAGE30US" xr:uid="{8F2CD11C-A9DC-48F6-B36F-E9983D40201B}"/>
+    <hyperlink ref="C16" r:id="rId10" display="https://fred.stlouisfed.org/series/ALTSALES" xr:uid="{2D32F66F-4919-4F12-87D4-BA6209F76557}"/>
+    <hyperlink ref="C17" r:id="rId11" display="https://fred.stlouisfed.org/series/AISRSA" xr:uid="{76DB66F4-8ABC-4A8A-858D-800BFFE7F11D}"/>
+    <hyperlink ref="C18" r:id="rId12" display="https://fred.stlouisfed.org/series/DAUTOSAAR" xr:uid="{EC4D1C19-1D1C-48A6-81D0-802A2698B542}"/>
+    <hyperlink ref="C19" r:id="rId13" display="https://fred.stlouisfed.org/series/DAUPSA" xr:uid="{62649C48-BB04-458B-8EE5-65510B11E0C0}"/>
+    <hyperlink ref="C23" r:id="rId14" display="https://fred.stlouisfed.org/series/UNEMPLOY" xr:uid="{F4E0FE54-BB53-4441-BC52-555C009C2A9D}"/>
+    <hyperlink ref="C24" r:id="rId15" display="https://fred.stlouisfed.org/series/UNRATE" xr:uid="{6D2B1CA5-A842-44D6-A2C7-A80FF1C0E142}"/>
+    <hyperlink ref="C25" r:id="rId16" display="https://fred.stlouisfed.org/series/AWHNONAG" xr:uid="{340737A8-4C52-4F1B-B21B-896875CA8F94}"/>
+    <hyperlink ref="C26" r:id="rId17" display="https://fred.stlouisfed.org/series/CLF16OV" xr:uid="{2695759F-61E1-4AB9-A361-DC5B15E1A1EC}"/>
+    <hyperlink ref="C29" r:id="rId18" display="https://fred.stlouisfed.org/series/INDPRO" xr:uid="{F3D77017-0712-413D-B595-2B7A6B73BD75}"/>
+    <hyperlink ref="C30" r:id="rId19" display="https://fred.stlouisfed.org/series/TCU" xr:uid="{19DF77CD-D739-4C59-9756-29742EF2F9C0}"/>
+    <hyperlink ref="C31" r:id="rId20" display="https://fred.stlouisfed.org/series/AMTMNO" xr:uid="{50444CED-9515-4BAD-AF80-5DACA9113328}"/>
+    <hyperlink ref="C32" r:id="rId21" display="https://fred.stlouisfed.org/series/DGORDER" xr:uid="{8B8268B7-469D-45B3-A2E1-1A858D362359}"/>
+    <hyperlink ref="C33" r:id="rId22" display="https://fred.stlouisfed.org/series/ANXAVS" xr:uid="{FD27DA25-3BE0-4EB2-84E7-53D768CF7C3A}"/>
+    <hyperlink ref="C36" r:id="rId23" display="https://fred.stlouisfed.org/series/BUSINV" xr:uid="{6A873BDB-B866-4000-A11D-171DDFC95CFC}"/>
+    <hyperlink ref="C37" r:id="rId24" display="https://fred.stlouisfed.org/series/ISRATIO" xr:uid="{59A2A9D5-DFAE-43B7-8327-569F1EE7C5BB}"/>
+    <hyperlink ref="C38" r:id="rId25" display="https://fred.stlouisfed.org/series/RETAILMPCIMSA" xr:uid="{8B3E4CC4-B704-4F2F-9A66-2BD5CF14EF3D}"/>
+    <hyperlink ref="C39" r:id="rId26" display="https://fred.stlouisfed.org/series/ACNGTI" xr:uid="{C70A1BE3-BE44-4565-8B3F-24D5B330E051}"/>
+    <hyperlink ref="C42" r:id="rId27" display="https://fred.stlouisfed.org/series/CPIAUCSL" xr:uid="{6371530A-9723-4AAF-93E4-A1B323ABFA0D}"/>
+    <hyperlink ref="C43" r:id="rId28" display="https://fred.stlouisfed.org/series/CPIFABSL" xr:uid="{8131B5C7-F019-40AE-86CC-B99F20C34796}"/>
+    <hyperlink ref="C44" r:id="rId29" display="https://fred.stlouisfed.org/series/CPIENGSL" xr:uid="{A4BD50DB-1CB2-450E-8744-14DAD65A4C09}"/>
+    <hyperlink ref="C45" r:id="rId30" display="https://fred.stlouisfed.org/series/CPILFESL" xr:uid="{F62AC6D2-1626-4D9F-AA7A-68539696D2EB}"/>
+    <hyperlink ref="C48" r:id="rId31" display="https://fred.stlouisfed.org/series/WPUFD49207" xr:uid="{41486A7F-88B8-4434-A528-B9AD8C44EB29}"/>
+    <hyperlink ref="C49" r:id="rId32" display="https://fred.stlouisfed.org/series/WPSID61" xr:uid="{B3211A87-677B-466E-AA73-799CE9BC959A}"/>
+    <hyperlink ref="C50" r:id="rId33" display="https://fred.stlouisfed.org/series/PRAWMINDEXM" xr:uid="{1D1E2913-ECED-4418-B52F-D41CE822CD78}"/>
+    <hyperlink ref="C52" r:id="rId34" display="https://fred.stlouisfed.org/series/DCOILWTICO" xr:uid="{4E3D9225-393C-42FD-9E54-70AEE5E19E18}"/>
+    <hyperlink ref="C53" r:id="rId35" display="https://fred.stlouisfed.org/series/DCOILBRENTEU" xr:uid="{83D96DB9-E00F-4BA2-8666-57BF72B8D947}"/>
+    <hyperlink ref="C54" r:id="rId36" display="https://fred.stlouisfed.org/series/DHHNGSP" xr:uid="{E6AB1452-CCE1-4708-95F8-38060A02B6FA}"/>
+    <hyperlink ref="C58" r:id="rId37" display="https://fred.stlouisfed.org/series/DHHNGSP" xr:uid="{5391735B-6370-41C4-8A0D-7335925C3313}"/>
+    <hyperlink ref="C59" r:id="rId38" display="https://fred.stlouisfed.org/series/PI" xr:uid="{8CF0F396-EA10-469F-A7D0-FB7D6966A1E9}"/>
+    <hyperlink ref="C60" r:id="rId39" display="https://fred.stlouisfed.org/series/DSPI" xr:uid="{6CF152BD-6FAB-48BB-8D73-317C9F8C4679}"/>
+    <hyperlink ref="C61" r:id="rId40" display="https://fred.stlouisfed.org/series/A229RX0" xr:uid="{6E66FA21-561F-442C-8AED-7F3451609ACD}"/>
+    <hyperlink ref="C62" r:id="rId41" display="https://fred.stlouisfed.org/series/PSAVERT" xr:uid="{9943EFA2-D33C-4335-8BDA-FB2CB49DD5B6}"/>
+    <hyperlink ref="C63" r:id="rId42" display="https://fred.stlouisfed.org/series/PCE" xr:uid="{A1C659D2-AB0F-4C23-9FC1-48B50847FE94}"/>
+    <hyperlink ref="C64" r:id="rId43" display="https://fred.stlouisfed.org/series/PCEC96" xr:uid="{96268601-C9C1-4CF0-BAE0-4E9328C26DF9}"/>
+    <hyperlink ref="C65" r:id="rId44" display="https://fred.stlouisfed.org/series/MRTSMPCSM44X72USS" xr:uid="{BEEA9057-2C8D-481E-A448-2FB895AAE0C9}"/>
+    <hyperlink ref="C66" r:id="rId45" display="https://fred.stlouisfed.org/series/TOTALSL" xr:uid="{F2FC4417-39A4-4E48-A780-56ED9F0EE6FF}"/>
+    <hyperlink ref="C67" r:id="rId46" display="https://fred.stlouisfed.org/series/PCEND" xr:uid="{AE2846B6-5848-4D02-B901-230031F5E80A}"/>
+    <hyperlink ref="C68" r:id="rId47" display="https://fred.stlouisfed.org/series/A22BVS" xr:uid="{1C163D8C-2DAC-4418-A07C-3D8CADC042CC}"/>
+    <hyperlink ref="C71" r:id="rId48" display="https://fred.stlouisfed.org/series/M1SL" xr:uid="{8EF7ABB6-14F0-41DE-AB94-712828CF85D9}"/>
+    <hyperlink ref="C72" r:id="rId49" display="https://fred.stlouisfed.org/series/M2SL" xr:uid="{77698096-D653-4B09-837C-96C6208BBD36}"/>
+    <hyperlink ref="C74" r:id="rId50" display="https://fred.stlouisfed.org/series/DTB3" xr:uid="{E4DB2C80-A0A0-4131-9A1D-E2698E1F78B6}"/>
+    <hyperlink ref="C75" r:id="rId51" display="https://fred.stlouisfed.org/series/DPRIME" xr:uid="{F32BBCEB-B780-4AFB-AFFE-998E3274BB02}"/>
+    <hyperlink ref="C76" r:id="rId52" display="https://fred.stlouisfed.org/series/DGS10" xr:uid="{D83A0E77-4079-4364-A0A3-45F5ADFA276B}"/>
+    <hyperlink ref="C79" r:id="rId53" display="https://fred.stlouisfed.org/series/DFII10" xr:uid="{BA89AFCD-D387-4E00-AAB5-C2D2534E8743}"/>
+    <hyperlink ref="C80" r:id="rId54" display="https://fred.stlouisfed.org/series/DGS30" xr:uid="{7F7EC27E-527B-4C0C-9FDA-6C912680F336}"/>
+    <hyperlink ref="C82" r:id="rId55" display="https://fred.stlouisfed.org/series/DEXUSEU" xr:uid="{25F3C874-FE00-4535-B4DD-3A30518EA849}"/>
+    <hyperlink ref="C83" r:id="rId56" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{9030AF68-3C49-44A8-90AA-1A5E4F6113B7}"/>
+    <hyperlink ref="C87" r:id="rId57" display="https://fred.stlouisfed.org/series/GDPC1" xr:uid="{9DB904B5-3BC5-4510-A748-7C3D4C0F38D1}"/>
+    <hyperlink ref="C88" r:id="rId58" display="https://fred.stlouisfed.org/series/GDP" xr:uid="{1ACAA390-08C4-45BF-8571-843776D1C1D9}"/>
+    <hyperlink ref="C89" r:id="rId59" display="https://fred.stlouisfed.org/series/PCEDG" xr:uid="{9C517E6D-3EAB-4F68-AB29-11398FFBF0CC}"/>
+    <hyperlink ref="C90" r:id="rId60" display="https://fred.stlouisfed.org/series/PNFIC1" xr:uid="{8215BF73-261D-4E83-8323-8A1F57F57AEE}"/>
+    <hyperlink ref="C91" r:id="rId61" display="https://fred.stlouisfed.org/series/PRFIC1" xr:uid="{EC1D0141-1585-4214-BC09-A622DB9C9859}"/>
+    <hyperlink ref="C92" r:id="rId62" display="https://fred.stlouisfed.org/series/CBI" xr:uid="{CA41EBBB-B5D7-4058-AEDF-3C8BF63849A3}"/>
+    <hyperlink ref="C93" r:id="rId63" display="https://fred.stlouisfed.org/series/NETEXC" xr:uid="{3945D75E-2482-4E4B-8209-2945EF1A71E7}"/>
+    <hyperlink ref="C94" r:id="rId64" display="https://fred.stlouisfed.org/series/IEABC" xr:uid="{BEA7FC97-9663-4B3F-BBA8-1F8E3A5330B2}"/>
+    <hyperlink ref="C73" r:id="rId65" display="https://fred.stlouisfed.org/series/BOPGSTB" xr:uid="{3C7CCF8A-2F44-43C9-91B3-971D9DE9FF3A}"/>
+    <hyperlink ref="C95" r:id="rId66" display="https://fred.stlouisfed.org/series/GCEC1" xr:uid="{64A0DE43-DCDF-4F61-BF15-39FC5587A039}"/>
+    <hyperlink ref="C96" r:id="rId67" display="https://fred.stlouisfed.org/series/EVACANTUSQ176N" xr:uid="{3D5744C7-269C-4BAC-9EC1-3C19036537AB}"/>
+    <hyperlink ref="C81" r:id="rId68" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{7859D2DF-84ED-4A6B-B4CE-B86D61DB02DD}"/>
+    <hyperlink ref="C78" r:id="rId69" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{B3EBFDE6-6BA5-46D4-A8D0-54F6B03E1A07}"/>
+    <hyperlink ref="C77" r:id="rId70" display="https://fred.stlouisfed.org/series/DGS10" xr:uid="{4400573F-16B8-4D59-B5A7-D292678946C7}"/>
+    <hyperlink ref="C51" r:id="rId71" display="https://fred.stlouisfed.org/series/PRAWMINDEXM" xr:uid="{34D3BF34-58B8-49DA-BC33-66C43975517E}"/>
+    <hyperlink ref="C22" r:id="rId72" display="https://fred.stlouisfed.org/series/PAYEMS" xr:uid="{AEE8F153-1FCF-44F3-BB12-DA8A3701FBB8}"/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.3" footer="0.3"/>
   <pageSetup scale="64" orientation="landscape" r:id="rId73"/>
   <drawing r:id="rId74"/>
+  <legacyDrawing r:id="rId75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Publish EconSheet 261019 (October 19, 2026)
</commit_message>
<xml_diff>
--- a/files/EconSheet.xlsx
+++ b/files/EconSheet.xlsx
@@ -8,44 +8,44 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.0.130\Documents\Business\EconSheet\FREDData\ToDistribute\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{40A155C1-B606-4BD7-A082-15B1842CB866}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{BED8F52D-4100-4EA3-88DA-3D0A44F283A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5295" windowWidth="29040" windowHeight="15720" xr2:uid="{AFA123A0-8550-40FB-95F4-DD256DF0E98B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{0425FD2D-B739-4B05-B6DC-E6B9D2EE0831}"/>
   </bookViews>
   <sheets>
-    <sheet name="261016 EconSheet" sheetId="1" r:id="rId1"/>
+    <sheet name="261019 EconSheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId2"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'261016 EconSheet'!$A$28:$AF$33</definedName>
-    <definedName name="Conditions" localSheetId="0">'261016 EconSheet'!$AH$3:$AH$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'261019 EconSheet'!$A$28:$AF$33</definedName>
+    <definedName name="Conditions" localSheetId="0">'261019 EconSheet'!$AH$3:$AH$96</definedName>
     <definedName name="CurrDates">[1]Currencies!$A$8:$A$14337</definedName>
     <definedName name="DataStart">'[1]Retrieved Data'!$A$1</definedName>
-    <definedName name="DataTable" localSheetId="0">'261016 EconSheet'!$G$4:$AD$96</definedName>
-    <definedName name="DataTableStart" localSheetId="0">'261016 EconSheet'!$G$4</definedName>
-    <definedName name="DatesAndSeries" localSheetId="0">'261016 EconSheet'!$E$4:$F$96</definedName>
+    <definedName name="DataTable" localSheetId="0">'261019 EconSheet'!$G$4:$AD$96</definedName>
+    <definedName name="DataTableStart" localSheetId="0">'261019 EconSheet'!$G$4</definedName>
+    <definedName name="DatesAndSeries" localSheetId="0">'261019 EconSheet'!$E$4:$F$96</definedName>
     <definedName name="DatesAndSeries">[1]EconSheet!$E$4:$F$96</definedName>
-    <definedName name="DatesCol" localSheetId="0">'261016 EconSheet'!$E$4:$E$96</definedName>
+    <definedName name="DatesCol" localSheetId="0">'261019 EconSheet'!$E$4:$E$96</definedName>
     <definedName name="DatesCol">[1]EconSheet!$E$4:$E$96</definedName>
-    <definedName name="ESSeries" localSheetId="0">'261016 EconSheet'!$B$4:$B$103</definedName>
-    <definedName name="ForceAll" localSheetId="0">'261016 EconSheet'!#REF!</definedName>
+    <definedName name="ESSeries" localSheetId="0">'261019 EconSheet'!$B$4:$B$103</definedName>
+    <definedName name="ForceAll" localSheetId="0">'261019 EconSheet'!#REF!</definedName>
     <definedName name="FormatOptions">[1]Calculations!$U$3:$U$14</definedName>
-    <definedName name="FormatTable" localSheetId="0">'261016 EconSheet'!$A$1:$AD$96</definedName>
+    <definedName name="FormatTable" localSheetId="0">'261019 EconSheet'!$A$1:$AD$96</definedName>
     <definedName name="PPIGreen">'[1]Producer Price Archive'!$AB$8:$AD$1023</definedName>
     <definedName name="PPIRaw">'[1]Producer Price Archive'!$B$7:$F$1023</definedName>
     <definedName name="PPIRed">'[1]Producer Price Archive'!$AF$8:$AH$1023</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'261016 EconSheet'!$F$1:$AD$54,'261016 EconSheet'!$F$56:$AD$96</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'261019 EconSheet'!$F$1:$AD$54,'261019 EconSheet'!$F$56:$AD$96</definedName>
     <definedName name="ReleaseData">[1]ReleaseDates!$A$2:$E$1882</definedName>
     <definedName name="ReleaseDates">[1]ReleaseDates!$A$2:$A$1898</definedName>
     <definedName name="SDSeries">[1]SeriesData!$A$2:$A$76</definedName>
     <definedName name="SeriesLookup">'[1]Retrieved Data'!$A$1:$ET$1</definedName>
-    <definedName name="SpFormat1" localSheetId="0">'261016 EconSheet'!$AH$131</definedName>
-    <definedName name="SpFormat2" localSheetId="0">'261016 EconSheet'!$AH$136</definedName>
-    <definedName name="TrueFalse" localSheetId="0">'261016 EconSheet'!#REF!</definedName>
+    <definedName name="SpFormat1" localSheetId="0">'261019 EconSheet'!$AH$131</definedName>
+    <definedName name="SpFormat2" localSheetId="0">'261019 EconSheet'!$AH$136</definedName>
+    <definedName name="TrueFalse" localSheetId="0">'261019 EconSheet'!#REF!</definedName>
     <definedName name="TrueFalse">[1]EconSheet!$AU$1:$AU$2</definedName>
-    <definedName name="WholeTable" localSheetId="0">'261016 EconSheet'!$F$1:$AD$96</definedName>
+    <definedName name="WholeTable" localSheetId="0">'261019 EconSheet'!$F$1:$AD$96</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -76,20 +76,7 @@
     <author>Ron Levin</author>
   </authors>
   <commentList>
-    <comment ref="AD13" authorId="0" shapeId="0" xr:uid="{AACE8B5E-70C0-44D8-AADB-034DF6FD0328}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>New Value</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H36" authorId="0" shapeId="0" xr:uid="{6917E528-D49F-4EF6-9728-74582F40C3B4}">
+    <comment ref="X29" authorId="0" shapeId="0" xr:uid="{55797B3F-3B6C-489D-BBDE-A7D108AF02E3}">
       <text>
         <r>
           <rPr>
@@ -99,25 +86,11 @@
             <family val="2"/>
           </rPr>
           <t>Previous Value:
--0.3</t>
+0.8</t>
         </r>
       </text>
     </comment>
-    <comment ref="I36" authorId="0" shapeId="0" xr:uid="{C0F198E9-75F1-43FE-AA99-DE9DD947E22F}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.4</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J36" authorId="0" shapeId="0" xr:uid="{57DC5E10-9ED6-4369-BD33-E62A20EAFD79}">
+    <comment ref="Y29" authorId="0" shapeId="0" xr:uid="{2C91E6BE-B914-4483-A3D3-F3A35CB76275}">
       <text>
         <r>
           <rPr>
@@ -131,7 +104,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K36" authorId="0" shapeId="0" xr:uid="{513EE235-028E-48A6-BFB9-03EA8C6AB9AC}">
+    <comment ref="Z29" authorId="0" shapeId="0" xr:uid="{FCEEBA06-DA9D-4788-92A6-E23B4D2C7ABC}">
       <text>
         <r>
           <rPr>
@@ -141,11 +114,11 @@
             <family val="2"/>
           </rPr>
           <t>Previous Value:
-0.1</t>
+0.2</t>
         </r>
       </text>
     </comment>
-    <comment ref="L36" authorId="0" shapeId="0" xr:uid="{127ECCE7-D62D-4963-B3CE-880AE0C69427}">
+    <comment ref="AA29" authorId="0" shapeId="0" xr:uid="{BD3070E4-BE85-498A-86A6-B33628FD63FF}">
       <text>
         <r>
           <rPr>
@@ -155,11 +128,11 @@
             <family val="2"/>
           </rPr>
           <t>Previous Value:
--0.1</t>
+0.2</t>
         </r>
       </text>
     </comment>
-    <comment ref="M36" authorId="0" shapeId="0" xr:uid="{05C80877-DA46-49D8-8EF9-E101868E5D07}">
+    <comment ref="AB29" authorId="0" shapeId="0" xr:uid="{BB441084-368F-4909-8EFD-8688D269F7E0}">
       <text>
         <r>
           <rPr>
@@ -173,203 +146,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="N36" authorId="0" shapeId="0" xr:uid="{B5BB57D2-6D76-47E5-8899-57806A92446A}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O36" authorId="0" shapeId="0" xr:uid="{A037C7BC-DDBD-4796-A448-42A0E3F3A22E}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.1</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P36" authorId="0" shapeId="0" xr:uid="{957D1557-FA7A-4C4D-94A4-C45E1A4F47F9}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.0</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Q36" authorId="0" shapeId="0" xr:uid="{D1ACFCDB-1DC6-4AAE-A4A1-121672730AD6}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.3</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R36" authorId="0" shapeId="0" xr:uid="{39758CA3-A332-428E-916A-A98CA7445A13}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="S36" authorId="0" shapeId="0" xr:uid="{F9A7531A-4B21-4F46-B311-E86CEF315E51}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.0</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="T36" authorId="0" shapeId="0" xr:uid="{33C14ACE-D84F-4554-AC99-A28475049079}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.0</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U36" authorId="0" shapeId="0" xr:uid="{289A127F-2EC7-4418-9B11-15A60047C25C}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.0</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="V36" authorId="0" shapeId="0" xr:uid="{BD963C80-441A-4B2A-B2C9-409BEB3CA716}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.4</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="W36" authorId="0" shapeId="0" xr:uid="{F6A29DE3-82B4-489F-BDF1-D41946BBD3E3}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.0</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="X36" authorId="0" shapeId="0" xr:uid="{879E304A-8C5E-4069-8B66-75B944FEE459}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.6</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Y36" authorId="0" shapeId="0" xr:uid="{CC92B3B2-2210-4C04-81C1-D873D27FB72E}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.4</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Z36" authorId="0" shapeId="0" xr:uid="{CA83DBC6-CDCD-456F-9B02-F3F7D229656A}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.1</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AA36" authorId="0" shapeId="0" xr:uid="{C15BA281-2789-4865-8555-E9FECAD6960A}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.8</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AB36" authorId="0" shapeId="0" xr:uid="{832115A4-604B-42C0-8480-B65DC7D376C6}">
+    <comment ref="AC29" authorId="0" shapeId="0" xr:uid="{9F9822E7-A64D-4D53-A9DD-8D8EA88E8535}">
       <text>
         <r>
           <rPr>
@@ -382,7 +159,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="H37" authorId="0" shapeId="0" xr:uid="{D2192B0B-EA69-40F7-86F6-3ED03A71E3ED}">
+    <comment ref="X30" authorId="0" shapeId="0" xr:uid="{163FB9E0-E092-4563-888B-CDE197D1AA7F}">
       <text>
         <r>
           <rPr>
@@ -392,11 +169,11 @@
             <family val="2"/>
           </rPr>
           <t>Previous Value:
-1.39</t>
+76.2</t>
         </r>
       </text>
     </comment>
-    <comment ref="I37" authorId="0" shapeId="0" xr:uid="{037072A4-B7EC-4043-B806-AB68CE845B61}">
+    <comment ref="Y30" authorId="0" shapeId="0" xr:uid="{D5B91344-1001-465D-B76A-0E6E78AF3F7B}">
       <text>
         <r>
           <rPr>
@@ -406,11 +183,11 @@
             <family val="2"/>
           </rPr>
           <t>Previous Value:
-1.40</t>
+76.2</t>
         </r>
       </text>
     </comment>
-    <comment ref="J37" authorId="0" shapeId="0" xr:uid="{03F128C3-814A-46AE-B812-E11EA9150859}">
+    <comment ref="Z30" authorId="0" shapeId="0" xr:uid="{62EEC66D-2F1F-4647-9FBC-77D07824B6AA}">
       <text>
         <r>
           <rPr>
@@ -420,11 +197,11 @@
             <family val="2"/>
           </rPr>
           <t>Previous Value:
-1.39</t>
+76.2</t>
         </r>
       </text>
     </comment>
-    <comment ref="K37" authorId="0" shapeId="0" xr:uid="{0257BA0E-A54E-480A-B23F-D3815229F6DB}">
+    <comment ref="AA30" authorId="0" shapeId="0" xr:uid="{3168B595-DB14-4EE2-A5F9-BF14301BCCA3}">
       <text>
         <r>
           <rPr>
@@ -434,11 +211,11 @@
             <family val="2"/>
           </rPr>
           <t>Previous Value:
-1.38</t>
+76.3</t>
         </r>
       </text>
     </comment>
-    <comment ref="L37" authorId="0" shapeId="0" xr:uid="{0E8D9DFD-3F3E-4184-AFEA-8DBCC7B270FB}">
+    <comment ref="AB30" authorId="0" shapeId="0" xr:uid="{EAABAAFE-CF63-4960-93C1-2F173295B25D}">
       <text>
         <r>
           <rPr>
@@ -448,874 +225,11 @@
             <family val="2"/>
           </rPr>
           <t>Previous Value:
-1.38</t>
+76.3</t>
         </r>
       </text>
     </comment>
-    <comment ref="M37" authorId="0" shapeId="0" xr:uid="{D3F498B0-76F8-4401-AB19-AD484DD2A81F}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.39</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N37" authorId="0" shapeId="0" xr:uid="{10F49DD7-2949-4403-B674-600FD378B5D2}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.39</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O37" authorId="0" shapeId="0" xr:uid="{431D624E-607D-4D16-B873-4B34525D5B60}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.37</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P37" authorId="0" shapeId="0" xr:uid="{C60A3608-179E-4B18-948A-8E93EF2B9AFE}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.37</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Q37" authorId="0" shapeId="0" xr:uid="{1C12A93B-72E0-4B41-B7F6-3CF045ACBD58}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.37</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R37" authorId="0" shapeId="0" xr:uid="{1537E8A0-204F-4F2A-B574-EFF1635A55EE}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.38</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="S37" authorId="0" shapeId="0" xr:uid="{6FF0F7B4-0122-477A-9F5B-65B7F550E356}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.37</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="T37" authorId="0" shapeId="0" xr:uid="{21B040A0-E1EA-46CE-A553-8CF0699A0421}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.36</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U37" authorId="0" shapeId="0" xr:uid="{743BA0E1-A864-4A40-8C5D-EAC5F9AD64C1}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.35</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="V37" authorId="0" shapeId="0" xr:uid="{4B4BDC34-C11B-47CC-A85C-2695C5D5AFC7}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.33</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="W37" authorId="0" shapeId="0" xr:uid="{443EEB95-7EE1-4EC4-B4A6-EC67F3DEB2FC}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.32</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="X37" authorId="0" shapeId="0" xr:uid="{E26CF813-0044-4E92-8741-BB3A68EEB645}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.30</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Y37" authorId="0" shapeId="0" xr:uid="{8D239474-90C3-4950-A8D1-2142D52BDC82}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.28</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Z37" authorId="0" shapeId="0" xr:uid="{6417D85E-E342-4429-A1EE-BCF639AA6C7D}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.30</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AA37" authorId="0" shapeId="0" xr:uid="{8D51EDB3-4681-4643-A12C-35E110C98DCF}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.30</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AB37" authorId="0" shapeId="0" xr:uid="{7576C52B-77CF-4019-898B-05CD58B26622}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>New Value</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I38" authorId="0" shapeId="0" xr:uid="{99F15BC6-7299-4134-A9C6-2364C6ED32BD}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K38" authorId="0" shapeId="0" xr:uid="{186AB709-824B-48ED-816F-918324A87CEE}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
--0.2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L38" authorId="0" shapeId="0" xr:uid="{1236DF39-6435-49D9-BF26-34CB7B6D9BF0}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
--0.3</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M38" authorId="0" shapeId="0" xr:uid="{18BCEB68-3721-40E5-9B7A-21234FE583D5}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P38" authorId="0" shapeId="0" xr:uid="{6394CABC-E682-4E67-A5EA-A7C043D3A852}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.1</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Q38" authorId="0" shapeId="0" xr:uid="{E01A061D-F9A0-46D3-819D-D6E6ABA2E167}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.5</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R38" authorId="0" shapeId="0" xr:uid="{57C052CE-5250-44F4-B0D4-912B2AE546F7}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.5</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="S38" authorId="0" shapeId="0" xr:uid="{742D2B0A-BB49-4750-B77B-1DD0F08A9372}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
--0.4</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="T38" authorId="0" shapeId="0" xr:uid="{60332EB0-36D2-4B47-B2D3-7EB79AAEA8A1}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.1</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="V38" authorId="0" shapeId="0" xr:uid="{17CC143E-9ACF-41A2-AD46-3E9A9665D9BF}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.0</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="W38" authorId="0" shapeId="0" xr:uid="{F4C03697-BD67-4D96-ACD4-652F9E075838}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.8</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Y38" authorId="0" shapeId="0" xr:uid="{EFC18014-E2D9-4A46-ADB1-C09044D12EFB}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.8</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AA38" authorId="0" shapeId="0" xr:uid="{D20096C7-17A0-4FE6-8FEB-C3CF752E1A86}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.8</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AB38" authorId="0" shapeId="0" xr:uid="{A17FEAF0-576B-4704-BB31-39C1E7C57079}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>New Value</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Y48" authorId="0" shapeId="0" xr:uid="{C9CB00F2-B023-4207-B2E5-5F7B0D141779}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-8.7</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Z48" authorId="0" shapeId="0" xr:uid="{E0603812-86A7-4C25-A598-6DF13D2F4081}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-6.6</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AA48" authorId="0" shapeId="0" xr:uid="{C75981D3-6DFF-4682-8CF0-64203EC25362}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-5.8</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AB48" authorId="0" shapeId="0" xr:uid="{59F993D5-AC55-4818-8B67-99C3249ACFF2}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-6.6</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AC48" authorId="0" shapeId="0" xr:uid="{F9778AB6-F88F-4BF0-B429-E4BB0B2EFC34}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>New Value</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Y49" authorId="0" shapeId="0" xr:uid="{F7F4C09C-B333-4F26-97CB-C695DDEADAA2}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-12.2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Z49" authorId="0" shapeId="0" xr:uid="{4213F7D0-C9F7-4BA4-901D-37B1EFA0D343}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-11.1</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AA49" authorId="0" shapeId="0" xr:uid="{40736EED-DD2D-4340-A2C7-450736A7A834}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-10.0</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AB49" authorId="0" shapeId="0" xr:uid="{713E6D77-2F30-4326-8BC7-5E624C1F0DAD}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-11.5</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AC49" authorId="0" shapeId="0" xr:uid="{4DBFD375-9FE4-4332-A1B9-0119BB6735B4}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>New Value</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Y50" authorId="0" shapeId="0" xr:uid="{EF359A2D-559B-4CC4-9311-73A03D2B991B}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-20.7</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Z50" authorId="0" shapeId="0" xr:uid="{6A5CB423-8F67-44D0-B328-4E40D22DC390}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-10.4</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AA50" authorId="0" shapeId="0" xr:uid="{39BF0F61-4F59-4EB2-B162-D0287232A3B4}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-9.8</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AB50" authorId="0" shapeId="0" xr:uid="{1C1F565A-1A95-403C-AA9F-B3DAE5213957}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-13.1</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AC50" authorId="0" shapeId="0" xr:uid="{325D045D-8989-4827-9A26-CA944163C091}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>New Value</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="H65" authorId="0" shapeId="0" xr:uid="{32B97E2B-BEDE-4867-B932-06CC3838DAAD}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.8</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="I65" authorId="0" shapeId="0" xr:uid="{3F0EA7F7-2F8D-4F32-8976-20241A5A5171}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
--0.8</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="J65" authorId="0" shapeId="0" xr:uid="{6820366A-83C1-4302-9A51-DF00743153FC}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.0</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="K65" authorId="0" shapeId="0" xr:uid="{4D4B9020-57D6-44BC-B39A-616D7553308D}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.7</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L65" authorId="0" shapeId="0" xr:uid="{A0D736A2-9F7A-4EA9-8087-749B726D5B45}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
--0.1</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="M65" authorId="0" shapeId="0" xr:uid="{18491495-C5B1-41F9-B207-2A8B1B70BCC6}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
--1.1</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="N65" authorId="0" shapeId="0" xr:uid="{60757197-6144-47C3-BF95-2AD7364A2098}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.7</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="O65" authorId="0" shapeId="0" xr:uid="{65377BAE-CB77-4E46-A648-AEE55EC000CD}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1.2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Q65" authorId="0" shapeId="0" xr:uid="{8EA7DEDE-9B48-48EA-B094-F6685A4B8605}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.3</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R65" authorId="0" shapeId="0" xr:uid="{1E1E9973-5165-40F8-BEF1-637332591B00}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
--0.2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="S65" authorId="0" shapeId="0" xr:uid="{D28B73C8-5B8F-48B8-9A0F-016C41594B43}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.5</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="T65" authorId="0" shapeId="0" xr:uid="{B22790C3-EF5F-414C-8CEA-98ABC5D72363}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.0</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="U65" authorId="0" shapeId="0" xr:uid="{D0534125-06FA-41B0-84DC-D649C9355ED4}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.0</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="X65" authorId="0" shapeId="0" xr:uid="{CB6FDFC2-CD46-455F-AA66-F666918946F5}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.7</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Y65" authorId="0" shapeId="0" xr:uid="{CC86C16B-CD4A-4059-B507-6688AF1688DB}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.9</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Z65" authorId="0" shapeId="0" xr:uid="{75608576-AF8B-4D34-B45E-01D2BFC679D4}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.3</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AA65" authorId="0" shapeId="0" xr:uid="{6EC52A88-CB1A-4F87-8D66-656324621307}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
--0.5</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AB65" authorId="0" shapeId="0" xr:uid="{599FEB3C-2645-4ABA-B68A-B4A4C9D94566}">
+    <comment ref="AC30" authorId="0" shapeId="0" xr:uid="{32D17454-8188-4CDE-B9D1-061BFBF337F6}">
       <text>
         <r>
           <rPr>
@@ -1893,7 +807,7 @@
     <t>Green if</t>
   </si>
   <si>
-    <t>Next Update: 10/16/26</t>
+    <t>Next Update: 10/20/26</t>
   </si>
   <si>
     <t>Next Update</t>
@@ -2046,7 +960,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="9">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -2105,26 +1019,6 @@
       <right style="thick">
         <color indexed="64"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thick">
-        <color indexed="64"/>
-      </left>
-      <right style="thick">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color indexed="64"/>
-      </right>
       <top style="thick">
         <color indexed="64"/>
       </top>
@@ -2150,7 +1044,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="87">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -2218,9 +1112,6 @@
     <xf numFmtId="14" fontId="12" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="14" fontId="12" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="4" fillId="3" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="4" fillId="2" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2229,27 +1120,18 @@
     </xf>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="2" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="2" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="4" fillId="4" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="2" fontId="4" fillId="2" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="168" fontId="9" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="22" fontId="9" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -2262,7 +1144,7 @@
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{BB3A8590-DB71-4F61-988A-2875B9025D6C}"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{D0FE01E7-A8B7-45DE-A2D6-B3C532B960D9}"/>
   </cellStyles>
   <dxfs count="237">
     <dxf>
@@ -3616,7 +2498,9 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="0"/>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF10651B"/>
       </font>
     </dxf>
     <dxf>
@@ -3628,9 +2512,21 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
         <color rgb="FF10651B"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF711204"/>
       </font>
     </dxf>
     <dxf>
@@ -3642,7 +2538,19 @@
       <font>
         <b/>
         <i val="0"/>
+        <color rgb="FF10651B"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
         <color rgb="FF711204"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
       </font>
     </dxf>
     <dxf>
@@ -3654,11 +2562,6 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <b/>
         <i val="0"/>
         <color rgb="FF711204"/>
@@ -3666,28 +2569,7 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF10651B"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF711204"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF10651B"/>
       </font>
     </dxf>
     <dxf>
@@ -3898,7 +2780,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{D89AFA7C-43A7-4F53-979C-3295F0ABD96B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B89EDBD4-4CA4-4396-8E4C-322A27C3062B}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -3943,7 +2825,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{58D09224-793C-44CF-B3A1-2A08230B148B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F9D60A36-CBD4-4FF0-AEF3-959CF7C68926}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -4186,7 +3068,7 @@
         </row>
         <row r="29">
           <cell r="E29">
-            <v>46311.38898148149</v>
+            <v>46343.389108796298</v>
           </cell>
           <cell r="F29" t="str">
             <v>Industrial Production (% Δ)</v>
@@ -4194,7 +3076,7 @@
         </row>
         <row r="30">
           <cell r="E30">
-            <v>46311.387928240743</v>
+            <v>46343.387777777767</v>
           </cell>
           <cell r="F30" t="str">
             <v>Capacity Utilization, Industrial (%)</v>
@@ -4488,7 +3370,7 @@
         </row>
         <row r="74">
           <cell r="E74">
-            <v>46311.678611111114</v>
+            <v>46316.678391203706</v>
           </cell>
           <cell r="F74" t="str">
             <v>3-Month Treasury Bills, Secondary market (%)</v>
@@ -4496,7 +3378,7 @@
         </row>
         <row r="75">
           <cell r="E75">
-            <v>46311.678460648138</v>
+            <v>46316.678148148145</v>
           </cell>
           <cell r="F75" t="str">
             <v>Bank Prime Rate (%)</v>
@@ -4504,7 +3386,7 @@
         </row>
         <row r="76">
           <cell r="E76">
-            <v>46311.678576388891</v>
+            <v>46316.678495370375</v>
           </cell>
           <cell r="F76" t="str">
             <v>2-yr. Treasury Bond Yield at Constant Maturity (%)</v>
@@ -4512,7 +3394,7 @@
         </row>
         <row r="77">
           <cell r="E77">
-            <v>46311.678483796306</v>
+            <v>46316.678310185176</v>
           </cell>
           <cell r="F77" t="str">
             <v>10-yr. Treasury Bond Yield at Constant Maturity (%)</v>
@@ -4520,7 +3402,7 @@
         </row>
         <row r="78">
           <cell r="E78">
-            <v>46311.710868055554</v>
+            <v>46316.710868055554</v>
           </cell>
           <cell r="F78" t="str">
             <v>10 Yr - 2 Yr Treasury Spread - Const Maturity %</v>
@@ -4528,7 +3410,7 @@
         </row>
         <row r="79">
           <cell r="E79">
-            <v>46311.678437499999</v>
+            <v>46316.678263888898</v>
           </cell>
           <cell r="F79" t="str">
             <v>10-yr. Treasury Bond Yield at Const. Mat. Inflation Indexed (%)</v>
@@ -4536,7 +3418,7 @@
         </row>
         <row r="80">
           <cell r="E80">
-            <v>46311.678587962961</v>
+            <v>46316.678472222222</v>
           </cell>
           <cell r="F80" t="str">
             <v>30-yr. Treasury Bond Yield at Constant Maturity (%)</v>
@@ -4544,7 +3426,7 @@
         </row>
         <row r="81">
           <cell r="E81">
-            <v>46311.710844907415</v>
+            <v>46316.710891203693</v>
           </cell>
           <cell r="F81" t="str">
             <v>10 Yr - 3 Month Treasury Spread - Const Maturity %</v>
@@ -4552,7 +3434,7 @@
         </row>
         <row r="82">
           <cell r="E82">
-            <v>46314.678506944445</v>
+            <v>46321.678344907414</v>
           </cell>
           <cell r="F82" t="str">
             <v>USD/EUR Exchange Rate - Last Day of Month</v>
@@ -4560,7 +3442,7 @@
         </row>
         <row r="83">
           <cell r="E83">
-            <v>46314.67859953703</v>
+            <v>46321.678553240738</v>
           </cell>
           <cell r="F83" t="str">
             <v>Nominal Broad USD Index - Last Day of Month</v>
@@ -49804,10 +48686,10 @@
             <v>46314</v>
           </cell>
           <cell r="C330" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D330">
-            <v>46314</v>
+            <v>0</v>
           </cell>
           <cell r="E330">
             <v>330</v>
@@ -54615,10 +53497,10 @@
             <v>46311</v>
           </cell>
           <cell r="C613" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D613">
-            <v>46311</v>
+            <v>0</v>
           </cell>
           <cell r="E613">
             <v>613</v>
@@ -54632,10 +53514,10 @@
             <v>46314</v>
           </cell>
           <cell r="C614" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D614">
-            <v>46314</v>
+            <v>0</v>
           </cell>
           <cell r="E614">
             <v>614</v>
@@ -54649,10 +53531,10 @@
             <v>46315</v>
           </cell>
           <cell r="C615" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D615">
-            <v>46315</v>
+            <v>0</v>
           </cell>
           <cell r="E615">
             <v>615</v>
@@ -60140,10 +59022,10 @@
             <v>46311</v>
           </cell>
           <cell r="C938" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D938">
-            <v>46311</v>
+            <v>0</v>
           </cell>
           <cell r="E938">
             <v>938</v>
@@ -60157,10 +59039,10 @@
             <v>46314</v>
           </cell>
           <cell r="C939" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D939">
-            <v>46314</v>
+            <v>0</v>
           </cell>
           <cell r="E939">
             <v>939</v>
@@ -60174,10 +59056,10 @@
             <v>46315</v>
           </cell>
           <cell r="C940" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D940">
-            <v>46315</v>
+            <v>0</v>
           </cell>
           <cell r="E940">
             <v>940</v>
@@ -61857,10 +60739,10 @@
             <v>46311</v>
           </cell>
           <cell r="C1039" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1039">
-            <v>46311</v>
+            <v>0</v>
           </cell>
           <cell r="E1039">
             <v>1039</v>
@@ -69728,10 +68610,10 @@
             <v>46311</v>
           </cell>
           <cell r="C1502" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1502">
-            <v>46311</v>
+            <v>0</v>
           </cell>
           <cell r="E1502">
             <v>1502</v>
@@ -69745,10 +68627,10 @@
             <v>46314</v>
           </cell>
           <cell r="C1503" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1503">
-            <v>46314</v>
+            <v>0</v>
           </cell>
           <cell r="E1503">
             <v>1503</v>
@@ -69762,10 +68644,10 @@
             <v>46315</v>
           </cell>
           <cell r="C1504" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1504">
-            <v>46315</v>
+            <v>0</v>
           </cell>
           <cell r="E1504">
             <v>1504</v>
@@ -75321,10 +74203,10 @@
             <v>46311</v>
           </cell>
           <cell r="C1831" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1831">
-            <v>46311</v>
+            <v>0</v>
           </cell>
           <cell r="E1831">
             <v>1831</v>
@@ -75338,10 +74220,10 @@
             <v>46314</v>
           </cell>
           <cell r="C1832" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1832">
-            <v>46314</v>
+            <v>0</v>
           </cell>
           <cell r="E1832">
             <v>1832</v>
@@ -75355,10 +74237,10 @@
             <v>46315</v>
           </cell>
           <cell r="C1833" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1833">
-            <v>46315</v>
+            <v>0</v>
           </cell>
           <cell r="E1833">
             <v>1833</v>
@@ -76579,8 +75461,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="0" row="0">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{23E45F88-1DAE-413F-B9A3-ABD066DC41AF}">
+  <we:reference id="wa200003692" version="1.0.0.1" store="en-US" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="wa200003692" version="1.0.0.1" store="" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties/>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C76B3D8D-162D-4B8C-A27F-1037F2E9F651}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DFA9851-77AC-49AA-A71B-D92A92205070}">
   <sheetPr codeName="Sheet22">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -76607,13 +75509,13 @@
     <col min="34" max="34" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" s="84" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="86"/>
-      <c r="B1" s="86"/>
-      <c r="C1" s="86"/>
+    <row r="1" spans="1:34" s="72" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="74"/>
+      <c r="B1" s="74"/>
+      <c r="C1" s="74"/>
       <c r="D1" s="37"/>
       <c r="E1" s="37"/>
-      <c r="F1" s="86" t="s">
+      <c r="F1" s="74" t="s">
         <v>190</v>
       </c>
       <c r="G1" s="34">
@@ -76689,7 +75591,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:34" s="84" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:34" s="72" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="25"/>
       <c r="B2" s="25"/>
       <c r="C2" s="25" t="s">
@@ -76704,79 +75606,79 @@
       <c r="F2" s="25" t="s">
         <v>186</v>
       </c>
-      <c r="G2" s="85">
+      <c r="G2" s="73">
         <v>45597</v>
       </c>
-      <c r="H2" s="85">
+      <c r="H2" s="73">
         <v>45627</v>
       </c>
-      <c r="I2" s="85">
+      <c r="I2" s="73">
         <v>45658</v>
       </c>
-      <c r="J2" s="85">
+      <c r="J2" s="73">
         <v>45689</v>
       </c>
-      <c r="K2" s="85">
+      <c r="K2" s="73">
         <v>45717</v>
       </c>
-      <c r="L2" s="85">
+      <c r="L2" s="73">
         <v>45748</v>
       </c>
-      <c r="M2" s="85">
+      <c r="M2" s="73">
         <v>45778</v>
       </c>
-      <c r="N2" s="85">
+      <c r="N2" s="73">
         <v>45809</v>
       </c>
-      <c r="O2" s="85">
+      <c r="O2" s="73">
         <v>45839</v>
       </c>
-      <c r="P2" s="85">
+      <c r="P2" s="73">
         <v>45870</v>
       </c>
-      <c r="Q2" s="85">
+      <c r="Q2" s="73">
         <v>45901</v>
       </c>
-      <c r="R2" s="85">
+      <c r="R2" s="73">
         <v>45931</v>
       </c>
-      <c r="S2" s="85">
+      <c r="S2" s="73">
         <v>45962</v>
       </c>
-      <c r="T2" s="85">
+      <c r="T2" s="73">
         <v>45992</v>
       </c>
-      <c r="U2" s="85">
+      <c r="U2" s="73">
         <v>46023</v>
       </c>
-      <c r="V2" s="85">
+      <c r="V2" s="73">
         <v>46054</v>
       </c>
-      <c r="W2" s="85">
+      <c r="W2" s="73">
         <v>46082</v>
       </c>
-      <c r="X2" s="85">
+      <c r="X2" s="73">
         <v>46113</v>
       </c>
-      <c r="Y2" s="85">
+      <c r="Y2" s="73">
         <v>46143</v>
       </c>
-      <c r="Z2" s="85">
+      <c r="Z2" s="73">
         <v>46174</v>
       </c>
-      <c r="AA2" s="85">
+      <c r="AA2" s="73">
         <v>46204</v>
       </c>
-      <c r="AB2" s="85">
+      <c r="AB2" s="73">
         <v>46235</v>
       </c>
-      <c r="AC2" s="85">
+      <c r="AC2" s="73">
         <v>46266</v>
       </c>
-      <c r="AD2" s="85">
+      <c r="AD2" s="73">
         <v>46296</v>
       </c>
-      <c r="AH2" s="84" t="s">
+      <c r="AH2" s="72" t="s">
         <v>185</v>
       </c>
     </row>
@@ -76786,11 +75688,11 @@
         <v>184</v>
       </c>
       <c r="C3" s="10"/>
-      <c r="D3" s="83">
-        <v>46310.876238425924</v>
-      </c>
-      <c r="E3" s="82">
-        <v>46311.387928240743</v>
+      <c r="D3" s="71">
+        <v>46314.678553240738</v>
+      </c>
+      <c r="E3" s="70">
+        <v>46315.35601851852</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>183</v>
@@ -76914,7 +75816,7 @@
       <c r="AD4" s="7" t="e">
         <v>#N/A</v>
       </c>
-      <c r="AE4" s="81" t="s">
+      <c r="AE4" s="69" t="s">
         <v>35</v>
       </c>
       <c r="AH4" t="s">
@@ -77557,13 +76459,13 @@
       <c r="Y11" s="13">
         <v>1252</v>
       </c>
-      <c r="Z11" s="78">
+      <c r="Z11" s="67">
         <v>1256</v>
       </c>
-      <c r="AA11" s="78">
+      <c r="AA11" s="67">
         <v>1267</v>
       </c>
-      <c r="AB11" s="78">
+      <c r="AB11" s="67">
         <v>1271</v>
       </c>
       <c r="AC11" s="13" t="e">
@@ -77576,7 +76478,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:34" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A12" s="6">
         <v>133</v>
       </c>
@@ -77658,20 +76560,20 @@
       <c r="AA12" s="4">
         <v>4.2940300000000002</v>
       </c>
-      <c r="AB12" s="66">
+      <c r="AB12" s="59">
         <v>-2.0935100000000002</v>
       </c>
       <c r="AC12" s="4" t="e">
         <v>#N/A</v>
       </c>
-      <c r="AD12" s="7" t="e">
+      <c r="AD12" s="4" t="e">
         <v>#N/A</v>
       </c>
       <c r="AH12" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A13" s="25">
         <v>13</v>
       </c>
@@ -77759,14 +76661,14 @@
       <c r="AC13" s="40">
         <v>6.86</v>
       </c>
-      <c r="AD13" s="80">
+      <c r="AD13" s="40">
         <v>7.36</v>
       </c>
       <c r="AH13" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:34" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A14" s="25"/>
       <c r="B14" s="25"/>
       <c r="C14" s="25"/>
@@ -77788,10 +76690,10 @@
       <c r="S14" s="36"/>
       <c r="T14" s="36"/>
       <c r="U14" s="36"/>
-      <c r="V14" s="79"/>
-      <c r="W14" s="79"/>
-      <c r="X14" s="79"/>
-      <c r="Y14" s="79"/>
+      <c r="V14" s="68"/>
+      <c r="W14" s="68"/>
+      <c r="X14" s="68"/>
+      <c r="Y14" s="68"/>
       <c r="Z14" s="36"/>
       <c r="AA14" s="36"/>
       <c r="AB14" s="36"/>
@@ -78108,10 +77010,10 @@
       <c r="Z18" s="4">
         <v>1.867</v>
       </c>
-      <c r="AA18" s="66">
+      <c r="AA18" s="59">
         <v>1.837</v>
       </c>
-      <c r="AB18" s="66">
+      <c r="AB18" s="59">
         <v>1.8080000000000001</v>
       </c>
       <c r="AC18" s="4" t="e">
@@ -78375,13 +77277,13 @@
       <c r="AA22" s="13">
         <v>-10</v>
       </c>
-      <c r="AB22" s="78">
+      <c r="AB22" s="67">
         <v>133</v>
       </c>
-      <c r="AC22" s="78">
+      <c r="AC22" s="67">
         <v>29</v>
       </c>
-      <c r="AD22" s="77" t="e">
+      <c r="AD22" s="66" t="e">
         <v>#N/A</v>
       </c>
       <c r="AH22" t="s">
@@ -78476,7 +77378,7 @@
       <c r="AC23" s="12">
         <v>78</v>
       </c>
-      <c r="AD23" s="77" t="e">
+      <c r="AD23" s="66" t="e">
         <v>#N/A</v>
       </c>
       <c r="AH23" t="s">
@@ -78565,10 +77467,10 @@
       <c r="AA24" s="4">
         <v>4.0999999999999996</v>
       </c>
-      <c r="AB24" s="66">
+      <c r="AB24" s="59">
         <v>4.0999999999999996</v>
       </c>
-      <c r="AC24" s="66">
+      <c r="AC24" s="59">
         <v>4.2</v>
       </c>
       <c r="AD24" s="4" t="e">
@@ -78803,7 +77705,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:34" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
@@ -78829,18 +77731,18 @@
       <c r="U28" s="9"/>
       <c r="V28" s="9"/>
       <c r="W28" s="9"/>
-      <c r="X28" s="9"/>
-      <c r="Y28" s="9"/>
-      <c r="Z28" s="9"/>
-      <c r="AA28" s="9"/>
-      <c r="AB28" s="9"/>
-      <c r="AC28" s="9"/>
+      <c r="X28" s="36"/>
+      <c r="Y28" s="36"/>
+      <c r="Z28" s="36"/>
+      <c r="AA28" s="36"/>
+      <c r="AB28" s="36"/>
+      <c r="AC28" s="36"/>
       <c r="AD28" s="9"/>
       <c r="AH28" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="29" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A29" s="1">
         <v>101</v>
       </c>
@@ -78851,10 +77753,10 @@
         <v>37</v>
       </c>
       <c r="D29" s="24">
-        <v>46283.388981481483</v>
+        <v>46311.389108796298</v>
       </c>
       <c r="E29" s="49">
-        <v>46311.38898148149</v>
+        <v>46343.389108796298</v>
       </c>
       <c r="F29" s="48" t="s">
         <v>138</v>
@@ -78910,23 +77812,23 @@
       <c r="W29" s="7">
         <v>-0.16849</v>
       </c>
-      <c r="X29" s="28">
-        <v>0.83030999999999999</v>
-      </c>
-      <c r="Y29" s="28">
-        <v>5.9760000000000001E-2</v>
-      </c>
-      <c r="Z29" s="28">
-        <v>0.19719</v>
-      </c>
-      <c r="AA29" s="28">
-        <v>0.19778000000000001</v>
-      </c>
-      <c r="AB29" s="28">
-        <v>2.213E-2</v>
-      </c>
-      <c r="AC29" s="7" t="e">
-        <v>#N/A</v>
+      <c r="X29" s="65">
+        <v>0.82882999999999996</v>
+      </c>
+      <c r="Y29" s="64">
+        <v>0.14272000000000001</v>
+      </c>
+      <c r="Z29" s="64">
+        <v>0.23150000000000001</v>
+      </c>
+      <c r="AA29" s="64">
+        <v>0.23271</v>
+      </c>
+      <c r="AB29" s="64">
+        <v>6.3759999999999997E-2</v>
+      </c>
+      <c r="AC29" s="64">
+        <v>0.66256000000000004</v>
       </c>
       <c r="AD29" s="7" t="e">
         <v>#N/A</v>
@@ -78935,7 +77837,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A30" s="1">
         <v>111</v>
       </c>
@@ -78946,10 +77848,10 @@
         <v>37</v>
       </c>
       <c r="D30" s="24">
-        <v>46283.387928240743</v>
+        <v>46311.387777777774</v>
       </c>
       <c r="E30" s="49">
-        <v>46311.387928240743</v>
+        <v>46343.387777777767</v>
       </c>
       <c r="F30" s="48" t="s">
         <v>136</v>
@@ -79005,23 +77907,23 @@
       <c r="W30" s="7">
         <v>75.617800000000003</v>
       </c>
-      <c r="X30" s="7">
-        <v>76.180300000000003</v>
-      </c>
-      <c r="Y30" s="7">
-        <v>76.160499999999999</v>
-      </c>
-      <c r="Z30" s="7">
-        <v>76.243799999999993</v>
-      </c>
-      <c r="AA30" s="7">
-        <v>76.325900000000004</v>
-      </c>
-      <c r="AB30" s="54">
-        <v>76.271699999999996</v>
-      </c>
-      <c r="AC30" s="7" t="e">
-        <v>#N/A</v>
+      <c r="X30" s="63">
+        <v>76.179199999999994</v>
+      </c>
+      <c r="Y30" s="62">
+        <v>76.222499999999997</v>
+      </c>
+      <c r="Z30" s="62">
+        <v>76.332099999999997</v>
+      </c>
+      <c r="AA30" s="62">
+        <v>76.440899999999999</v>
+      </c>
+      <c r="AB30" s="62">
+        <v>76.418400000000005</v>
+      </c>
+      <c r="AC30" s="61">
+        <v>76.850399999999993</v>
       </c>
       <c r="AD30" s="7" t="e">
         <v>#N/A</v>
@@ -79036,7 +77938,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:34" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A31" s="6">
         <v>109</v>
       </c>
@@ -79356,7 +78258,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="35" spans="1:34" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A35" s="10"/>
       <c r="B35" s="10"/>
       <c r="C35" s="10"/>
@@ -79366,34 +78268,34 @@
         <v>128</v>
       </c>
       <c r="G35" s="9"/>
-      <c r="H35" s="36"/>
-      <c r="I35" s="36"/>
-      <c r="J35" s="36"/>
-      <c r="K35" s="36"/>
-      <c r="L35" s="36"/>
-      <c r="M35" s="36"/>
-      <c r="N35" s="36"/>
-      <c r="O35" s="36"/>
-      <c r="P35" s="36"/>
-      <c r="Q35" s="36"/>
-      <c r="R35" s="36"/>
-      <c r="S35" s="36"/>
-      <c r="T35" s="36"/>
-      <c r="U35" s="36"/>
-      <c r="V35" s="36"/>
-      <c r="W35" s="36"/>
-      <c r="X35" s="36"/>
-      <c r="Y35" s="36"/>
-      <c r="Z35" s="36"/>
-      <c r="AA35" s="36"/>
-      <c r="AB35" s="36"/>
+      <c r="H35" s="9"/>
+      <c r="I35" s="9"/>
+      <c r="J35" s="9"/>
+      <c r="K35" s="9"/>
+      <c r="L35" s="9"/>
+      <c r="M35" s="9"/>
+      <c r="N35" s="9"/>
+      <c r="O35" s="9"/>
+      <c r="P35" s="9"/>
+      <c r="Q35" s="9"/>
+      <c r="R35" s="9"/>
+      <c r="S35" s="9"/>
+      <c r="T35" s="9"/>
+      <c r="U35" s="9"/>
+      <c r="V35" s="9"/>
+      <c r="W35" s="9"/>
+      <c r="X35" s="9"/>
+      <c r="Y35" s="9"/>
+      <c r="Z35" s="9"/>
+      <c r="AA35" s="9"/>
+      <c r="AB35" s="9"/>
       <c r="AC35" s="9"/>
       <c r="AD35" s="9"/>
       <c r="AH35" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="36" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>55</v>
       </c>
@@ -79415,67 +78317,67 @@
       <c r="G36" s="7">
         <v>0.29459000000000002</v>
       </c>
-      <c r="H36" s="76">
+      <c r="H36" s="7">
         <v>-0.31867000000000001</v>
       </c>
-      <c r="I36" s="75">
+      <c r="I36" s="7">
         <v>0.37806000000000001</v>
       </c>
-      <c r="J36" s="75">
+      <c r="J36" s="7">
         <v>0.12834000000000001</v>
       </c>
-      <c r="K36" s="75">
+      <c r="K36" s="7">
         <v>7.0419999999999996E-2</v>
       </c>
-      <c r="L36" s="75">
+      <c r="L36" s="7">
         <v>-8.6269999999999999E-2</v>
       </c>
-      <c r="M36" s="75">
+      <c r="M36" s="7">
         <v>-3.2259999999999997E-2</v>
       </c>
-      <c r="N36" s="75">
+      <c r="N36" s="7">
         <v>0.20338000000000001</v>
       </c>
-      <c r="O36" s="75">
+      <c r="O36" s="7">
         <v>0.10838</v>
       </c>
-      <c r="P36" s="75">
+      <c r="P36" s="7">
         <v>-0.10174</v>
       </c>
-      <c r="Q36" s="75">
+      <c r="Q36" s="7">
         <v>0.29274</v>
       </c>
-      <c r="R36" s="75">
+      <c r="R36" s="7">
         <v>0.26362000000000002</v>
       </c>
-      <c r="S36" s="75">
+      <c r="S36" s="7">
         <v>0.23005</v>
       </c>
-      <c r="T36" s="75">
+      <c r="T36" s="7">
         <v>-6.0589999999999998E-2</v>
       </c>
-      <c r="U36" s="74">
+      <c r="U36" s="54">
         <v>1.643E-2</v>
       </c>
-      <c r="V36" s="74">
+      <c r="V36" s="54">
         <v>0.42576999999999998</v>
       </c>
-      <c r="W36" s="74">
+      <c r="W36" s="54">
         <v>0.97848999999999997</v>
       </c>
-      <c r="X36" s="74">
+      <c r="X36" s="54">
         <v>0.55288999999999999</v>
       </c>
-      <c r="Y36" s="74">
+      <c r="Y36" s="54">
         <v>0.38057000000000002</v>
       </c>
-      <c r="Z36" s="74">
+      <c r="Z36" s="54">
         <v>0.11377</v>
       </c>
-      <c r="AA36" s="74">
+      <c r="AA36" s="54">
         <v>0.88497000000000003</v>
       </c>
-      <c r="AB36" s="74">
+      <c r="AB36" s="54">
         <v>0.41588000000000003</v>
       </c>
       <c r="AC36" s="7" t="e">
@@ -79488,7 +78390,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="37" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>59</v>
       </c>
@@ -79510,67 +78412,67 @@
       <c r="G37" s="42">
         <v>1.43</v>
       </c>
-      <c r="H37" s="73">
+      <c r="H37" s="42">
         <v>1.42</v>
       </c>
-      <c r="I37" s="71">
+      <c r="I37" s="42">
         <v>1.43</v>
       </c>
-      <c r="J37" s="72">
+      <c r="J37" s="42">
         <v>1.42</v>
       </c>
-      <c r="K37" s="71">
+      <c r="K37" s="42">
         <v>1.41</v>
       </c>
-      <c r="L37" s="71">
+      <c r="L37" s="42">
         <v>1.41</v>
       </c>
-      <c r="M37" s="71">
+      <c r="M37" s="42">
         <v>1.42</v>
       </c>
-      <c r="N37" s="72">
+      <c r="N37" s="42">
         <v>1.42</v>
       </c>
-      <c r="O37" s="72">
+      <c r="O37" s="42">
         <v>1.4</v>
       </c>
-      <c r="P37" s="71">
+      <c r="P37" s="42">
         <v>1.4</v>
       </c>
-      <c r="Q37" s="71">
+      <c r="Q37" s="42">
         <v>1.4</v>
       </c>
-      <c r="R37" s="71">
+      <c r="R37" s="42">
         <v>1.41</v>
       </c>
-      <c r="S37" s="71">
+      <c r="S37" s="42">
         <v>1.4</v>
       </c>
-      <c r="T37" s="71">
+      <c r="T37" s="42">
         <v>1.39</v>
       </c>
-      <c r="U37" s="72">
+      <c r="U37" s="42">
         <v>1.38</v>
       </c>
-      <c r="V37" s="71">
+      <c r="V37" s="42">
         <v>1.37</v>
       </c>
-      <c r="W37" s="71">
+      <c r="W37" s="42">
         <v>1.35</v>
       </c>
-      <c r="X37" s="72">
+      <c r="X37" s="42">
         <v>1.34</v>
       </c>
-      <c r="Y37" s="71">
+      <c r="Y37" s="42">
         <v>1.31</v>
       </c>
-      <c r="Z37" s="72">
+      <c r="Z37" s="42">
         <v>1.33</v>
       </c>
-      <c r="AA37" s="71">
+      <c r="AA37" s="42">
         <v>1.34</v>
       </c>
-      <c r="AB37" s="70">
+      <c r="AB37" s="41">
         <v>1.33</v>
       </c>
       <c r="AC37" s="42" t="e">
@@ -79583,7 +78485,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="38" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A38" s="6">
         <v>139</v>
       </c>
@@ -79608,19 +78510,19 @@
       <c r="H38" s="4">
         <v>-0.5</v>
       </c>
-      <c r="I38" s="57">
+      <c r="I38" s="4">
         <v>0.1</v>
       </c>
       <c r="J38" s="4">
         <v>-0.1</v>
       </c>
-      <c r="K38" s="57">
+      <c r="K38" s="4">
         <v>-0.3</v>
       </c>
-      <c r="L38" s="56">
+      <c r="L38" s="4">
         <v>-0.4</v>
       </c>
-      <c r="M38" s="56">
+      <c r="M38" s="4">
         <v>0.1</v>
       </c>
       <c r="N38" s="4">
@@ -79629,43 +78531,43 @@
       <c r="O38" s="4">
         <v>0.1</v>
       </c>
-      <c r="P38" s="57">
+      <c r="P38" s="4">
         <v>-0.2</v>
       </c>
-      <c r="Q38" s="56">
+      <c r="Q38" s="4">
         <v>0.4</v>
       </c>
-      <c r="R38" s="56">
+      <c r="R38" s="4">
         <v>0.6</v>
       </c>
-      <c r="S38" s="56">
+      <c r="S38" s="4">
         <v>0.3</v>
       </c>
-      <c r="T38" s="56">
+      <c r="T38" s="4">
         <v>-0.1</v>
       </c>
       <c r="U38" s="4">
         <v>0.3</v>
       </c>
-      <c r="V38" s="57">
+      <c r="V38" s="4">
         <v>0.3</v>
       </c>
-      <c r="W38" s="56">
+      <c r="W38" s="4">
         <v>0.7</v>
       </c>
       <c r="X38" s="4">
         <v>0.7</v>
       </c>
-      <c r="Y38" s="57">
+      <c r="Y38" s="4">
         <v>0.7</v>
       </c>
       <c r="Z38" s="4">
         <v>-0.2</v>
       </c>
-      <c r="AA38" s="69">
+      <c r="AA38" s="59">
         <v>0.9</v>
       </c>
-      <c r="AB38" s="68">
+      <c r="AB38" s="59">
         <v>0.2</v>
       </c>
       <c r="AC38" s="4" t="e">
@@ -79678,7 +78580,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="39" spans="1:34" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A39" s="25">
         <v>57</v>
       </c>
@@ -79780,30 +78682,30 @@
       <c r="D40" s="37"/>
       <c r="E40" s="14"/>
       <c r="F40" s="25"/>
-      <c r="G40" s="67"/>
-      <c r="H40" s="67"/>
-      <c r="I40" s="67"/>
-      <c r="J40" s="67"/>
-      <c r="K40" s="67"/>
-      <c r="L40" s="67"/>
-      <c r="M40" s="67"/>
-      <c r="N40" s="67"/>
-      <c r="O40" s="67"/>
-      <c r="P40" s="67"/>
-      <c r="Q40" s="67"/>
-      <c r="R40" s="67"/>
-      <c r="S40" s="67"/>
-      <c r="T40" s="67"/>
-      <c r="U40" s="67"/>
-      <c r="V40" s="67"/>
-      <c r="W40" s="67"/>
-      <c r="X40" s="67"/>
-      <c r="Y40" s="67"/>
-      <c r="Z40" s="67"/>
-      <c r="AA40" s="67"/>
-      <c r="AB40" s="67"/>
-      <c r="AC40" s="67"/>
-      <c r="AD40" s="67"/>
+      <c r="G40" s="60"/>
+      <c r="H40" s="60"/>
+      <c r="I40" s="60"/>
+      <c r="J40" s="60"/>
+      <c r="K40" s="60"/>
+      <c r="L40" s="60"/>
+      <c r="M40" s="60"/>
+      <c r="N40" s="60"/>
+      <c r="O40" s="60"/>
+      <c r="P40" s="60"/>
+      <c r="Q40" s="60"/>
+      <c r="R40" s="60"/>
+      <c r="S40" s="60"/>
+      <c r="T40" s="60"/>
+      <c r="U40" s="60"/>
+      <c r="V40" s="60"/>
+      <c r="W40" s="60"/>
+      <c r="X40" s="60"/>
+      <c r="Y40" s="60"/>
+      <c r="Z40" s="60"/>
+      <c r="AA40" s="60"/>
+      <c r="AB40" s="60"/>
+      <c r="AC40" s="60"/>
+      <c r="AD40" s="60"/>
       <c r="AH40" t="s">
         <v>34</v>
       </c>
@@ -80099,28 +79001,28 @@
       <c r="U44" s="4">
         <v>-0.29616999999999999</v>
       </c>
-      <c r="V44" s="66">
+      <c r="V44" s="59">
         <v>0.39950999999999998</v>
       </c>
-      <c r="W44" s="66">
+      <c r="W44" s="59">
         <v>12.589549999999999</v>
       </c>
-      <c r="X44" s="66">
+      <c r="X44" s="59">
         <v>17.536049999999999</v>
       </c>
-      <c r="Y44" s="66">
+      <c r="Y44" s="59">
         <v>22.97287</v>
       </c>
-      <c r="Z44" s="66">
+      <c r="Z44" s="59">
         <v>15.451370000000001</v>
       </c>
-      <c r="AA44" s="66">
+      <c r="AA44" s="59">
         <v>14.44533</v>
       </c>
-      <c r="AB44" s="66">
+      <c r="AB44" s="59">
         <v>16.04935</v>
       </c>
-      <c r="AC44" s="66">
+      <c r="AC44" s="59">
         <v>20.354109999999999</v>
       </c>
       <c r="AD44" s="4" t="e">
@@ -80260,7 +79162,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="47" spans="1:34" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A47" s="10"/>
       <c r="B47" s="10"/>
       <c r="C47" s="10"/>
@@ -80287,17 +79189,17 @@
       <c r="V47" s="9"/>
       <c r="W47" s="9"/>
       <c r="X47" s="9"/>
-      <c r="Y47" s="36"/>
-      <c r="Z47" s="36"/>
-      <c r="AA47" s="36"/>
-      <c r="AB47" s="36"/>
-      <c r="AC47" s="36"/>
+      <c r="Y47" s="9"/>
+      <c r="Z47" s="9"/>
+      <c r="AA47" s="9"/>
+      <c r="AB47" s="9"/>
+      <c r="AC47" s="9"/>
       <c r="AD47" s="9"/>
       <c r="AH47" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="48" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>123</v>
       </c>
@@ -80370,19 +79272,19 @@
       <c r="X48" s="8">
         <v>6.4635600000000002</v>
       </c>
-      <c r="Y48" s="63">
+      <c r="Y48" s="8">
         <v>8.7441399999999998</v>
       </c>
-      <c r="Z48" s="62">
+      <c r="Z48" s="8">
         <v>6.5667900000000001</v>
       </c>
-      <c r="AA48" s="62">
+      <c r="AA48" s="8">
         <v>5.8784000000000001</v>
       </c>
-      <c r="AB48" s="62">
+      <c r="AB48" s="8">
         <v>6.5574199999999996</v>
       </c>
-      <c r="AC48" s="62">
+      <c r="AC48" s="8">
         <v>8.4082600000000003</v>
       </c>
       <c r="AD48" s="7" t="e">
@@ -80392,7 +79294,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="49" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>119</v>
       </c>
@@ -80465,19 +79367,19 @@
       <c r="X49" s="8">
         <v>9.4268000000000001</v>
       </c>
-      <c r="Y49" s="65">
+      <c r="Y49" s="8">
         <v>12.258459999999999</v>
       </c>
-      <c r="Z49" s="64">
+      <c r="Z49" s="8">
         <v>11.152200000000001</v>
       </c>
-      <c r="AA49" s="64">
+      <c r="AA49" s="8">
         <v>10.01108</v>
       </c>
-      <c r="AB49" s="64">
+      <c r="AB49" s="8">
         <v>11.58319</v>
       </c>
-      <c r="AC49" s="64">
+      <c r="AC49" s="8">
         <v>14.15049</v>
       </c>
       <c r="AD49" s="7" t="e">
@@ -80487,7 +79389,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="50" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A50" s="6">
         <v>121</v>
       </c>
@@ -80560,19 +79462,19 @@
       <c r="X50" s="5">
         <v>15.40253</v>
       </c>
-      <c r="Y50" s="63">
+      <c r="Y50" s="5">
         <v>20.731300000000001</v>
       </c>
-      <c r="Z50" s="62">
+      <c r="Z50" s="5">
         <v>10.42502</v>
       </c>
-      <c r="AA50" s="62">
+      <c r="AA50" s="5">
         <v>8.7532700000000006</v>
       </c>
-      <c r="AB50" s="62">
+      <c r="AB50" s="5">
         <v>11.737130000000001</v>
       </c>
-      <c r="AC50" s="62">
+      <c r="AC50" s="5">
         <v>21.706589999999998</v>
       </c>
       <c r="AD50" s="4" t="e">
@@ -80582,7 +79484,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="51" spans="1:34" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A51" s="48">
         <v>115</v>
       </c>
@@ -80854,10 +79756,10 @@
       <c r="AA53" s="46">
         <v>83.76</v>
       </c>
-      <c r="AB53" s="61">
+      <c r="AB53" s="58">
         <v>91.08</v>
       </c>
-      <c r="AC53" s="61">
+      <c r="AC53" s="58">
         <v>114.16</v>
       </c>
       <c r="AD53" s="44" t="s">
@@ -80868,10 +79770,10 @@
       </c>
     </row>
     <row r="54" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A54" s="60">
+      <c r="A54" s="57">
         <v>117</v>
       </c>
-      <c r="B54" s="60" t="s">
+      <c r="B54" s="57" t="s">
         <v>94</v>
       </c>
       <c r="C54" s="16" t="s">
@@ -80883,7 +79785,7 @@
       <c r="E54" s="23">
         <v>46316.676724537043</v>
       </c>
-      <c r="F54" s="60" t="s">
+      <c r="F54" s="57" t="s">
         <v>92</v>
       </c>
       <c r="G54" s="42">
@@ -81006,76 +79908,76 @@
       <c r="F56" s="25" t="s">
         <v>91</v>
       </c>
-      <c r="G56" s="59">
+      <c r="G56" s="56">
         <v>2024</v>
       </c>
-      <c r="H56" s="59" t="s">
+      <c r="H56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="I56" s="59">
+      <c r="I56" s="56">
         <v>2025</v>
       </c>
-      <c r="J56" s="59" t="s">
+      <c r="J56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="K56" s="59" t="s">
+      <c r="K56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="L56" s="59" t="s">
+      <c r="L56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="M56" s="59" t="s">
+      <c r="M56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="N56" s="59" t="s">
+      <c r="N56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="O56" s="59" t="s">
+      <c r="O56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="P56" s="59" t="s">
+      <c r="P56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="Q56" s="59">
+      <c r="Q56" s="56">
         <v>2025</v>
       </c>
-      <c r="R56" s="59" t="s">
+      <c r="R56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="S56" s="59" t="s">
+      <c r="S56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="T56" s="59" t="s">
+      <c r="T56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="U56" s="59">
+      <c r="U56" s="56">
         <v>2026</v>
       </c>
-      <c r="V56" s="59" t="s">
+      <c r="V56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="W56" s="59" t="s">
+      <c r="W56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="X56" s="59" t="s">
+      <c r="X56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="Y56" s="59" t="s">
+      <c r="Y56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="Z56" s="59" t="s">
+      <c r="Z56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="AA56" s="59" t="s">
+      <c r="AA56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="AB56" s="59" t="s">
+      <c r="AB56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="AC56" s="59" t="s">
+      <c r="AC56" s="56" t="s">
         <v>35</v>
       </c>
-      <c r="AD56" s="59">
+      <c r="AD56" s="56">
         <v>2026</v>
       </c>
       <c r="AH56" t="s">
@@ -81091,76 +79993,76 @@
       <c r="F57" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="G57" s="58">
+      <c r="G57" s="55">
         <v>45597</v>
       </c>
-      <c r="H57" s="58">
+      <c r="H57" s="55">
         <v>45627</v>
       </c>
-      <c r="I57" s="58">
+      <c r="I57" s="55">
         <v>45658</v>
       </c>
-      <c r="J57" s="58">
+      <c r="J57" s="55">
         <v>45689</v>
       </c>
-      <c r="K57" s="58">
+      <c r="K57" s="55">
         <v>45717</v>
       </c>
-      <c r="L57" s="58">
+      <c r="L57" s="55">
         <v>45748</v>
       </c>
-      <c r="M57" s="58">
+      <c r="M57" s="55">
         <v>45778</v>
       </c>
-      <c r="N57" s="58">
+      <c r="N57" s="55">
         <v>45809</v>
       </c>
-      <c r="O57" s="58">
+      <c r="O57" s="55">
         <v>45839</v>
       </c>
-      <c r="P57" s="58">
+      <c r="P57" s="55">
         <v>45870</v>
       </c>
-      <c r="Q57" s="58">
+      <c r="Q57" s="55">
         <v>45901</v>
       </c>
-      <c r="R57" s="58">
+      <c r="R57" s="55">
         <v>45931</v>
       </c>
-      <c r="S57" s="58">
+      <c r="S57" s="55">
         <v>45962</v>
       </c>
-      <c r="T57" s="58">
+      <c r="T57" s="55">
         <v>45992</v>
       </c>
-      <c r="U57" s="58">
+      <c r="U57" s="55">
         <v>46023</v>
       </c>
-      <c r="V57" s="58">
+      <c r="V57" s="55">
         <v>46054</v>
       </c>
-      <c r="W57" s="58">
+      <c r="W57" s="55">
         <v>46082</v>
       </c>
-      <c r="X57" s="58">
+      <c r="X57" s="55">
         <v>46113</v>
       </c>
-      <c r="Y57" s="58">
+      <c r="Y57" s="55">
         <v>46143</v>
       </c>
-      <c r="Z57" s="58">
+      <c r="Z57" s="55">
         <v>46174</v>
       </c>
-      <c r="AA57" s="58">
+      <c r="AA57" s="55">
         <v>46204</v>
       </c>
-      <c r="AB57" s="58">
+      <c r="AB57" s="55">
         <v>46235</v>
       </c>
-      <c r="AC57" s="58">
+      <c r="AC57" s="55">
         <v>46266</v>
       </c>
-      <c r="AD57" s="58">
+      <c r="AD57" s="55">
         <v>46296</v>
       </c>
       <c r="AH57" t="s">
@@ -81737,7 +80639,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="64" spans="1:34" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A64" s="25">
         <v>37</v>
       </c>
@@ -81832,7 +80734,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="65" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A65" s="1">
         <v>137</v>
       </c>
@@ -81854,46 +80756,46 @@
       <c r="G65" s="7">
         <v>0.6</v>
       </c>
-      <c r="H65" s="57">
+      <c r="H65" s="7">
         <v>0.9</v>
       </c>
-      <c r="I65" s="56">
+      <c r="I65" s="7">
         <v>-0.7</v>
       </c>
-      <c r="J65" s="56">
+      <c r="J65" s="7">
         <v>-0.5</v>
       </c>
-      <c r="K65" s="56">
+      <c r="K65" s="7">
         <v>1.6</v>
       </c>
-      <c r="L65" s="56">
+      <c r="L65" s="7">
         <v>0.1</v>
       </c>
-      <c r="M65" s="56">
+      <c r="M65" s="7">
         <v>-1.4</v>
       </c>
-      <c r="N65" s="56">
+      <c r="N65" s="7">
         <v>0.9</v>
       </c>
-      <c r="O65" s="56">
+      <c r="O65" s="7">
         <v>0.9</v>
       </c>
       <c r="P65" s="7">
         <v>0.3</v>
       </c>
-      <c r="Q65" s="57">
+      <c r="Q65" s="7">
         <v>0.1</v>
       </c>
-      <c r="R65" s="56">
+      <c r="R65" s="7">
         <v>0</v>
       </c>
-      <c r="S65" s="56">
+      <c r="S65" s="7">
         <v>0.7</v>
       </c>
-      <c r="T65" s="56">
+      <c r="T65" s="7">
         <v>0.1</v>
       </c>
-      <c r="U65" s="56">
+      <c r="U65" s="7">
         <v>-0.6</v>
       </c>
       <c r="V65" s="7">
@@ -81902,19 +80804,19 @@
       <c r="W65" s="7">
         <v>1.7</v>
       </c>
-      <c r="X65" s="57">
+      <c r="X65" s="7">
         <v>0.6</v>
       </c>
-      <c r="Y65" s="56">
+      <c r="Y65" s="7">
         <v>1</v>
       </c>
-      <c r="Z65" s="56">
+      <c r="Z65" s="7">
         <v>0.2</v>
       </c>
-      <c r="AA65" s="56">
+      <c r="AA65" s="7">
         <v>-0.4</v>
       </c>
-      <c r="AB65" s="55">
+      <c r="AB65" s="28">
         <v>1.3</v>
       </c>
       <c r="AC65" s="7" t="e">
@@ -81927,7 +80829,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="66" spans="1:34" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A66" s="6">
         <v>29</v>
       </c>
@@ -82580,10 +81482,10 @@
         <v>37</v>
       </c>
       <c r="D74" s="24">
-        <v>46308.678611111114</v>
+        <v>46314.678391203706</v>
       </c>
       <c r="E74" s="49">
-        <v>46311.678611111114</v>
+        <v>46316.678391203706</v>
       </c>
       <c r="F74" s="48" t="s">
         <v>57</v>
@@ -82675,10 +81577,10 @@
         <v>37</v>
       </c>
       <c r="D75" s="15">
-        <v>46300.678460648145</v>
+        <v>46309.678148148145</v>
       </c>
       <c r="E75" s="52">
-        <v>46311.678460648138</v>
+        <v>46316.678148148145</v>
       </c>
       <c r="F75" s="43" t="s">
         <v>55</v>
@@ -82770,10 +81672,10 @@
         <v>37</v>
       </c>
       <c r="D76" s="21">
-        <v>46308.678576388891</v>
+        <v>46314.678495370368</v>
       </c>
       <c r="E76" s="53">
-        <v>46311.678576388891</v>
+        <v>46316.678495370375</v>
       </c>
       <c r="F76" s="47" t="s">
         <v>53</v>
@@ -82865,10 +81767,10 @@
         <v>37</v>
       </c>
       <c r="D77" s="24">
-        <v>46308.678483796299</v>
+        <v>46314.678310185183</v>
       </c>
       <c r="E77" s="52">
-        <v>46311.678483796306</v>
+        <v>46316.678310185176</v>
       </c>
       <c r="F77" s="48" t="s">
         <v>51</v>
@@ -82963,7 +81865,7 @@
         <v>46296.710868055554</v>
       </c>
       <c r="E78" s="52">
-        <v>46311.710868055554</v>
+        <v>46316.710868055554</v>
       </c>
       <c r="F78" s="43" t="s">
         <v>49</v>
@@ -83056,10 +81958,10 @@
         <v>37</v>
       </c>
       <c r="D79" s="21">
-        <v>46308.678437499999</v>
+        <v>46314.678263888891</v>
       </c>
       <c r="E79" s="50">
-        <v>46311.678437499999</v>
+        <v>46316.678263888898</v>
       </c>
       <c r="F79" s="47" t="s">
         <v>47</v>
@@ -83151,10 +82053,10 @@
         <v>37</v>
       </c>
       <c r="D80" s="24">
-        <v>46308.678587962961</v>
+        <v>46314.678472222222</v>
       </c>
       <c r="E80" s="49">
-        <v>46311.678587962961</v>
+        <v>46316.678472222222</v>
       </c>
       <c r="F80" s="48" t="s">
         <v>45</v>
@@ -83246,10 +82148,10 @@
         <v>42</v>
       </c>
       <c r="D81" s="15">
-        <v>46308.710844907408</v>
+        <v>46311.7108912037</v>
       </c>
       <c r="E81" s="14">
-        <v>46311.710844907415</v>
+        <v>46316.710891203693</v>
       </c>
       <c r="F81" s="43" t="s">
         <v>41</v>
@@ -83341,10 +82243,10 @@
         <v>37</v>
       </c>
       <c r="D82" s="21">
-        <v>46308.678506944445</v>
+        <v>46314.678344907406</v>
       </c>
       <c r="E82" s="20">
-        <v>46314.678506944445</v>
+        <v>46321.678344907414</v>
       </c>
       <c r="F82" s="47" t="s">
         <v>39</v>
@@ -83436,10 +82338,10 @@
         <v>37</v>
       </c>
       <c r="D83" s="15">
-        <v>46308.678599537037</v>
+        <v>46314.678553240738</v>
       </c>
       <c r="E83" s="23">
-        <v>46314.67859953703</v>
+        <v>46321.678553240738</v>
       </c>
       <c r="F83" s="43" t="s">
         <v>36</v>
@@ -86299,63 +85201,47 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G5:AD5">
-    <cfRule type="cellIs" dxfId="218" priority="219" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>0</formula>
+    <cfRule type="expression" dxfId="218" priority="217">
+      <formula>ISERROR(G5)</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G5:AD5">
     <cfRule type="cellIs" dxfId="217" priority="218" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G5:AD5">
-    <cfRule type="expression" dxfId="216" priority="217">
-      <formula>ISERROR(G5)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G6:AD6">
-    <cfRule type="cellIs" dxfId="215" priority="216" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="216" priority="219" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G6:AD6">
+    <cfRule type="expression" dxfId="215" priority="214">
+      <formula>ISERROR(G6)</formula>
+    </cfRule>
     <cfRule type="cellIs" dxfId="214" priority="215" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G6:AD6">
-    <cfRule type="expression" dxfId="213" priority="214">
-      <formula>ISERROR(G6)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G7:AD7">
-    <cfRule type="cellIs" dxfId="212" priority="213" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="213" priority="216" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G7:AD7">
+    <cfRule type="expression" dxfId="212" priority="211">
+      <formula>ISERROR(G7)</formula>
+    </cfRule>
     <cfRule type="cellIs" dxfId="211" priority="212" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G7:AD7">
-    <cfRule type="expression" dxfId="210" priority="211">
-      <formula>ISERROR(G7)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G8:AD8">
-    <cfRule type="cellIs" dxfId="209" priority="210" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="210" priority="213" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G8:AD8">
+    <cfRule type="expression" dxfId="209" priority="208">
+      <formula>ISERROR(G8)</formula>
+    </cfRule>
     <cfRule type="cellIs" dxfId="208" priority="209" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G8:AD8">
-    <cfRule type="expression" dxfId="207" priority="208">
-      <formula>ISERROR(G8)</formula>
+    <cfRule type="cellIs" dxfId="207" priority="210" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G9:AD9">
@@ -87397,83 +86283,83 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="AH3:AH96" xr:uid="{A9D9558E-5429-4BF1-B699-6B32B5587400}">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="AH3:AH96" xr:uid="{C1C4EC35-DC8A-4C87-8226-D605F47849DA}">
       <formula1>FormatOptions</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" display="https://fred.stlouisfed.org/series/MPCTXXXXS" xr:uid="{17E8B901-EBA9-4E3C-BF7C-6F33D4F30BD7}"/>
-    <hyperlink ref="C5" r:id="rId2" display="https://fred.stlouisfed.org/series/TLPRVCONS" xr:uid="{CA58FAD9-64CA-4324-95C4-4A36C9882A92}"/>
-    <hyperlink ref="C6" r:id="rId3" display="https://fred.stlouisfed.org/series/TLRESCONS" xr:uid="{11DCD466-18AA-468C-B1E3-5BE1A79156B2}"/>
-    <hyperlink ref="C7" r:id="rId4" display="https://fred.stlouisfed.org/series/TLHWYCONS" xr:uid="{7E1C2004-7AAE-4D79-BD5C-FD86CEB13A0C}"/>
-    <hyperlink ref="C8" r:id="rId5" display="https://fred.stlouisfed.org/series/HSN1F" xr:uid="{6705D8E3-FC3C-4E57-A956-00D83D466233}"/>
-    <hyperlink ref="C9" r:id="rId6" display="https://fred.stlouisfed.org/series/HOUST" xr:uid="{29E2F40B-8DA2-49E1-B7A4-0C37D2BEF5CE}"/>
-    <hyperlink ref="C11" r:id="rId7" display="https://fred.stlouisfed.org/series/UNDCONTSA" xr:uid="{74E645C9-1DB2-4556-9FE1-E755635C8796}"/>
-    <hyperlink ref="C12" r:id="rId8" display="https://fred.stlouisfed.org/series/PERMIT" xr:uid="{2C3D9BAA-CBD7-471C-8F81-691D2713D8C2}"/>
-    <hyperlink ref="C13" r:id="rId9" display="https://fred.stlouisfed.org/series/MORTGAGE30US" xr:uid="{89C94F64-9B5F-4D69-B91B-B16D15E57734}"/>
-    <hyperlink ref="C16" r:id="rId10" display="https://fred.stlouisfed.org/series/ALTSALES" xr:uid="{D2806F55-5483-4398-994A-E636976D5B00}"/>
-    <hyperlink ref="C17" r:id="rId11" display="https://fred.stlouisfed.org/series/AISRSA" xr:uid="{00F46B32-0273-460B-B639-F04A10244516}"/>
-    <hyperlink ref="C18" r:id="rId12" display="https://fred.stlouisfed.org/series/DAUTOSAAR" xr:uid="{15378A91-A16C-4E78-95DA-8DD64CB8D990}"/>
-    <hyperlink ref="C19" r:id="rId13" display="https://fred.stlouisfed.org/series/DAUPSA" xr:uid="{F776E3F5-EF3D-46C3-AA76-D4BBD56A3141}"/>
-    <hyperlink ref="C23" r:id="rId14" display="https://fred.stlouisfed.org/series/UNEMPLOY" xr:uid="{8070FA8E-5462-46B7-8AE1-94E0DD3C7843}"/>
-    <hyperlink ref="C24" r:id="rId15" display="https://fred.stlouisfed.org/series/UNRATE" xr:uid="{4FE5554B-B0C5-4C5A-8F7D-ECD924E7B172}"/>
-    <hyperlink ref="C25" r:id="rId16" display="https://fred.stlouisfed.org/series/AWHNONAG" xr:uid="{DA6AD826-2E4D-4E95-9800-4801BFAC3545}"/>
-    <hyperlink ref="C26" r:id="rId17" display="https://fred.stlouisfed.org/series/CLF16OV" xr:uid="{209ABD7D-6B1F-4E9A-B85D-DEBE38A5BE5C}"/>
-    <hyperlink ref="C29" r:id="rId18" display="https://fred.stlouisfed.org/series/INDPRO" xr:uid="{BF67B6B6-DF96-4F8F-87FD-B1DDF3785A13}"/>
-    <hyperlink ref="C30" r:id="rId19" display="https://fred.stlouisfed.org/series/TCU" xr:uid="{77FDA013-89C9-4F46-8FC2-52A55F02B061}"/>
-    <hyperlink ref="C31" r:id="rId20" display="https://fred.stlouisfed.org/series/AMTMNO" xr:uid="{58A7A0B4-A168-4794-B277-FC1301935CB1}"/>
-    <hyperlink ref="C32" r:id="rId21" display="https://fred.stlouisfed.org/series/DGORDER" xr:uid="{06FE6577-9693-435B-B63D-83F4AF742C48}"/>
-    <hyperlink ref="C33" r:id="rId22" display="https://fred.stlouisfed.org/series/ANXAVS" xr:uid="{B69C4488-9C63-4E26-99B1-4631CC5035B7}"/>
-    <hyperlink ref="C36" r:id="rId23" display="https://fred.stlouisfed.org/series/BUSINV" xr:uid="{58E5B345-A391-41EA-AE55-632E18B37CF2}"/>
-    <hyperlink ref="C37" r:id="rId24" display="https://fred.stlouisfed.org/series/ISRATIO" xr:uid="{5CA0C970-719A-4BA2-AF9B-3F6B5FF08FCD}"/>
-    <hyperlink ref="C38" r:id="rId25" display="https://fred.stlouisfed.org/series/RETAILMPCIMSA" xr:uid="{867FAC62-546F-4C2E-8EA9-AA8BB2DA4841}"/>
-    <hyperlink ref="C39" r:id="rId26" display="https://fred.stlouisfed.org/series/ACNGTI" xr:uid="{40001B3A-5116-4E9D-8B0D-AAF83220A981}"/>
-    <hyperlink ref="C42" r:id="rId27" display="https://fred.stlouisfed.org/series/CPIAUCSL" xr:uid="{FA583E57-3603-4820-8CAA-7216BB19ED29}"/>
-    <hyperlink ref="C43" r:id="rId28" display="https://fred.stlouisfed.org/series/CPIFABSL" xr:uid="{E12FD306-50B5-45A4-9C04-42F179F629D0}"/>
-    <hyperlink ref="C44" r:id="rId29" display="https://fred.stlouisfed.org/series/CPIENGSL" xr:uid="{AF16824F-D8CE-41EA-B79C-8B18D0DF0872}"/>
-    <hyperlink ref="C45" r:id="rId30" display="https://fred.stlouisfed.org/series/CPILFESL" xr:uid="{BBB59E40-90B2-4DCB-B6D3-E96CFD4BAC79}"/>
-    <hyperlink ref="C48" r:id="rId31" display="https://fred.stlouisfed.org/series/WPUFD49207" xr:uid="{D7D03978-DA2B-44EA-982C-A52B3D882F3E}"/>
-    <hyperlink ref="C49" r:id="rId32" display="https://fred.stlouisfed.org/series/WPSID61" xr:uid="{C4E8D3D8-0287-4990-B923-13A0F15B8EDF}"/>
-    <hyperlink ref="C50" r:id="rId33" display="https://fred.stlouisfed.org/series/PRAWMINDEXM" xr:uid="{645ABDF1-A464-48F4-A525-BECD670F259F}"/>
-    <hyperlink ref="C52" r:id="rId34" display="https://fred.stlouisfed.org/series/DCOILWTICO" xr:uid="{4A30E72A-A915-402F-814A-C3D5485769BC}"/>
-    <hyperlink ref="C53" r:id="rId35" display="https://fred.stlouisfed.org/series/DCOILBRENTEU" xr:uid="{F55C9448-994E-4722-B4AD-E0E9D039337F}"/>
-    <hyperlink ref="C54" r:id="rId36" display="https://fred.stlouisfed.org/series/DHHNGSP" xr:uid="{1C36EA57-C63C-4BC4-ACD1-47F4935D521F}"/>
-    <hyperlink ref="C58" r:id="rId37" display="https://fred.stlouisfed.org/series/DHHNGSP" xr:uid="{93EA94E8-8E77-45BA-91EA-C031CCBB7ECC}"/>
-    <hyperlink ref="C59" r:id="rId38" display="https://fred.stlouisfed.org/series/PI" xr:uid="{B263E9E8-93C4-467B-86DB-A62DEC6DA90A}"/>
-    <hyperlink ref="C60" r:id="rId39" display="https://fred.stlouisfed.org/series/DSPI" xr:uid="{01AA1D18-E6F6-49F5-B9F9-369D15C47FCA}"/>
-    <hyperlink ref="C61" r:id="rId40" display="https://fred.stlouisfed.org/series/A229RX0" xr:uid="{E573397F-5202-443E-AEDC-611E9CD974B5}"/>
-    <hyperlink ref="C62" r:id="rId41" display="https://fred.stlouisfed.org/series/PSAVERT" xr:uid="{E89AAFC2-09B9-418A-8549-2B664E29CAF4}"/>
-    <hyperlink ref="C63" r:id="rId42" display="https://fred.stlouisfed.org/series/PCE" xr:uid="{0470B37E-D629-4D26-9038-D616204B2E90}"/>
-    <hyperlink ref="C64" r:id="rId43" display="https://fred.stlouisfed.org/series/PCEC96" xr:uid="{1B3D443C-A064-408A-9347-E73A7DE6F125}"/>
-    <hyperlink ref="C65" r:id="rId44" display="https://fred.stlouisfed.org/series/MRTSMPCSM44X72USS" xr:uid="{46B4B882-0B06-4A25-B43C-F29CED029993}"/>
-    <hyperlink ref="C66" r:id="rId45" display="https://fred.stlouisfed.org/series/TOTALSL" xr:uid="{97FF2585-2F6F-4265-AAE1-EA737F97E5C2}"/>
-    <hyperlink ref="C67" r:id="rId46" display="https://fred.stlouisfed.org/series/PCEND" xr:uid="{06BE4DBE-0FA1-43C8-AC23-DE2F9D943726}"/>
-    <hyperlink ref="C68" r:id="rId47" display="https://fred.stlouisfed.org/series/A22BVS" xr:uid="{DF0242DB-2BE1-4275-9064-580D512E9010}"/>
-    <hyperlink ref="C71" r:id="rId48" display="https://fred.stlouisfed.org/series/M1SL" xr:uid="{CFE68BA7-DDA6-474C-BF32-46471C207DEE}"/>
-    <hyperlink ref="C72" r:id="rId49" display="https://fred.stlouisfed.org/series/M2SL" xr:uid="{C0D7087F-DA62-4F55-91A0-F4504F50BB7A}"/>
-    <hyperlink ref="C74" r:id="rId50" display="https://fred.stlouisfed.org/series/DTB3" xr:uid="{3DC83600-057D-4156-8480-0DFECF911026}"/>
-    <hyperlink ref="C75" r:id="rId51" display="https://fred.stlouisfed.org/series/DPRIME" xr:uid="{71BF243A-8E99-4B4F-8C6E-C27CCC1A62C3}"/>
-    <hyperlink ref="C76" r:id="rId52" display="https://fred.stlouisfed.org/series/DGS10" xr:uid="{5DAA4E2D-32D0-42ED-94C0-9D0B522CB784}"/>
-    <hyperlink ref="C79" r:id="rId53" display="https://fred.stlouisfed.org/series/DFII10" xr:uid="{EC2B69AD-408E-4318-89F0-4F2B1354A786}"/>
-    <hyperlink ref="C80" r:id="rId54" display="https://fred.stlouisfed.org/series/DGS30" xr:uid="{9E84FB9E-8614-40B4-B36F-1EFDDFD828D1}"/>
-    <hyperlink ref="C82" r:id="rId55" display="https://fred.stlouisfed.org/series/DEXUSEU" xr:uid="{6593C8AC-1B07-473B-8D48-C9F4891BE421}"/>
-    <hyperlink ref="C83" r:id="rId56" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{DC3F9DEE-6206-4308-B737-5091BC6D04B6}"/>
-    <hyperlink ref="C87" r:id="rId57" display="https://fred.stlouisfed.org/series/GDPC1" xr:uid="{8727B8CA-3858-4553-8A7C-051F5323DC01}"/>
-    <hyperlink ref="C88" r:id="rId58" display="https://fred.stlouisfed.org/series/GDP" xr:uid="{3FD13192-8FD0-42B5-980F-0F9372A157E6}"/>
-    <hyperlink ref="C89" r:id="rId59" display="https://fred.stlouisfed.org/series/PCEDG" xr:uid="{FECFA1FD-56CD-4F49-B1E6-B3F273FD4E7B}"/>
-    <hyperlink ref="C90" r:id="rId60" display="https://fred.stlouisfed.org/series/PNFIC1" xr:uid="{AE6970E2-8649-457E-900F-9C60B6F006DF}"/>
-    <hyperlink ref="C91" r:id="rId61" display="https://fred.stlouisfed.org/series/PRFIC1" xr:uid="{019F6A9C-3894-4849-9BF0-0EB1FB7407F0}"/>
-    <hyperlink ref="C92" r:id="rId62" display="https://fred.stlouisfed.org/series/CBI" xr:uid="{0CB60F77-88EC-4926-891E-14A6F1741724}"/>
-    <hyperlink ref="C93" r:id="rId63" display="https://fred.stlouisfed.org/series/NETEXC" xr:uid="{5F459512-539A-4C66-B37A-E08A71715C0C}"/>
-    <hyperlink ref="C94" r:id="rId64" display="https://fred.stlouisfed.org/series/IEABC" xr:uid="{D75EF6A1-4807-43FC-A428-65971F1CD5F2}"/>
-    <hyperlink ref="C73" r:id="rId65" display="https://fred.stlouisfed.org/series/BOPGSTB" xr:uid="{6D7AB9AE-BCDB-46A7-8AF0-5A157400CF5D}"/>
-    <hyperlink ref="C95" r:id="rId66" display="https://fred.stlouisfed.org/series/GCEC1" xr:uid="{5121CB33-8812-4A95-9A0E-4919B0DC84A9}"/>
-    <hyperlink ref="C96" r:id="rId67" display="https://fred.stlouisfed.org/series/EVACANTUSQ176N" xr:uid="{F7B4FCFA-DC3F-4E2F-88A4-6CBCFA12DCA8}"/>
-    <hyperlink ref="C81" r:id="rId68" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{68713AC5-7C7B-4901-90E0-01FA9FB35F84}"/>
-    <hyperlink ref="C78" r:id="rId69" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{C47C161D-CA57-4BE8-934E-984F4E416D23}"/>
-    <hyperlink ref="C77" r:id="rId70" display="https://fred.stlouisfed.org/series/DGS10" xr:uid="{09C7050A-DA34-459B-9C0F-E253909FEBBE}"/>
-    <hyperlink ref="C51" r:id="rId71" display="https://fred.stlouisfed.org/series/PRAWMINDEXM" xr:uid="{D8F2165E-0C3D-418C-82CD-AEE4168BC466}"/>
-    <hyperlink ref="C22" r:id="rId72" display="https://fred.stlouisfed.org/series/PAYEMS" xr:uid="{7597B993-5237-4E34-A0B4-EEC3B5F5DDF4}"/>
+    <hyperlink ref="C4" r:id="rId1" display="https://fred.stlouisfed.org/series/MPCTXXXXS" xr:uid="{CF562D95-77DF-463A-81CC-636269FBA42E}"/>
+    <hyperlink ref="C5" r:id="rId2" display="https://fred.stlouisfed.org/series/TLPRVCONS" xr:uid="{8C494690-1C0A-4EA1-B518-334AFC20BDB1}"/>
+    <hyperlink ref="C6" r:id="rId3" display="https://fred.stlouisfed.org/series/TLRESCONS" xr:uid="{4606C91C-70A9-40C6-938A-685BF93775E3}"/>
+    <hyperlink ref="C7" r:id="rId4" display="https://fred.stlouisfed.org/series/TLHWYCONS" xr:uid="{634DE402-8226-48EA-A6C9-72424EB7A1A2}"/>
+    <hyperlink ref="C8" r:id="rId5" display="https://fred.stlouisfed.org/series/HSN1F" xr:uid="{F7187EBE-4443-4DF1-ABA4-A814D18C4730}"/>
+    <hyperlink ref="C9" r:id="rId6" display="https://fred.stlouisfed.org/series/HOUST" xr:uid="{3D90EA5C-6EE1-4ACA-8266-9953FCD68BE6}"/>
+    <hyperlink ref="C11" r:id="rId7" display="https://fred.stlouisfed.org/series/UNDCONTSA" xr:uid="{FF7E682F-76C4-4CAE-B72B-C7E0382A91B6}"/>
+    <hyperlink ref="C12" r:id="rId8" display="https://fred.stlouisfed.org/series/PERMIT" xr:uid="{360B60BB-D93C-412B-8010-D85542BEEB74}"/>
+    <hyperlink ref="C13" r:id="rId9" display="https://fred.stlouisfed.org/series/MORTGAGE30US" xr:uid="{28D477DE-31FF-4CF6-88FC-F349B761E769}"/>
+    <hyperlink ref="C16" r:id="rId10" display="https://fred.stlouisfed.org/series/ALTSALES" xr:uid="{62774A1B-E813-462D-A3C8-B54F32DD75A7}"/>
+    <hyperlink ref="C17" r:id="rId11" display="https://fred.stlouisfed.org/series/AISRSA" xr:uid="{4B9D3D16-05A1-4F1B-8986-CC2AFD1124FB}"/>
+    <hyperlink ref="C18" r:id="rId12" display="https://fred.stlouisfed.org/series/DAUTOSAAR" xr:uid="{E19626E5-F306-4F83-96B4-0293E9399306}"/>
+    <hyperlink ref="C19" r:id="rId13" display="https://fred.stlouisfed.org/series/DAUPSA" xr:uid="{E18C780B-6D16-45F6-B2C6-4E96265D85C6}"/>
+    <hyperlink ref="C23" r:id="rId14" display="https://fred.stlouisfed.org/series/UNEMPLOY" xr:uid="{2A27EF66-83BB-4B10-BF17-206F6E700666}"/>
+    <hyperlink ref="C24" r:id="rId15" display="https://fred.stlouisfed.org/series/UNRATE" xr:uid="{FA49F51E-6348-49EF-960B-72E9CB0BC8A9}"/>
+    <hyperlink ref="C25" r:id="rId16" display="https://fred.stlouisfed.org/series/AWHNONAG" xr:uid="{A3BEF371-A6F1-4A68-A332-0A226320B24E}"/>
+    <hyperlink ref="C26" r:id="rId17" display="https://fred.stlouisfed.org/series/CLF16OV" xr:uid="{FC53E953-1958-42B5-BEB5-A0802E39B40D}"/>
+    <hyperlink ref="C29" r:id="rId18" display="https://fred.stlouisfed.org/series/INDPRO" xr:uid="{D012F5A8-BFF2-41DD-8E3D-874A47E9721C}"/>
+    <hyperlink ref="C30" r:id="rId19" display="https://fred.stlouisfed.org/series/TCU" xr:uid="{6FBDBF95-0FE4-4D21-85EC-6BE7C0F96FF4}"/>
+    <hyperlink ref="C31" r:id="rId20" display="https://fred.stlouisfed.org/series/AMTMNO" xr:uid="{2A326159-DD63-4C31-8041-A13ACA187AC4}"/>
+    <hyperlink ref="C32" r:id="rId21" display="https://fred.stlouisfed.org/series/DGORDER" xr:uid="{D9E2DDA6-AE91-4AD5-ACB1-A3FA3172BD80}"/>
+    <hyperlink ref="C33" r:id="rId22" display="https://fred.stlouisfed.org/series/ANXAVS" xr:uid="{6729710C-1955-46FB-9A36-AD1447C4916A}"/>
+    <hyperlink ref="C36" r:id="rId23" display="https://fred.stlouisfed.org/series/BUSINV" xr:uid="{D4B9F793-7BF2-4540-AA71-73E369FDB0DD}"/>
+    <hyperlink ref="C37" r:id="rId24" display="https://fred.stlouisfed.org/series/ISRATIO" xr:uid="{3635BEF7-AD8F-4B7D-AC36-756A48933CB5}"/>
+    <hyperlink ref="C38" r:id="rId25" display="https://fred.stlouisfed.org/series/RETAILMPCIMSA" xr:uid="{44BC184D-1C05-4539-BAE0-803E418F78B1}"/>
+    <hyperlink ref="C39" r:id="rId26" display="https://fred.stlouisfed.org/series/ACNGTI" xr:uid="{E83143F4-7734-4A90-8913-BDCF58854D25}"/>
+    <hyperlink ref="C42" r:id="rId27" display="https://fred.stlouisfed.org/series/CPIAUCSL" xr:uid="{4754EE6A-75E0-4F28-982B-1A2AF52D284A}"/>
+    <hyperlink ref="C43" r:id="rId28" display="https://fred.stlouisfed.org/series/CPIFABSL" xr:uid="{B5DBBAEC-9FA2-4228-B3B0-B292FAA6BB56}"/>
+    <hyperlink ref="C44" r:id="rId29" display="https://fred.stlouisfed.org/series/CPIENGSL" xr:uid="{0BF3E961-627C-42D9-96B1-57332FE72031}"/>
+    <hyperlink ref="C45" r:id="rId30" display="https://fred.stlouisfed.org/series/CPILFESL" xr:uid="{23633F4C-CD5D-4692-B2EE-B4D9D2ACBCBE}"/>
+    <hyperlink ref="C48" r:id="rId31" display="https://fred.stlouisfed.org/series/WPUFD49207" xr:uid="{D114408D-9660-49D9-861F-8113E471CB40}"/>
+    <hyperlink ref="C49" r:id="rId32" display="https://fred.stlouisfed.org/series/WPSID61" xr:uid="{275E4CF3-8879-4989-8FE4-13EDAAD37ABA}"/>
+    <hyperlink ref="C50" r:id="rId33" display="https://fred.stlouisfed.org/series/PRAWMINDEXM" xr:uid="{7D80E8EA-7B77-4AC9-8F0D-F5DA1F312DBE}"/>
+    <hyperlink ref="C52" r:id="rId34" display="https://fred.stlouisfed.org/series/DCOILWTICO" xr:uid="{AAB67C0A-B21A-4D58-B50B-0C4AFB228547}"/>
+    <hyperlink ref="C53" r:id="rId35" display="https://fred.stlouisfed.org/series/DCOILBRENTEU" xr:uid="{9A86CB8B-8C04-4E35-A7E2-54579C53E91F}"/>
+    <hyperlink ref="C54" r:id="rId36" display="https://fred.stlouisfed.org/series/DHHNGSP" xr:uid="{2C16E224-C3BD-4137-8FCD-9594D9D5B585}"/>
+    <hyperlink ref="C58" r:id="rId37" display="https://fred.stlouisfed.org/series/DHHNGSP" xr:uid="{3F262E2D-EA22-464F-9DB9-BA59AABC28DB}"/>
+    <hyperlink ref="C59" r:id="rId38" display="https://fred.stlouisfed.org/series/PI" xr:uid="{21569B9C-C2AD-4E0F-BAFD-7CE64C33FB90}"/>
+    <hyperlink ref="C60" r:id="rId39" display="https://fred.stlouisfed.org/series/DSPI" xr:uid="{61869BC9-BAF4-4DAC-B141-86F531C90736}"/>
+    <hyperlink ref="C61" r:id="rId40" display="https://fred.stlouisfed.org/series/A229RX0" xr:uid="{27E4895C-EB1B-4CE7-8DCD-0B774804C245}"/>
+    <hyperlink ref="C62" r:id="rId41" display="https://fred.stlouisfed.org/series/PSAVERT" xr:uid="{A92B07B3-36C5-41A3-B2CF-0993D31B8038}"/>
+    <hyperlink ref="C63" r:id="rId42" display="https://fred.stlouisfed.org/series/PCE" xr:uid="{C52F2B8C-278E-41EC-B982-3FDCCC563887}"/>
+    <hyperlink ref="C64" r:id="rId43" display="https://fred.stlouisfed.org/series/PCEC96" xr:uid="{7BE8C9E1-F701-488D-8ACC-D9A0DDF6A86B}"/>
+    <hyperlink ref="C65" r:id="rId44" display="https://fred.stlouisfed.org/series/MRTSMPCSM44X72USS" xr:uid="{96571A34-126C-4D5C-B192-6018B3347B28}"/>
+    <hyperlink ref="C66" r:id="rId45" display="https://fred.stlouisfed.org/series/TOTALSL" xr:uid="{441D994A-6343-43BC-B404-00268E8A132D}"/>
+    <hyperlink ref="C67" r:id="rId46" display="https://fred.stlouisfed.org/series/PCEND" xr:uid="{6A732520-3DBD-4885-BA1E-97C9AFD5BFEE}"/>
+    <hyperlink ref="C68" r:id="rId47" display="https://fred.stlouisfed.org/series/A22BVS" xr:uid="{C60F5F87-72DB-4C08-8BB4-C055A8D0B0BA}"/>
+    <hyperlink ref="C71" r:id="rId48" display="https://fred.stlouisfed.org/series/M1SL" xr:uid="{C33366E6-16B8-4A32-B908-D27298DFB7B9}"/>
+    <hyperlink ref="C72" r:id="rId49" display="https://fred.stlouisfed.org/series/M2SL" xr:uid="{2203B1FB-5C4B-4FCC-A707-407631381606}"/>
+    <hyperlink ref="C74" r:id="rId50" display="https://fred.stlouisfed.org/series/DTB3" xr:uid="{D937E583-65DE-4D9E-9717-1C3F3EBFCCD2}"/>
+    <hyperlink ref="C75" r:id="rId51" display="https://fred.stlouisfed.org/series/DPRIME" xr:uid="{7E883408-6D78-47B8-BCAA-45F649C4DEC0}"/>
+    <hyperlink ref="C76" r:id="rId52" display="https://fred.stlouisfed.org/series/DGS10" xr:uid="{6D73C1BC-9303-4BA6-B122-C19894E23F67}"/>
+    <hyperlink ref="C79" r:id="rId53" display="https://fred.stlouisfed.org/series/DFII10" xr:uid="{8FC678B4-A334-4987-A4F0-7B22956B50B9}"/>
+    <hyperlink ref="C80" r:id="rId54" display="https://fred.stlouisfed.org/series/DGS30" xr:uid="{292CF90C-3D97-424F-BC2B-7CE99BB00206}"/>
+    <hyperlink ref="C82" r:id="rId55" display="https://fred.stlouisfed.org/series/DEXUSEU" xr:uid="{811824CA-1C69-4548-B771-1C5EFF998A60}"/>
+    <hyperlink ref="C83" r:id="rId56" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{0057E3E9-4010-4CC3-9970-AF8E9F70AFB4}"/>
+    <hyperlink ref="C87" r:id="rId57" display="https://fred.stlouisfed.org/series/GDPC1" xr:uid="{6FD6C9EC-B7EC-4567-80C3-5B54C3A7F39C}"/>
+    <hyperlink ref="C88" r:id="rId58" display="https://fred.stlouisfed.org/series/GDP" xr:uid="{0B9EA38B-FF63-4491-B0A2-5F006EE61A49}"/>
+    <hyperlink ref="C89" r:id="rId59" display="https://fred.stlouisfed.org/series/PCEDG" xr:uid="{E012DCC7-02BD-4B94-BB81-EFA086DC9F35}"/>
+    <hyperlink ref="C90" r:id="rId60" display="https://fred.stlouisfed.org/series/PNFIC1" xr:uid="{B318CB31-CE2A-40E2-8BA4-78CFC38B38CF}"/>
+    <hyperlink ref="C91" r:id="rId61" display="https://fred.stlouisfed.org/series/PRFIC1" xr:uid="{B8DDA874-1E07-4B0F-B56B-A706F6F7964A}"/>
+    <hyperlink ref="C92" r:id="rId62" display="https://fred.stlouisfed.org/series/CBI" xr:uid="{2629D423-F984-45E8-8100-4F414E965B21}"/>
+    <hyperlink ref="C93" r:id="rId63" display="https://fred.stlouisfed.org/series/NETEXC" xr:uid="{0443940F-9918-43E0-9C87-8E14D6FB970F}"/>
+    <hyperlink ref="C94" r:id="rId64" display="https://fred.stlouisfed.org/series/IEABC" xr:uid="{FF63A1A7-6D7D-4CF1-B8B8-639A144D2795}"/>
+    <hyperlink ref="C73" r:id="rId65" display="https://fred.stlouisfed.org/series/BOPGSTB" xr:uid="{CC908B37-E115-4BF9-BA2B-C868CF63A3EF}"/>
+    <hyperlink ref="C95" r:id="rId66" display="https://fred.stlouisfed.org/series/GCEC1" xr:uid="{7AD691CE-D4C5-4F5B-8C28-D5D144374A94}"/>
+    <hyperlink ref="C96" r:id="rId67" display="https://fred.stlouisfed.org/series/EVACANTUSQ176N" xr:uid="{09EF3F06-48BA-4537-8C90-A2561AE81204}"/>
+    <hyperlink ref="C81" r:id="rId68" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{CADAA938-7E05-4E34-B0E8-23D9412E1025}"/>
+    <hyperlink ref="C78" r:id="rId69" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{E6D706A3-B3BF-445A-A58C-4DD3A4C3C1CF}"/>
+    <hyperlink ref="C77" r:id="rId70" display="https://fred.stlouisfed.org/series/DGS10" xr:uid="{E1A72690-BF2C-430A-BA17-54A478B1D95A}"/>
+    <hyperlink ref="C51" r:id="rId71" display="https://fred.stlouisfed.org/series/PRAWMINDEXM" xr:uid="{D79B4C81-B8AF-4791-A538-EA979757ACBC}"/>
+    <hyperlink ref="C22" r:id="rId72" display="https://fred.stlouisfed.org/series/PAYEMS" xr:uid="{F823A10C-C3AD-4D41-BE55-DE5F2B1BC197}"/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.3" footer="0.3"/>
   <pageSetup scale="64" orientation="landscape" r:id="rId73"/>

</xml_diff>

<commit_message>
Publish EconSheet 261020 (October 20, 2026)
</commit_message>
<xml_diff>
--- a/files/EconSheet.xlsx
+++ b/files/EconSheet.xlsx
@@ -8,44 +8,44 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.0.130\Documents\Business\EconSheet\FREDData\ToDistribute\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{BED8F52D-4100-4EA3-88DA-3D0A44F283A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA137B4E-0FDB-4396-8D52-96235E809950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{0425FD2D-B739-4B05-B6DC-E6B9D2EE0831}"/>
+    <workbookView xWindow="-28920" yWindow="5295" windowWidth="29040" windowHeight="15720" xr2:uid="{5D5A21E5-3D6F-4F88-A7F3-0ABA08D205B7}"/>
   </bookViews>
   <sheets>
-    <sheet name="261019 EconSheet" sheetId="1" r:id="rId1"/>
+    <sheet name="261020 EconSheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId2"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'261019 EconSheet'!$A$28:$AF$33</definedName>
-    <definedName name="Conditions" localSheetId="0">'261019 EconSheet'!$AH$3:$AH$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'261020 EconSheet'!$A$28:$AF$33</definedName>
+    <definedName name="Conditions" localSheetId="0">'261020 EconSheet'!$AH$3:$AH$96</definedName>
     <definedName name="CurrDates">[1]Currencies!$A$8:$A$14337</definedName>
     <definedName name="DataStart">'[1]Retrieved Data'!$A$1</definedName>
-    <definedName name="DataTable" localSheetId="0">'261019 EconSheet'!$G$4:$AD$96</definedName>
-    <definedName name="DataTableStart" localSheetId="0">'261019 EconSheet'!$G$4</definedName>
-    <definedName name="DatesAndSeries" localSheetId="0">'261019 EconSheet'!$E$4:$F$96</definedName>
+    <definedName name="DataTable" localSheetId="0">'261020 EconSheet'!$G$4:$AD$96</definedName>
+    <definedName name="DataTableStart" localSheetId="0">'261020 EconSheet'!$G$4</definedName>
+    <definedName name="DatesAndSeries" localSheetId="0">'261020 EconSheet'!$E$4:$F$96</definedName>
     <definedName name="DatesAndSeries">[1]EconSheet!$E$4:$F$96</definedName>
-    <definedName name="DatesCol" localSheetId="0">'261019 EconSheet'!$E$4:$E$96</definedName>
+    <definedName name="DatesCol" localSheetId="0">'261020 EconSheet'!$E$4:$E$96</definedName>
     <definedName name="DatesCol">[1]EconSheet!$E$4:$E$96</definedName>
-    <definedName name="ESSeries" localSheetId="0">'261019 EconSheet'!$B$4:$B$103</definedName>
-    <definedName name="ForceAll" localSheetId="0">'261019 EconSheet'!#REF!</definedName>
+    <definedName name="ESSeries" localSheetId="0">'261020 EconSheet'!$B$4:$B$103</definedName>
+    <definedName name="ForceAll" localSheetId="0">'261020 EconSheet'!#REF!</definedName>
     <definedName name="FormatOptions">[1]Calculations!$U$3:$U$14</definedName>
-    <definedName name="FormatTable" localSheetId="0">'261019 EconSheet'!$A$1:$AD$96</definedName>
+    <definedName name="FormatTable" localSheetId="0">'261020 EconSheet'!$A$1:$AD$96</definedName>
     <definedName name="PPIGreen">'[1]Producer Price Archive'!$AB$8:$AD$1023</definedName>
     <definedName name="PPIRaw">'[1]Producer Price Archive'!$B$7:$F$1023</definedName>
     <definedName name="PPIRed">'[1]Producer Price Archive'!$AF$8:$AH$1023</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'261019 EconSheet'!$F$1:$AD$54,'261019 EconSheet'!$F$56:$AD$96</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'261020 EconSheet'!$F$1:$AD$54,'261020 EconSheet'!$F$56:$AD$96</definedName>
     <definedName name="ReleaseData">[1]ReleaseDates!$A$2:$E$1882</definedName>
     <definedName name="ReleaseDates">[1]ReleaseDates!$A$2:$A$1898</definedName>
     <definedName name="SDSeries">[1]SeriesData!$A$2:$A$76</definedName>
     <definedName name="SeriesLookup">'[1]Retrieved Data'!$A$1:$ET$1</definedName>
-    <definedName name="SpFormat1" localSheetId="0">'261019 EconSheet'!$AH$131</definedName>
-    <definedName name="SpFormat2" localSheetId="0">'261019 EconSheet'!$AH$136</definedName>
-    <definedName name="TrueFalse" localSheetId="0">'261019 EconSheet'!#REF!</definedName>
+    <definedName name="SpFormat1" localSheetId="0">'261020 EconSheet'!$AH$131</definedName>
+    <definedName name="SpFormat2" localSheetId="0">'261020 EconSheet'!$AH$136</definedName>
+    <definedName name="TrueFalse" localSheetId="0">'261020 EconSheet'!#REF!</definedName>
     <definedName name="TrueFalse">[1]EconSheet!$AU$1:$AU$2</definedName>
-    <definedName name="WholeTable" localSheetId="0">'261019 EconSheet'!$F$1:$AD$96</definedName>
+    <definedName name="WholeTable" localSheetId="0">'261020 EconSheet'!$F$1:$AD$96</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -76,7 +76,7 @@
     <author>Ron Levin</author>
   </authors>
   <commentList>
-    <comment ref="X29" authorId="0" shapeId="0" xr:uid="{55797B3F-3B6C-489D-BBDE-A7D108AF02E3}">
+    <comment ref="AA9" authorId="0" shapeId="0" xr:uid="{9E692B9A-28CC-4E72-A432-9BB7B9CE993D}">
       <text>
         <r>
           <rPr>
@@ -86,11 +86,11 @@
             <family val="2"/>
           </rPr>
           <t>Previous Value:
-0.8</t>
+1,309</t>
         </r>
       </text>
     </comment>
-    <comment ref="Y29" authorId="0" shapeId="0" xr:uid="{2C91E6BE-B914-4483-A3D3-F3A35CB76275}">
+    <comment ref="AB9" authorId="0" shapeId="0" xr:uid="{7583EB98-9947-4C84-B81D-F120C8D9C52E}">
       <text>
         <r>
           <rPr>
@@ -100,53 +100,11 @@
             <family val="2"/>
           </rPr>
           <t>Previous Value:
-0.1</t>
+1,275</t>
         </r>
       </text>
     </comment>
-    <comment ref="Z29" authorId="0" shapeId="0" xr:uid="{FCEEBA06-DA9D-4788-92A6-E23B4D2C7ABC}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AA29" authorId="0" shapeId="0" xr:uid="{BD3070E4-BE85-498A-86A6-B33628FD63FF}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AB29" authorId="0" shapeId="0" xr:uid="{BB441084-368F-4909-8EFD-8688D269F7E0}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-0.0</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AC29" authorId="0" shapeId="0" xr:uid="{9F9822E7-A64D-4D53-A9DD-8D8EA88E8535}">
+    <comment ref="AC9" authorId="0" shapeId="0" xr:uid="{F5971552-6335-4A0E-B942-BC3017D90F6A}">
       <text>
         <r>
           <rPr>
@@ -159,7 +117,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X30" authorId="0" shapeId="0" xr:uid="{163FB9E0-E092-4563-888B-CDE197D1AA7F}">
+    <comment ref="AB11" authorId="0" shapeId="0" xr:uid="{916C8F4A-23EC-45CF-8ED5-CAFD2BF0441D}">
       <text>
         <r>
           <rPr>
@@ -169,11 +127,11 @@
             <family val="2"/>
           </rPr>
           <t>Previous Value:
-76.2</t>
+1,271</t>
         </r>
       </text>
     </comment>
-    <comment ref="Y30" authorId="0" shapeId="0" xr:uid="{D5B91344-1001-465D-B76A-0E6E78AF3F7B}">
+    <comment ref="AC11" authorId="0" shapeId="0" xr:uid="{A68CC196-00B3-4203-931A-D564A3E0DC0F}">
       <text>
         <r>
           <rPr>
@@ -182,54 +140,11 @@
             <rFont val="Tahoma"/>
             <family val="2"/>
           </rPr>
-          <t>Previous Value:
-76.2</t>
+          <t>New Value</t>
         </r>
       </text>
     </comment>
-    <comment ref="Z30" authorId="0" shapeId="0" xr:uid="{62EEC66D-2F1F-4647-9FBC-77D07824B6AA}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-76.2</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AA30" authorId="0" shapeId="0" xr:uid="{3168B595-DB14-4EE2-A5F9-BF14301BCCA3}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-76.3</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AB30" authorId="0" shapeId="0" xr:uid="{EAABAAFE-CF63-4960-93C1-2F173295B25D}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-76.3</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AC30" authorId="0" shapeId="0" xr:uid="{32D17454-8188-4CDE-B9D1-061BFBF337F6}">
+    <comment ref="AC12" authorId="0" shapeId="0" xr:uid="{9687FA9B-AE28-472A-941C-5CB9355BD05C}">
       <text>
         <r>
           <rPr>
@@ -807,7 +722,7 @@
     <t>Green if</t>
   </si>
   <si>
-    <t>Next Update: 10/20/26</t>
+    <t>Next Update: 10/21/26</t>
   </si>
   <si>
     <t>Next Update</t>
@@ -960,7 +875,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -983,19 +898,6 @@
       <top/>
       <bottom style="thin">
         <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color indexed="64"/>
-      </right>
-      <top style="thick">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thick">
-        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -1026,16 +928,16 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thick">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="thick">
         <color indexed="64"/>
       </right>
       <top style="thick">
-        <color auto="1"/>
+        <color indexed="64"/>
       </top>
-      <bottom/>
+      <bottom style="thick">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -1124,14 +1026,14 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="6" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="4" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="4" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="168" fontId="9" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="22" fontId="9" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -1144,7 +1046,7 @@
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{D0FE01E7-A8B7-45DE-A2D6-B3C532B960D9}"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{CE4BE9F1-32C3-44C5-B291-7BF686F9B6A6}"/>
   </cellStyles>
   <dxfs count="237">
     <dxf>
@@ -2232,7 +2134,9 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="0"/>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF10651B"/>
       </font>
     </dxf>
     <dxf>
@@ -2244,9 +2148,21 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
         <color rgb="FF10651B"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF711204"/>
       </font>
     </dxf>
     <dxf>
@@ -2258,7 +2174,19 @@
       <font>
         <b/>
         <i val="0"/>
+        <color rgb="FF10651B"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
         <color rgb="FF711204"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
       </font>
     </dxf>
     <dxf>
@@ -2270,7 +2198,21 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF711204"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF10651B"/>
       </font>
     </dxf>
     <dxf>
@@ -2282,9 +2224,21 @@
     </dxf>
     <dxf>
       <font>
+        <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <b/>
         <i val="0"/>
         <color rgb="FF10651B"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF711204"/>
       </font>
     </dxf>
     <dxf>
@@ -2296,7 +2250,19 @@
       <font>
         <b/>
         <i val="0"/>
+        <color rgb="FF10651B"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
         <color rgb="FF711204"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
       </font>
     </dxf>
     <dxf>
@@ -2308,7 +2274,21 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF711204"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF10651B"/>
       </font>
     </dxf>
     <dxf>
@@ -2320,103 +2300,20 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF10651B"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF711204"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF10651B"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF711204"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF10651B"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF711204"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF10651B"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF711204"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF10651B"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <color theme="0"/>
       </font>
     </dxf>
     <dxf>
       <border>
         <left style="thin">
-          <color indexed="10"/>
+          <color indexed="17"/>
         </left>
       </border>
     </dxf>
     <dxf>
       <border>
         <left style="thin">
-          <color indexed="17"/>
+          <color indexed="10"/>
         </left>
       </border>
     </dxf>
@@ -2429,7 +2326,19 @@
       <font>
         <b/>
         <i val="0"/>
+        <color rgb="FF10651B"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
         <color rgb="FF711204"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
       </font>
     </dxf>
     <dxf>
@@ -2441,7 +2350,21 @@
     </dxf>
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF711204"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF10651B"/>
       </font>
     </dxf>
     <dxf>
@@ -2453,14 +2376,14 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF10651B"/>
+        <color theme="0"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <color theme="0"/>
+        <b/>
+        <i val="0"/>
+        <color rgb="FF10651B"/>
       </font>
     </dxf>
     <dxf>
@@ -2472,28 +2395,7 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF10651B"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <color theme="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF711204"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <color rgb="FF10651B"/>
       </font>
     </dxf>
     <dxf>
@@ -2780,7 +2682,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B89EDBD4-4CA4-4396-8E4C-322A27C3062B}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7E933BE9-B345-4892-A5E3-30895A269C8F}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2825,7 +2727,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F9D60A36-CBD4-4FF0-AEF3-959CF7C68926}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F456B20C-A8A6-4CF4-BDD0-D068DB2FCC14}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2944,7 +2846,7 @@
         </row>
         <row r="9">
           <cell r="E9">
-            <v>46315.35601851852</v>
+            <v>46322.356678240743</v>
           </cell>
           <cell r="F9" t="str">
             <v>Housing Starts (000's of units, AR)</v>
@@ -2957,7 +2859,7 @@
         </row>
         <row r="11">
           <cell r="E11">
-            <v>46315.356180555566</v>
+            <v>46322.356747685175</v>
           </cell>
           <cell r="F11" t="str">
             <v>Housing Under Construction (000's of units, AR)</v>
@@ -2965,7 +2867,7 @@
         </row>
         <row r="12">
           <cell r="E12">
-            <v>46315.419166666659</v>
+            <v>46322.356828703705</v>
           </cell>
           <cell r="F12" t="str">
             <v>Housing Permits (% Δ)</v>
@@ -43637,10 +43539,10 @@
             <v>46315</v>
           </cell>
           <cell r="C33" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D33">
-            <v>46315</v>
+            <v>0</v>
           </cell>
           <cell r="E33">
             <v>33</v>
@@ -75482,7 +75384,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DFA9851-77AC-49AA-A71B-D92A92205070}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8996EBC1-CAA1-4757-AC2A-3D6476573764}">
   <sheetPr codeName="Sheet22">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -75689,10 +75591,10 @@
       </c>
       <c r="C3" s="10"/>
       <c r="D3" s="71">
-        <v>46314.678553240738</v>
+        <v>46315.356828703705</v>
       </c>
       <c r="E3" s="70">
-        <v>46315.35601851852</v>
+        <v>46316.675405092596</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>183</v>
@@ -76108,7 +76010,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:34" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1">
         <v>9</v>
       </c>
@@ -76203,7 +76105,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6">
         <v>7</v>
       </c>
@@ -76214,10 +76116,10 @@
         <v>166</v>
       </c>
       <c r="D9" s="21">
-        <v>46282.35601851852</v>
+        <v>46315.356678240743</v>
       </c>
       <c r="E9" s="50">
-        <v>46315.35601851852</v>
+        <v>46322.356678240743</v>
       </c>
       <c r="F9" s="47" t="s">
         <v>171</v>
@@ -76282,14 +76184,14 @@
       <c r="Z9" s="18">
         <v>1439</v>
       </c>
-      <c r="AA9" s="17">
-        <v>1309</v>
-      </c>
-      <c r="AB9" s="17">
-        <v>1275</v>
-      </c>
-      <c r="AC9" s="18" t="e">
-        <v>#N/A</v>
+      <c r="AA9" s="68">
+        <v>1369</v>
+      </c>
+      <c r="AB9" s="67">
+        <v>1288</v>
+      </c>
+      <c r="AC9" s="67">
+        <v>1221</v>
       </c>
       <c r="AD9" s="18" t="e">
         <v>#N/A</v>
@@ -76298,7 +76200,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="25"/>
       <c r="B10" s="25"/>
       <c r="C10" s="16" t="s">
@@ -76368,13 +76270,13 @@
         <v>21.742808798646362</v>
       </c>
       <c r="AA10" s="54">
-        <v>-9.0340514246004169</v>
+        <v>-4.864489228630994</v>
       </c>
       <c r="AB10" s="54">
-        <v>-2.5974025974025974</v>
-      </c>
-      <c r="AC10" s="7" t="e">
-        <v>#N/A</v>
+        <v>-5.9167275383491598</v>
+      </c>
+      <c r="AC10" s="54">
+        <v>-5.2018633540372674</v>
       </c>
       <c r="AD10" s="7" t="e">
         <v>#N/A</v>
@@ -76383,7 +76285,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="1">
         <v>131</v>
       </c>
@@ -76394,10 +76296,10 @@
         <v>166</v>
       </c>
       <c r="D11" s="24">
-        <v>46282.356180555558</v>
+        <v>46315.356747685182</v>
       </c>
       <c r="E11" s="23">
-        <v>46315.356180555566</v>
+        <v>46322.356747685175</v>
       </c>
       <c r="F11" s="48" t="s">
         <v>168</v>
@@ -76459,17 +76361,17 @@
       <c r="Y11" s="13">
         <v>1252</v>
       </c>
-      <c r="Z11" s="67">
+      <c r="Z11" s="62">
         <v>1256</v>
       </c>
-      <c r="AA11" s="67">
+      <c r="AA11" s="62">
         <v>1267</v>
       </c>
-      <c r="AB11" s="67">
-        <v>1271</v>
-      </c>
-      <c r="AC11" s="13" t="e">
-        <v>#N/A</v>
+      <c r="AB11" s="66">
+        <v>1280</v>
+      </c>
+      <c r="AC11" s="65">
+        <v>1280</v>
       </c>
       <c r="AD11" s="13" t="e">
         <v>#N/A</v>
@@ -76478,7 +76380,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6">
         <v>133</v>
       </c>
@@ -76489,10 +76391,10 @@
         <v>166</v>
       </c>
       <c r="D12" s="21">
-        <v>46289.419166666667</v>
+        <v>46315.356828703705</v>
       </c>
       <c r="E12" s="20">
-        <v>46315.419166666659</v>
+        <v>46322.356828703705</v>
       </c>
       <c r="F12" s="47" t="s">
         <v>165</v>
@@ -76563,8 +76465,8 @@
       <c r="AB12" s="59">
         <v>-2.0935100000000002</v>
       </c>
-      <c r="AC12" s="4" t="e">
-        <v>#N/A</v>
+      <c r="AC12" s="64">
+        <v>-0.21382999999999999</v>
       </c>
       <c r="AD12" s="4" t="e">
         <v>#N/A</v>
@@ -76573,7 +76475,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:34" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A13" s="25">
         <v>13</v>
       </c>
@@ -76690,10 +76592,10 @@
       <c r="S14" s="36"/>
       <c r="T14" s="36"/>
       <c r="U14" s="36"/>
-      <c r="V14" s="68"/>
-      <c r="W14" s="68"/>
-      <c r="X14" s="68"/>
-      <c r="Y14" s="68"/>
+      <c r="V14" s="63"/>
+      <c r="W14" s="63"/>
+      <c r="X14" s="63"/>
+      <c r="Y14" s="63"/>
       <c r="Z14" s="36"/>
       <c r="AA14" s="36"/>
       <c r="AB14" s="36"/>
@@ -77277,13 +77179,13 @@
       <c r="AA22" s="13">
         <v>-10</v>
       </c>
-      <c r="AB22" s="67">
+      <c r="AB22" s="62">
         <v>133</v>
       </c>
-      <c r="AC22" s="67">
+      <c r="AC22" s="62">
         <v>29</v>
       </c>
-      <c r="AD22" s="66" t="e">
+      <c r="AD22" s="61" t="e">
         <v>#N/A</v>
       </c>
       <c r="AH22" t="s">
@@ -77378,7 +77280,7 @@
       <c r="AC23" s="12">
         <v>78</v>
       </c>
-      <c r="AD23" s="66" t="e">
+      <c r="AD23" s="61" t="e">
         <v>#N/A</v>
       </c>
       <c r="AH23" t="s">
@@ -77705,7 +77607,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="28" spans="1:34" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A28" s="10"/>
       <c r="B28" s="10"/>
       <c r="C28" s="10"/>
@@ -77731,18 +77633,18 @@
       <c r="U28" s="9"/>
       <c r="V28" s="9"/>
       <c r="W28" s="9"/>
-      <c r="X28" s="36"/>
-      <c r="Y28" s="36"/>
-      <c r="Z28" s="36"/>
-      <c r="AA28" s="36"/>
-      <c r="AB28" s="36"/>
-      <c r="AC28" s="36"/>
+      <c r="X28" s="9"/>
+      <c r="Y28" s="9"/>
+      <c r="Z28" s="9"/>
+      <c r="AA28" s="9"/>
+      <c r="AB28" s="9"/>
+      <c r="AC28" s="9"/>
       <c r="AD28" s="9"/>
       <c r="AH28" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="29" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>101</v>
       </c>
@@ -77812,22 +77714,22 @@
       <c r="W29" s="7">
         <v>-0.16849</v>
       </c>
-      <c r="X29" s="65">
+      <c r="X29" s="28">
         <v>0.82882999999999996</v>
       </c>
-      <c r="Y29" s="64">
+      <c r="Y29" s="28">
         <v>0.14272000000000001</v>
       </c>
-      <c r="Z29" s="64">
+      <c r="Z29" s="28">
         <v>0.23150000000000001</v>
       </c>
-      <c r="AA29" s="64">
+      <c r="AA29" s="28">
         <v>0.23271</v>
       </c>
-      <c r="AB29" s="64">
+      <c r="AB29" s="28">
         <v>6.3759999999999997E-2</v>
       </c>
-      <c r="AC29" s="64">
+      <c r="AC29" s="28">
         <v>0.66256000000000004</v>
       </c>
       <c r="AD29" s="7" t="e">
@@ -77837,7 +77739,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>111</v>
       </c>
@@ -77907,22 +77809,22 @@
       <c r="W30" s="7">
         <v>75.617800000000003</v>
       </c>
-      <c r="X30" s="63">
+      <c r="X30" s="7">
         <v>76.179199999999994</v>
       </c>
-      <c r="Y30" s="62">
+      <c r="Y30" s="7">
         <v>76.222499999999997</v>
       </c>
-      <c r="Z30" s="62">
+      <c r="Z30" s="7">
         <v>76.332099999999997</v>
       </c>
-      <c r="AA30" s="62">
+      <c r="AA30" s="7">
         <v>76.440899999999999</v>
       </c>
-      <c r="AB30" s="62">
+      <c r="AB30" s="7">
         <v>76.418400000000005</v>
       </c>
-      <c r="AC30" s="61">
+      <c r="AC30" s="28">
         <v>76.850399999999993</v>
       </c>
       <c r="AD30" s="7" t="e">
@@ -77938,7 +77840,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="31" spans="1:34" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A31" s="6">
         <v>109</v>
       </c>
@@ -85245,213 +85147,157 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G9:AD9">
-    <cfRule type="cellIs" dxfId="206" priority="207" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="expression" dxfId="206" priority="205">
+      <formula>ISERROR(G9)</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="205" priority="206" stopIfTrue="1" operator="lessThan">
+      <formula>F9</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="204" priority="207" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>F9</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G9:AD9">
-    <cfRule type="cellIs" dxfId="205" priority="206" stopIfTrue="1" operator="lessThan">
-      <formula>F9</formula>
+  <conditionalFormatting sqref="G10:AD10">
+    <cfRule type="expression" dxfId="203" priority="202">
+      <formula>ISERROR(G10)</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G9:AD9">
-    <cfRule type="expression" dxfId="204" priority="205">
-      <formula>ISERROR(G9)</formula>
+    <cfRule type="cellIs" dxfId="202" priority="203" stopIfTrue="1" operator="lessThan">
+      <formula>0</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G10:AD10">
-    <cfRule type="cellIs" dxfId="203" priority="204" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="201" priority="204" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G10:AD10">
-    <cfRule type="cellIs" dxfId="202" priority="203" stopIfTrue="1" operator="lessThan">
+  <conditionalFormatting sqref="G11:AD11">
+    <cfRule type="expression" dxfId="200" priority="199">
+      <formula>ISERROR(G11)</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="199" priority="200" stopIfTrue="1" operator="lessThan">
+      <formula>F11</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="198" priority="201" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>F11</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G12:AD12">
+    <cfRule type="expression" dxfId="197" priority="196">
+      <formula>ISERROR(G12)</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="196" priority="197" stopIfTrue="1" operator="lessThan">
+      <formula>0</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="195" priority="198" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G10:AD10">
-    <cfRule type="expression" dxfId="201" priority="202">
-      <formula>ISERROR(G10)</formula>
+  <conditionalFormatting sqref="G13:AD13">
+    <cfRule type="expression" dxfId="194" priority="193">
+      <formula>ISERROR(G13)</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G11:AD11">
-    <cfRule type="cellIs" dxfId="200" priority="201" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>F11</formula>
+    <cfRule type="cellIs" dxfId="193" priority="194" stopIfTrue="1" operator="greaterThan">
+      <formula>F13</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G11:AD11">
-    <cfRule type="cellIs" dxfId="199" priority="200" stopIfTrue="1" operator="lessThan">
-      <formula>F11</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G11:AD11">
-    <cfRule type="expression" dxfId="198" priority="199">
-      <formula>ISERROR(G11)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G12:AD12">
-    <cfRule type="cellIs" dxfId="197" priority="198" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G12:AD12">
-    <cfRule type="cellIs" dxfId="196" priority="197" stopIfTrue="1" operator="lessThan">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G12:AD12">
-    <cfRule type="expression" dxfId="195" priority="196">
-      <formula>ISERROR(G12)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G13:AD13">
-    <cfRule type="cellIs" dxfId="194" priority="195" stopIfTrue="1" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="192" priority="195" stopIfTrue="1" operator="lessThanOrEqual">
       <formula>F13</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G13:AD13">
-    <cfRule type="cellIs" dxfId="193" priority="194" stopIfTrue="1" operator="greaterThan">
-      <formula>F13</formula>
+  <conditionalFormatting sqref="G16:AD16">
+    <cfRule type="expression" dxfId="191" priority="190">
+      <formula>ISERROR(G16)</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G13:AD13">
-    <cfRule type="expression" dxfId="192" priority="193">
-      <formula>ISERROR(G13)</formula>
+    <cfRule type="cellIs" dxfId="190" priority="191" stopIfTrue="1" operator="lessThan">
+      <formula>F16</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G16:AD16">
-    <cfRule type="cellIs" dxfId="191" priority="192" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="189" priority="192" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>F16</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G16:AD16">
-    <cfRule type="cellIs" dxfId="190" priority="191" stopIfTrue="1" operator="lessThan">
-      <formula>F16</formula>
+  <conditionalFormatting sqref="G17:AD17">
+    <cfRule type="expression" dxfId="188" priority="187">
+      <formula>ISERROR(G17)</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G16:AD16">
-    <cfRule type="expression" dxfId="189" priority="190">
-      <formula>ISERROR(G16)</formula>
+    <cfRule type="cellIs" dxfId="187" priority="188" stopIfTrue="1" operator="greaterThan">
+      <formula>F17</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G17:AD17">
-    <cfRule type="cellIs" dxfId="188" priority="189" stopIfTrue="1" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="186" priority="189" stopIfTrue="1" operator="lessThanOrEqual">
       <formula>F17</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G17:AD17">
-    <cfRule type="cellIs" dxfId="187" priority="188" stopIfTrue="1" operator="greaterThan">
-      <formula>F17</formula>
+  <conditionalFormatting sqref="G18:AD18">
+    <cfRule type="expression" dxfId="185" priority="184">
+      <formula>ISERROR(G18)</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G17:AD17">
-    <cfRule type="expression" dxfId="186" priority="187">
-      <formula>ISERROR(G17)</formula>
+    <cfRule type="cellIs" dxfId="184" priority="185" stopIfTrue="1" operator="lessThan">
+      <formula>F18</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G18:AD18">
-    <cfRule type="cellIs" dxfId="185" priority="186" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="183" priority="186" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>F18</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G18:AD18">
-    <cfRule type="cellIs" dxfId="184" priority="185" stopIfTrue="1" operator="lessThan">
-      <formula>F18</formula>
+  <conditionalFormatting sqref="G19:AD19">
+    <cfRule type="expression" dxfId="182" priority="181">
+      <formula>ISERROR(G19)</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G18:AD18">
-    <cfRule type="expression" dxfId="183" priority="184">
-      <formula>ISERROR(G18)</formula>
+    <cfRule type="cellIs" dxfId="181" priority="182" stopIfTrue="1" operator="lessThan">
+      <formula>F19</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G19:AD19">
-    <cfRule type="cellIs" dxfId="182" priority="183" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="180" priority="183" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>F19</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G19:AD19">
-    <cfRule type="cellIs" dxfId="181" priority="182" stopIfTrue="1" operator="lessThan">
-      <formula>F19</formula>
+  <conditionalFormatting sqref="G22:AD22">
+    <cfRule type="expression" dxfId="179" priority="178">
+      <formula>ISERROR(G22)</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G19:AD19">
-    <cfRule type="expression" dxfId="180" priority="181">
-      <formula>ISERROR(G19)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G22:AD22">
-    <cfRule type="cellIs" dxfId="179" priority="180" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G22:AD22">
     <cfRule type="cellIs" dxfId="178" priority="179" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G22:AD22">
-    <cfRule type="expression" dxfId="177" priority="178">
-      <formula>ISERROR(G22)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G23:AD23">
-    <cfRule type="cellIs" dxfId="176" priority="177" stopIfTrue="1" operator="lessThanOrEqual">
+    <cfRule type="cellIs" dxfId="177" priority="180" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G23:AD23">
+    <cfRule type="expression" dxfId="176" priority="175">
+      <formula>ISERROR(G23)</formula>
+    </cfRule>
     <cfRule type="cellIs" dxfId="175" priority="176" stopIfTrue="1" operator="greaterThan">
       <formula>0</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G23:AD23">
-    <cfRule type="expression" dxfId="174" priority="175">
-      <formula>ISERROR(G23)</formula>
+    <cfRule type="cellIs" dxfId="174" priority="177" stopIfTrue="1" operator="lessThanOrEqual">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G24:AD24">
-    <cfRule type="cellIs" dxfId="173" priority="174" stopIfTrue="1" operator="lessThanOrEqual">
+    <cfRule type="expression" dxfId="173" priority="172">
+      <formula>ISERROR(G24)</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="172" priority="173" stopIfTrue="1" operator="greaterThan">
+      <formula>F24</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="171" priority="174" stopIfTrue="1" operator="lessThanOrEqual">
       <formula>F24</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G24:AD24">
-    <cfRule type="cellIs" dxfId="172" priority="173" stopIfTrue="1" operator="greaterThan">
-      <formula>F24</formula>
+  <conditionalFormatting sqref="G25:AD25">
+    <cfRule type="expression" dxfId="170" priority="169">
+      <formula>ISERROR(G25)</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G24:AD24">
-    <cfRule type="expression" dxfId="171" priority="172">
-      <formula>ISERROR(G24)</formula>
+    <cfRule type="cellIs" dxfId="169" priority="170" stopIfTrue="1" operator="lessThan">
+      <formula>F25</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G25:AD25">
-    <cfRule type="cellIs" dxfId="170" priority="171" stopIfTrue="1" operator="greaterThanOrEqual">
+    <cfRule type="cellIs" dxfId="168" priority="171" stopIfTrue="1" operator="greaterThanOrEqual">
       <formula>F25</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G25:AD25">
-    <cfRule type="cellIs" dxfId="169" priority="170" stopIfTrue="1" operator="lessThan">
-      <formula>F25</formula>
+  <conditionalFormatting sqref="G26:AD26">
+    <cfRule type="expression" dxfId="167" priority="166">
+      <formula>ISERROR(G26)</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G25:AD25">
-    <cfRule type="expression" dxfId="168" priority="169">
-      <formula>ISERROR(G25)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G26:AD26">
-    <cfRule type="cellIs" dxfId="167" priority="168" stopIfTrue="1" operator="greaterThanOrEqual">
-      <formula>0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G26:AD26">
     <cfRule type="cellIs" dxfId="166" priority="167" stopIfTrue="1" operator="lessThan">
       <formula>0</formula>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G26:AD26">
-    <cfRule type="expression" dxfId="165" priority="166">
-      <formula>ISERROR(G26)</formula>
+    <cfRule type="cellIs" dxfId="165" priority="168" stopIfTrue="1" operator="greaterThanOrEqual">
+      <formula>0</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G29:AD29">
@@ -86283,83 +86129,83 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="AH3:AH96" xr:uid="{C1C4EC35-DC8A-4C87-8226-D605F47849DA}">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="AH3:AH96" xr:uid="{88E6C84E-F064-4FC3-A541-ECE5120D7698}">
       <formula1>FormatOptions</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" display="https://fred.stlouisfed.org/series/MPCTXXXXS" xr:uid="{CF562D95-77DF-463A-81CC-636269FBA42E}"/>
-    <hyperlink ref="C5" r:id="rId2" display="https://fred.stlouisfed.org/series/TLPRVCONS" xr:uid="{8C494690-1C0A-4EA1-B518-334AFC20BDB1}"/>
-    <hyperlink ref="C6" r:id="rId3" display="https://fred.stlouisfed.org/series/TLRESCONS" xr:uid="{4606C91C-70A9-40C6-938A-685BF93775E3}"/>
-    <hyperlink ref="C7" r:id="rId4" display="https://fred.stlouisfed.org/series/TLHWYCONS" xr:uid="{634DE402-8226-48EA-A6C9-72424EB7A1A2}"/>
-    <hyperlink ref="C8" r:id="rId5" display="https://fred.stlouisfed.org/series/HSN1F" xr:uid="{F7187EBE-4443-4DF1-ABA4-A814D18C4730}"/>
-    <hyperlink ref="C9" r:id="rId6" display="https://fred.stlouisfed.org/series/HOUST" xr:uid="{3D90EA5C-6EE1-4ACA-8266-9953FCD68BE6}"/>
-    <hyperlink ref="C11" r:id="rId7" display="https://fred.stlouisfed.org/series/UNDCONTSA" xr:uid="{FF7E682F-76C4-4CAE-B72B-C7E0382A91B6}"/>
-    <hyperlink ref="C12" r:id="rId8" display="https://fred.stlouisfed.org/series/PERMIT" xr:uid="{360B60BB-D93C-412B-8010-D85542BEEB74}"/>
-    <hyperlink ref="C13" r:id="rId9" display="https://fred.stlouisfed.org/series/MORTGAGE30US" xr:uid="{28D477DE-31FF-4CF6-88FC-F349B761E769}"/>
-    <hyperlink ref="C16" r:id="rId10" display="https://fred.stlouisfed.org/series/ALTSALES" xr:uid="{62774A1B-E813-462D-A3C8-B54F32DD75A7}"/>
-    <hyperlink ref="C17" r:id="rId11" display="https://fred.stlouisfed.org/series/AISRSA" xr:uid="{4B9D3D16-05A1-4F1B-8986-CC2AFD1124FB}"/>
-    <hyperlink ref="C18" r:id="rId12" display="https://fred.stlouisfed.org/series/DAUTOSAAR" xr:uid="{E19626E5-F306-4F83-96B4-0293E9399306}"/>
-    <hyperlink ref="C19" r:id="rId13" display="https://fred.stlouisfed.org/series/DAUPSA" xr:uid="{E18C780B-6D16-45F6-B2C6-4E96265D85C6}"/>
-    <hyperlink ref="C23" r:id="rId14" display="https://fred.stlouisfed.org/series/UNEMPLOY" xr:uid="{2A27EF66-83BB-4B10-BF17-206F6E700666}"/>
-    <hyperlink ref="C24" r:id="rId15" display="https://fred.stlouisfed.org/series/UNRATE" xr:uid="{FA49F51E-6348-49EF-960B-72E9CB0BC8A9}"/>
-    <hyperlink ref="C25" r:id="rId16" display="https://fred.stlouisfed.org/series/AWHNONAG" xr:uid="{A3BEF371-A6F1-4A68-A332-0A226320B24E}"/>
-    <hyperlink ref="C26" r:id="rId17" display="https://fred.stlouisfed.org/series/CLF16OV" xr:uid="{FC53E953-1958-42B5-BEB5-A0802E39B40D}"/>
-    <hyperlink ref="C29" r:id="rId18" display="https://fred.stlouisfed.org/series/INDPRO" xr:uid="{D012F5A8-BFF2-41DD-8E3D-874A47E9721C}"/>
-    <hyperlink ref="C30" r:id="rId19" display="https://fred.stlouisfed.org/series/TCU" xr:uid="{6FBDBF95-0FE4-4D21-85EC-6BE7C0F96FF4}"/>
-    <hyperlink ref="C31" r:id="rId20" display="https://fred.stlouisfed.org/series/AMTMNO" xr:uid="{2A326159-DD63-4C31-8041-A13ACA187AC4}"/>
-    <hyperlink ref="C32" r:id="rId21" display="https://fred.stlouisfed.org/series/DGORDER" xr:uid="{D9E2DDA6-AE91-4AD5-ACB1-A3FA3172BD80}"/>
-    <hyperlink ref="C33" r:id="rId22" display="https://fred.stlouisfed.org/series/ANXAVS" xr:uid="{6729710C-1955-46FB-9A36-AD1447C4916A}"/>
-    <hyperlink ref="C36" r:id="rId23" display="https://fred.stlouisfed.org/series/BUSINV" xr:uid="{D4B9F793-7BF2-4540-AA71-73E369FDB0DD}"/>
-    <hyperlink ref="C37" r:id="rId24" display="https://fred.stlouisfed.org/series/ISRATIO" xr:uid="{3635BEF7-AD8F-4B7D-AC36-756A48933CB5}"/>
-    <hyperlink ref="C38" r:id="rId25" display="https://fred.stlouisfed.org/series/RETAILMPCIMSA" xr:uid="{44BC184D-1C05-4539-BAE0-803E418F78B1}"/>
-    <hyperlink ref="C39" r:id="rId26" display="https://fred.stlouisfed.org/series/ACNGTI" xr:uid="{E83143F4-7734-4A90-8913-BDCF58854D25}"/>
-    <hyperlink ref="C42" r:id="rId27" display="https://fred.stlouisfed.org/series/CPIAUCSL" xr:uid="{4754EE6A-75E0-4F28-982B-1A2AF52D284A}"/>
-    <hyperlink ref="C43" r:id="rId28" display="https://fred.stlouisfed.org/series/CPIFABSL" xr:uid="{B5DBBAEC-9FA2-4228-B3B0-B292FAA6BB56}"/>
-    <hyperlink ref="C44" r:id="rId29" display="https://fred.stlouisfed.org/series/CPIENGSL" xr:uid="{0BF3E961-627C-42D9-96B1-57332FE72031}"/>
-    <hyperlink ref="C45" r:id="rId30" display="https://fred.stlouisfed.org/series/CPILFESL" xr:uid="{23633F4C-CD5D-4692-B2EE-B4D9D2ACBCBE}"/>
-    <hyperlink ref="C48" r:id="rId31" display="https://fred.stlouisfed.org/series/WPUFD49207" xr:uid="{D114408D-9660-49D9-861F-8113E471CB40}"/>
-    <hyperlink ref="C49" r:id="rId32" display="https://fred.stlouisfed.org/series/WPSID61" xr:uid="{275E4CF3-8879-4989-8FE4-13EDAAD37ABA}"/>
-    <hyperlink ref="C50" r:id="rId33" display="https://fred.stlouisfed.org/series/PRAWMINDEXM" xr:uid="{7D80E8EA-7B77-4AC9-8F0D-F5DA1F312DBE}"/>
-    <hyperlink ref="C52" r:id="rId34" display="https://fred.stlouisfed.org/series/DCOILWTICO" xr:uid="{AAB67C0A-B21A-4D58-B50B-0C4AFB228547}"/>
-    <hyperlink ref="C53" r:id="rId35" display="https://fred.stlouisfed.org/series/DCOILBRENTEU" xr:uid="{9A86CB8B-8C04-4E35-A7E2-54579C53E91F}"/>
-    <hyperlink ref="C54" r:id="rId36" display="https://fred.stlouisfed.org/series/DHHNGSP" xr:uid="{2C16E224-C3BD-4137-8FCD-9594D9D5B585}"/>
-    <hyperlink ref="C58" r:id="rId37" display="https://fred.stlouisfed.org/series/DHHNGSP" xr:uid="{3F262E2D-EA22-464F-9DB9-BA59AABC28DB}"/>
-    <hyperlink ref="C59" r:id="rId38" display="https://fred.stlouisfed.org/series/PI" xr:uid="{21569B9C-C2AD-4E0F-BAFD-7CE64C33FB90}"/>
-    <hyperlink ref="C60" r:id="rId39" display="https://fred.stlouisfed.org/series/DSPI" xr:uid="{61869BC9-BAF4-4DAC-B141-86F531C90736}"/>
-    <hyperlink ref="C61" r:id="rId40" display="https://fred.stlouisfed.org/series/A229RX0" xr:uid="{27E4895C-EB1B-4CE7-8DCD-0B774804C245}"/>
-    <hyperlink ref="C62" r:id="rId41" display="https://fred.stlouisfed.org/series/PSAVERT" xr:uid="{A92B07B3-36C5-41A3-B2CF-0993D31B8038}"/>
-    <hyperlink ref="C63" r:id="rId42" display="https://fred.stlouisfed.org/series/PCE" xr:uid="{C52F2B8C-278E-41EC-B982-3FDCCC563887}"/>
-    <hyperlink ref="C64" r:id="rId43" display="https://fred.stlouisfed.org/series/PCEC96" xr:uid="{7BE8C9E1-F701-488D-8ACC-D9A0DDF6A86B}"/>
-    <hyperlink ref="C65" r:id="rId44" display="https://fred.stlouisfed.org/series/MRTSMPCSM44X72USS" xr:uid="{96571A34-126C-4D5C-B192-6018B3347B28}"/>
-    <hyperlink ref="C66" r:id="rId45" display="https://fred.stlouisfed.org/series/TOTALSL" xr:uid="{441D994A-6343-43BC-B404-00268E8A132D}"/>
-    <hyperlink ref="C67" r:id="rId46" display="https://fred.stlouisfed.org/series/PCEND" xr:uid="{6A732520-3DBD-4885-BA1E-97C9AFD5BFEE}"/>
-    <hyperlink ref="C68" r:id="rId47" display="https://fred.stlouisfed.org/series/A22BVS" xr:uid="{C60F5F87-72DB-4C08-8BB4-C055A8D0B0BA}"/>
-    <hyperlink ref="C71" r:id="rId48" display="https://fred.stlouisfed.org/series/M1SL" xr:uid="{C33366E6-16B8-4A32-B908-D27298DFB7B9}"/>
-    <hyperlink ref="C72" r:id="rId49" display="https://fred.stlouisfed.org/series/M2SL" xr:uid="{2203B1FB-5C4B-4FCC-A707-407631381606}"/>
-    <hyperlink ref="C74" r:id="rId50" display="https://fred.stlouisfed.org/series/DTB3" xr:uid="{D937E583-65DE-4D9E-9717-1C3F3EBFCCD2}"/>
-    <hyperlink ref="C75" r:id="rId51" display="https://fred.stlouisfed.org/series/DPRIME" xr:uid="{7E883408-6D78-47B8-BCAA-45F649C4DEC0}"/>
-    <hyperlink ref="C76" r:id="rId52" display="https://fred.stlouisfed.org/series/DGS10" xr:uid="{6D73C1BC-9303-4BA6-B122-C19894E23F67}"/>
-    <hyperlink ref="C79" r:id="rId53" display="https://fred.stlouisfed.org/series/DFII10" xr:uid="{8FC678B4-A334-4987-A4F0-7B22956B50B9}"/>
-    <hyperlink ref="C80" r:id="rId54" display="https://fred.stlouisfed.org/series/DGS30" xr:uid="{292CF90C-3D97-424F-BC2B-7CE99BB00206}"/>
-    <hyperlink ref="C82" r:id="rId55" display="https://fred.stlouisfed.org/series/DEXUSEU" xr:uid="{811824CA-1C69-4548-B771-1C5EFF998A60}"/>
-    <hyperlink ref="C83" r:id="rId56" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{0057E3E9-4010-4CC3-9970-AF8E9F70AFB4}"/>
-    <hyperlink ref="C87" r:id="rId57" display="https://fred.stlouisfed.org/series/GDPC1" xr:uid="{6FD6C9EC-B7EC-4567-80C3-5B54C3A7F39C}"/>
-    <hyperlink ref="C88" r:id="rId58" display="https://fred.stlouisfed.org/series/GDP" xr:uid="{0B9EA38B-FF63-4491-B0A2-5F006EE61A49}"/>
-    <hyperlink ref="C89" r:id="rId59" display="https://fred.stlouisfed.org/series/PCEDG" xr:uid="{E012DCC7-02BD-4B94-BB81-EFA086DC9F35}"/>
-    <hyperlink ref="C90" r:id="rId60" display="https://fred.stlouisfed.org/series/PNFIC1" xr:uid="{B318CB31-CE2A-40E2-8BA4-78CFC38B38CF}"/>
-    <hyperlink ref="C91" r:id="rId61" display="https://fred.stlouisfed.org/series/PRFIC1" xr:uid="{B8DDA874-1E07-4B0F-B56B-A706F6F7964A}"/>
-    <hyperlink ref="C92" r:id="rId62" display="https://fred.stlouisfed.org/series/CBI" xr:uid="{2629D423-F984-45E8-8100-4F414E965B21}"/>
-    <hyperlink ref="C93" r:id="rId63" display="https://fred.stlouisfed.org/series/NETEXC" xr:uid="{0443940F-9918-43E0-9C87-8E14D6FB970F}"/>
-    <hyperlink ref="C94" r:id="rId64" display="https://fred.stlouisfed.org/series/IEABC" xr:uid="{FF63A1A7-6D7D-4CF1-B8B8-639A144D2795}"/>
-    <hyperlink ref="C73" r:id="rId65" display="https://fred.stlouisfed.org/series/BOPGSTB" xr:uid="{CC908B37-E115-4BF9-BA2B-C868CF63A3EF}"/>
-    <hyperlink ref="C95" r:id="rId66" display="https://fred.stlouisfed.org/series/GCEC1" xr:uid="{7AD691CE-D4C5-4F5B-8C28-D5D144374A94}"/>
-    <hyperlink ref="C96" r:id="rId67" display="https://fred.stlouisfed.org/series/EVACANTUSQ176N" xr:uid="{09EF3F06-48BA-4537-8C90-A2561AE81204}"/>
-    <hyperlink ref="C81" r:id="rId68" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{CADAA938-7E05-4E34-B0E8-23D9412E1025}"/>
-    <hyperlink ref="C78" r:id="rId69" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{E6D706A3-B3BF-445A-A58C-4DD3A4C3C1CF}"/>
-    <hyperlink ref="C77" r:id="rId70" display="https://fred.stlouisfed.org/series/DGS10" xr:uid="{E1A72690-BF2C-430A-BA17-54A478B1D95A}"/>
-    <hyperlink ref="C51" r:id="rId71" display="https://fred.stlouisfed.org/series/PRAWMINDEXM" xr:uid="{D79B4C81-B8AF-4791-A538-EA979757ACBC}"/>
-    <hyperlink ref="C22" r:id="rId72" display="https://fred.stlouisfed.org/series/PAYEMS" xr:uid="{F823A10C-C3AD-4D41-BE55-DE5F2B1BC197}"/>
+    <hyperlink ref="C4" r:id="rId1" display="https://fred.stlouisfed.org/series/MPCTXXXXS" xr:uid="{7FE01B38-A3AD-4D57-965B-C523DD5E559B}"/>
+    <hyperlink ref="C5" r:id="rId2" display="https://fred.stlouisfed.org/series/TLPRVCONS" xr:uid="{964DA74E-E517-4930-A82D-DCD1F8D115E5}"/>
+    <hyperlink ref="C6" r:id="rId3" display="https://fred.stlouisfed.org/series/TLRESCONS" xr:uid="{5641A39B-6657-4681-9736-4C25135605FB}"/>
+    <hyperlink ref="C7" r:id="rId4" display="https://fred.stlouisfed.org/series/TLHWYCONS" xr:uid="{2A7E7C11-884B-4B9E-A240-9DF70B084BD7}"/>
+    <hyperlink ref="C8" r:id="rId5" display="https://fred.stlouisfed.org/series/HSN1F" xr:uid="{A9D8F207-9447-40D0-8C37-7A13276BC593}"/>
+    <hyperlink ref="C9" r:id="rId6" display="https://fred.stlouisfed.org/series/HOUST" xr:uid="{963A071D-2D6D-4A59-A27E-071FCFCEC865}"/>
+    <hyperlink ref="C11" r:id="rId7" display="https://fred.stlouisfed.org/series/UNDCONTSA" xr:uid="{E383E6F0-7CB8-4B4F-90D4-A04D33B07F45}"/>
+    <hyperlink ref="C12" r:id="rId8" display="https://fred.stlouisfed.org/series/PERMIT" xr:uid="{3B856B7F-91AF-4166-9533-A99C6CF66649}"/>
+    <hyperlink ref="C13" r:id="rId9" display="https://fred.stlouisfed.org/series/MORTGAGE30US" xr:uid="{0A124A9B-8D32-420B-962F-CF7BA73D921D}"/>
+    <hyperlink ref="C16" r:id="rId10" display="https://fred.stlouisfed.org/series/ALTSALES" xr:uid="{3B8E6461-79C0-4F65-96C3-8C95DB9CDF69}"/>
+    <hyperlink ref="C17" r:id="rId11" display="https://fred.stlouisfed.org/series/AISRSA" xr:uid="{98C603F5-3CD7-40ED-83A5-C2BFF4EA9671}"/>
+    <hyperlink ref="C18" r:id="rId12" display="https://fred.stlouisfed.org/series/DAUTOSAAR" xr:uid="{373D6F81-B00A-423A-9D01-BFD93895913B}"/>
+    <hyperlink ref="C19" r:id="rId13" display="https://fred.stlouisfed.org/series/DAUPSA" xr:uid="{D15220AD-AC60-46EB-912E-1EF944F661DB}"/>
+    <hyperlink ref="C23" r:id="rId14" display="https://fred.stlouisfed.org/series/UNEMPLOY" xr:uid="{B5F427E9-38C1-4D6E-BF8F-249E264EC417}"/>
+    <hyperlink ref="C24" r:id="rId15" display="https://fred.stlouisfed.org/series/UNRATE" xr:uid="{77498871-04FE-4760-97FA-0443C59AB29E}"/>
+    <hyperlink ref="C25" r:id="rId16" display="https://fred.stlouisfed.org/series/AWHNONAG" xr:uid="{8532A332-DBB3-4ABF-B0A9-71E35CD31CC8}"/>
+    <hyperlink ref="C26" r:id="rId17" display="https://fred.stlouisfed.org/series/CLF16OV" xr:uid="{BF4A67B3-2B9E-4810-B579-1ADC6ED099E5}"/>
+    <hyperlink ref="C29" r:id="rId18" display="https://fred.stlouisfed.org/series/INDPRO" xr:uid="{31C373F4-8FFF-400C-B3A0-C8759B7ADDD7}"/>
+    <hyperlink ref="C30" r:id="rId19" display="https://fred.stlouisfed.org/series/TCU" xr:uid="{52F33519-107A-4C0C-991B-0D2845F0C384}"/>
+    <hyperlink ref="C31" r:id="rId20" display="https://fred.stlouisfed.org/series/AMTMNO" xr:uid="{0046E6F3-C9C3-4F73-A235-A25E5D49DF8C}"/>
+    <hyperlink ref="C32" r:id="rId21" display="https://fred.stlouisfed.org/series/DGORDER" xr:uid="{03227960-78A4-463A-A845-E22B47327E0C}"/>
+    <hyperlink ref="C33" r:id="rId22" display="https://fred.stlouisfed.org/series/ANXAVS" xr:uid="{5B31B5FC-BDFE-48A6-BA01-F758058970C3}"/>
+    <hyperlink ref="C36" r:id="rId23" display="https://fred.stlouisfed.org/series/BUSINV" xr:uid="{F9D91AD2-94B9-43ED-9548-59AE5387FC68}"/>
+    <hyperlink ref="C37" r:id="rId24" display="https://fred.stlouisfed.org/series/ISRATIO" xr:uid="{FE545E5D-C4B6-46C4-AB9F-5B0CB03E5464}"/>
+    <hyperlink ref="C38" r:id="rId25" display="https://fred.stlouisfed.org/series/RETAILMPCIMSA" xr:uid="{E8027F13-EBE1-4273-8B7E-D7264C848DDB}"/>
+    <hyperlink ref="C39" r:id="rId26" display="https://fred.stlouisfed.org/series/ACNGTI" xr:uid="{42556524-E306-4BFF-BE01-15BDC05D3F94}"/>
+    <hyperlink ref="C42" r:id="rId27" display="https://fred.stlouisfed.org/series/CPIAUCSL" xr:uid="{D6BD34AD-045F-47C5-8468-9E2691214C80}"/>
+    <hyperlink ref="C43" r:id="rId28" display="https://fred.stlouisfed.org/series/CPIFABSL" xr:uid="{25840D65-2EE5-49F1-96FD-A3A83639580D}"/>
+    <hyperlink ref="C44" r:id="rId29" display="https://fred.stlouisfed.org/series/CPIENGSL" xr:uid="{48819B20-1AC4-456B-BABD-FFC1D8811050}"/>
+    <hyperlink ref="C45" r:id="rId30" display="https://fred.stlouisfed.org/series/CPILFESL" xr:uid="{F0D76998-766A-400F-B9F4-C5090E4B4D64}"/>
+    <hyperlink ref="C48" r:id="rId31" display="https://fred.stlouisfed.org/series/WPUFD49207" xr:uid="{F5FA2F6A-7063-4E76-A0AA-752BFB9A2381}"/>
+    <hyperlink ref="C49" r:id="rId32" display="https://fred.stlouisfed.org/series/WPSID61" xr:uid="{3C9EA920-666C-47A6-BD2F-B1B1F394334B}"/>
+    <hyperlink ref="C50" r:id="rId33" display="https://fred.stlouisfed.org/series/PRAWMINDEXM" xr:uid="{755F095A-4FAC-494C-9590-E0A8516EB873}"/>
+    <hyperlink ref="C52" r:id="rId34" display="https://fred.stlouisfed.org/series/DCOILWTICO" xr:uid="{FD90CB8C-6A1F-49DD-ADF1-4FE77EB50725}"/>
+    <hyperlink ref="C53" r:id="rId35" display="https://fred.stlouisfed.org/series/DCOILBRENTEU" xr:uid="{68909A2C-1957-4769-A91C-A290ADA458F6}"/>
+    <hyperlink ref="C54" r:id="rId36" display="https://fred.stlouisfed.org/series/DHHNGSP" xr:uid="{A2538FD1-1EEB-4416-B376-7FC5CA949835}"/>
+    <hyperlink ref="C58" r:id="rId37" display="https://fred.stlouisfed.org/series/DHHNGSP" xr:uid="{E00AB092-68CB-445A-9D48-28908B2BA7B3}"/>
+    <hyperlink ref="C59" r:id="rId38" display="https://fred.stlouisfed.org/series/PI" xr:uid="{DA693AB0-E80C-4F4B-8A89-055240EAB768}"/>
+    <hyperlink ref="C60" r:id="rId39" display="https://fred.stlouisfed.org/series/DSPI" xr:uid="{3FA7B551-F90F-41E7-A525-9CC8DF8A0A16}"/>
+    <hyperlink ref="C61" r:id="rId40" display="https://fred.stlouisfed.org/series/A229RX0" xr:uid="{3AF0D127-26A5-4501-9233-CAF10AB11406}"/>
+    <hyperlink ref="C62" r:id="rId41" display="https://fred.stlouisfed.org/series/PSAVERT" xr:uid="{F8571D3E-8330-4696-A1EE-28C818830989}"/>
+    <hyperlink ref="C63" r:id="rId42" display="https://fred.stlouisfed.org/series/PCE" xr:uid="{03E76F18-EAEB-40C1-8C55-7BD6C0BA8C79}"/>
+    <hyperlink ref="C64" r:id="rId43" display="https://fred.stlouisfed.org/series/PCEC96" xr:uid="{FBA2124B-7C43-40AC-9FDA-6E80AD66FAE7}"/>
+    <hyperlink ref="C65" r:id="rId44" display="https://fred.stlouisfed.org/series/MRTSMPCSM44X72USS" xr:uid="{8D8F07A4-739C-4053-BED1-980B18BB124F}"/>
+    <hyperlink ref="C66" r:id="rId45" display="https://fred.stlouisfed.org/series/TOTALSL" xr:uid="{AF6B8628-BA4E-40E1-9091-461FC44512E5}"/>
+    <hyperlink ref="C67" r:id="rId46" display="https://fred.stlouisfed.org/series/PCEND" xr:uid="{C17F6EEE-A597-4EA5-A5CA-EF6A08DE86F7}"/>
+    <hyperlink ref="C68" r:id="rId47" display="https://fred.stlouisfed.org/series/A22BVS" xr:uid="{9DE336FA-DDEC-41BD-B4A5-F4E9B3201E1D}"/>
+    <hyperlink ref="C71" r:id="rId48" display="https://fred.stlouisfed.org/series/M1SL" xr:uid="{E8092FC1-3BD3-4791-850A-ACF1BBDDA101}"/>
+    <hyperlink ref="C72" r:id="rId49" display="https://fred.stlouisfed.org/series/M2SL" xr:uid="{409F6FEC-3471-4CD1-A095-E451963826BB}"/>
+    <hyperlink ref="C74" r:id="rId50" display="https://fred.stlouisfed.org/series/DTB3" xr:uid="{C282C1F8-9A1E-48C0-9B70-5633368F4EE7}"/>
+    <hyperlink ref="C75" r:id="rId51" display="https://fred.stlouisfed.org/series/DPRIME" xr:uid="{EF653A18-25A3-47DB-9619-6CC165D86CC1}"/>
+    <hyperlink ref="C76" r:id="rId52" display="https://fred.stlouisfed.org/series/DGS10" xr:uid="{0F9B32FC-36CF-4242-B00E-54A99E32D405}"/>
+    <hyperlink ref="C79" r:id="rId53" display="https://fred.stlouisfed.org/series/DFII10" xr:uid="{D8284E1B-44CD-4A99-9920-0A79954597DE}"/>
+    <hyperlink ref="C80" r:id="rId54" display="https://fred.stlouisfed.org/series/DGS30" xr:uid="{76462D74-86DF-4053-91F3-252423DB4A35}"/>
+    <hyperlink ref="C82" r:id="rId55" display="https://fred.stlouisfed.org/series/DEXUSEU" xr:uid="{3C31135F-CF97-49B5-9EBE-47B6BC825FB5}"/>
+    <hyperlink ref="C83" r:id="rId56" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{4EBE0BCB-0013-42BC-8D26-03D99E453B35}"/>
+    <hyperlink ref="C87" r:id="rId57" display="https://fred.stlouisfed.org/series/GDPC1" xr:uid="{BA2A03C1-1A8B-473F-BB60-5416C585C91B}"/>
+    <hyperlink ref="C88" r:id="rId58" display="https://fred.stlouisfed.org/series/GDP" xr:uid="{0D40D6CA-9593-414E-8CEB-A5D591390BB9}"/>
+    <hyperlink ref="C89" r:id="rId59" display="https://fred.stlouisfed.org/series/PCEDG" xr:uid="{887DD5D8-D54A-45F4-AAAA-5B292CFD6730}"/>
+    <hyperlink ref="C90" r:id="rId60" display="https://fred.stlouisfed.org/series/PNFIC1" xr:uid="{2866E896-2C05-463A-9F71-C084426C46A6}"/>
+    <hyperlink ref="C91" r:id="rId61" display="https://fred.stlouisfed.org/series/PRFIC1" xr:uid="{7CEFCBBA-A890-43B2-B8D8-867AD59BF651}"/>
+    <hyperlink ref="C92" r:id="rId62" display="https://fred.stlouisfed.org/series/CBI" xr:uid="{25957A9D-9859-4425-B336-A88CA651DBFE}"/>
+    <hyperlink ref="C93" r:id="rId63" display="https://fred.stlouisfed.org/series/NETEXC" xr:uid="{2A6F419E-109B-4B28-BBFD-1C4307D0445E}"/>
+    <hyperlink ref="C94" r:id="rId64" display="https://fred.stlouisfed.org/series/IEABC" xr:uid="{64987267-8427-4F65-9A0B-9FFF23BB9770}"/>
+    <hyperlink ref="C73" r:id="rId65" display="https://fred.stlouisfed.org/series/BOPGSTB" xr:uid="{5D6B1EFA-5FBA-4914-A6AC-BF0F366D2349}"/>
+    <hyperlink ref="C95" r:id="rId66" display="https://fred.stlouisfed.org/series/GCEC1" xr:uid="{5F9B37BA-8AB3-4DAE-A01C-6F7C5E5C200C}"/>
+    <hyperlink ref="C96" r:id="rId67" display="https://fred.stlouisfed.org/series/EVACANTUSQ176N" xr:uid="{E3C5F381-FD06-488A-8C9F-B3063EF98A32}"/>
+    <hyperlink ref="C81" r:id="rId68" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{CDB27B35-002A-4D8A-BD32-CAD62DF03A98}"/>
+    <hyperlink ref="C78" r:id="rId69" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{99E4FB6A-9CA4-4263-89F8-C482767BDBB0}"/>
+    <hyperlink ref="C77" r:id="rId70" display="https://fred.stlouisfed.org/series/DGS10" xr:uid="{1BC2CE99-09BE-4CB6-8AE5-B826BE2062B3}"/>
+    <hyperlink ref="C51" r:id="rId71" display="https://fred.stlouisfed.org/series/PRAWMINDEXM" xr:uid="{E595BD7B-73BE-4455-A818-237C2E9CACFB}"/>
+    <hyperlink ref="C22" r:id="rId72" display="https://fred.stlouisfed.org/series/PAYEMS" xr:uid="{2FE9D0E0-162F-465E-B85C-F2B30714AB6F}"/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.3" footer="0.3"/>
   <pageSetup scale="64" orientation="landscape" r:id="rId73"/>

</xml_diff>

<commit_message>
Publish EconSheet 261022 (October 22, 2026)
</commit_message>
<xml_diff>
--- a/files/EconSheet.xlsx
+++ b/files/EconSheet.xlsx
@@ -8,44 +8,44 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\192.168.0.130\Documents\Business\EconSheet\FREDData\ToDistribute\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AA137B4E-0FDB-4396-8D52-96235E809950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E51F09B-F0FC-4EBF-8C68-F6D50534AF32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="5295" windowWidth="29040" windowHeight="15720" xr2:uid="{5D5A21E5-3D6F-4F88-A7F3-0ABA08D205B7}"/>
+    <workbookView xWindow="-4110" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{FB91B337-A3E0-4144-B35C-F779116F1D40}"/>
   </bookViews>
   <sheets>
-    <sheet name="261020 EconSheet" sheetId="1" r:id="rId1"/>
+    <sheet name="261022 EconSheet" sheetId="1" r:id="rId1"/>
   </sheets>
   <externalReferences>
     <externalReference r:id="rId2"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'261020 EconSheet'!$A$28:$AF$33</definedName>
-    <definedName name="Conditions" localSheetId="0">'261020 EconSheet'!$AH$3:$AH$96</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'261022 EconSheet'!$A$28:$AF$33</definedName>
+    <definedName name="Conditions" localSheetId="0">'261022 EconSheet'!$AH$3:$AH$96</definedName>
     <definedName name="CurrDates">[1]Currencies!$A$8:$A$14337</definedName>
     <definedName name="DataStart">'[1]Retrieved Data'!$A$1</definedName>
-    <definedName name="DataTable" localSheetId="0">'261020 EconSheet'!$G$4:$AD$96</definedName>
-    <definedName name="DataTableStart" localSheetId="0">'261020 EconSheet'!$G$4</definedName>
-    <definedName name="DatesAndSeries" localSheetId="0">'261020 EconSheet'!$E$4:$F$96</definedName>
+    <definedName name="DataTable" localSheetId="0">'261022 EconSheet'!$G$4:$AD$96</definedName>
+    <definedName name="DataTableStart" localSheetId="0">'261022 EconSheet'!$G$4</definedName>
+    <definedName name="DatesAndSeries" localSheetId="0">'261022 EconSheet'!$E$4:$F$96</definedName>
     <definedName name="DatesAndSeries">[1]EconSheet!$E$4:$F$96</definedName>
-    <definedName name="DatesCol" localSheetId="0">'261020 EconSheet'!$E$4:$E$96</definedName>
+    <definedName name="DatesCol" localSheetId="0">'261022 EconSheet'!$E$4:$E$96</definedName>
     <definedName name="DatesCol">[1]EconSheet!$E$4:$E$96</definedName>
-    <definedName name="ESSeries" localSheetId="0">'261020 EconSheet'!$B$4:$B$103</definedName>
-    <definedName name="ForceAll" localSheetId="0">'261020 EconSheet'!#REF!</definedName>
+    <definedName name="ESSeries" localSheetId="0">'261022 EconSheet'!$B$4:$B$103</definedName>
+    <definedName name="ForceAll" localSheetId="0">'261022 EconSheet'!#REF!</definedName>
     <definedName name="FormatOptions">[1]Calculations!$U$3:$U$14</definedName>
-    <definedName name="FormatTable" localSheetId="0">'261020 EconSheet'!$A$1:$AD$96</definedName>
+    <definedName name="FormatTable" localSheetId="0">'261022 EconSheet'!$A$1:$AD$96</definedName>
     <definedName name="PPIGreen">'[1]Producer Price Archive'!$AB$8:$AD$1023</definedName>
     <definedName name="PPIRaw">'[1]Producer Price Archive'!$B$7:$F$1023</definedName>
     <definedName name="PPIRed">'[1]Producer Price Archive'!$AF$8:$AH$1023</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'261020 EconSheet'!$F$1:$AD$54,'261020 EconSheet'!$F$56:$AD$96</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'261022 EconSheet'!$F$1:$AD$54,'261022 EconSheet'!$F$56:$AD$96</definedName>
     <definedName name="ReleaseData">[1]ReleaseDates!$A$2:$E$1882</definedName>
     <definedName name="ReleaseDates">[1]ReleaseDates!$A$2:$A$1898</definedName>
     <definedName name="SDSeries">[1]SeriesData!$A$2:$A$76</definedName>
     <definedName name="SeriesLookup">'[1]Retrieved Data'!$A$1:$ET$1</definedName>
-    <definedName name="SpFormat1" localSheetId="0">'261020 EconSheet'!$AH$131</definedName>
-    <definedName name="SpFormat2" localSheetId="0">'261020 EconSheet'!$AH$136</definedName>
-    <definedName name="TrueFalse" localSheetId="0">'261020 EconSheet'!#REF!</definedName>
+    <definedName name="SpFormat1" localSheetId="0">'261022 EconSheet'!$AH$131</definedName>
+    <definedName name="SpFormat2" localSheetId="0">'261022 EconSheet'!$AH$136</definedName>
+    <definedName name="TrueFalse" localSheetId="0">'261022 EconSheet'!#REF!</definedName>
     <definedName name="TrueFalse">[1]EconSheet!$AU$1:$AU$2</definedName>
-    <definedName name="WholeTable" localSheetId="0">'261020 EconSheet'!$F$1:$AD$96</definedName>
+    <definedName name="WholeTable" localSheetId="0">'261022 EconSheet'!$F$1:$AD$96</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -76,7 +76,7 @@
     <author>Ron Levin</author>
   </authors>
   <commentList>
-    <comment ref="AA9" authorId="0" shapeId="0" xr:uid="{9E692B9A-28CC-4E72-A432-9BB7B9CE993D}">
+    <comment ref="AD13" authorId="0" shapeId="0" xr:uid="{0E72D1D0-7ADC-43E5-8B95-56BF27A0FAE6}">
       <text>
         <r>
           <rPr>
@@ -86,74 +86,7 @@
             <family val="2"/>
           </rPr>
           <t>Previous Value:
-1,309</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AB9" authorId="0" shapeId="0" xr:uid="{7583EB98-9947-4C84-B81D-F120C8D9C52E}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1,275</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AC9" authorId="0" shapeId="0" xr:uid="{F5971552-6335-4A0E-B942-BC3017D90F6A}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>New Value</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AB11" authorId="0" shapeId="0" xr:uid="{916C8F4A-23EC-45CF-8ED5-CAFD2BF0441D}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Previous Value:
-1,271</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AC11" authorId="0" shapeId="0" xr:uid="{A68CC196-00B3-4203-931A-D564A3E0DC0F}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>New Value</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="AC12" authorId="0" shapeId="0" xr:uid="{9687FA9B-AE28-472A-941C-5CB9355BD05C}">
-      <text>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>New Value</t>
+7.36</t>
         </r>
       </text>
     </comment>
@@ -722,7 +655,7 @@
     <t>Green if</t>
   </si>
   <si>
-    <t>Next Update: 10/21/26</t>
+    <t>Next Update: 10/26/26</t>
   </si>
   <si>
     <t>Next Update</t>
@@ -875,7 +808,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -916,37 +849,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color indexed="64"/>
-      </right>
-      <top style="thick">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thick">
-        <color indexed="64"/>
-      </right>
-      <top style="thick">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thick">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="75">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1029,11 +938,7 @@
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="3" fontId="4" fillId="4" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="165" fontId="4" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="4" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="4" fillId="4" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="3" fontId="4" fillId="3" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="4" fillId="2" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="168" fontId="9" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="22" fontId="9" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
@@ -1046,7 +951,7 @@
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Normal 2" xfId="1" xr:uid="{CE4BE9F1-32C3-44C5-B291-7BF686F9B6A6}"/>
+    <cellStyle name="Normal 2" xfId="1" xr:uid="{C7BDB0DE-50DB-44AE-A57F-C305DAB366D2}"/>
   </cellStyles>
   <dxfs count="237">
     <dxf>
@@ -2682,7 +2587,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7E933BE9-B345-4892-A5E3-30895A269C8F}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{18048505-A72D-479B-B817-34DCAEC56628}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2727,7 +2632,7 @@
         <xdr:cNvPr id="3" name="Picture 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F456B20C-A8A6-4CF4-BDD0-D068DB2FCC14}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DE9A6906-27EF-443D-87EF-182618FB0910}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2875,7 +2780,7 @@
         </row>
         <row r="13">
           <cell r="E13">
-            <v>46317.501782407402</v>
+            <v>46324.501689814817</v>
           </cell>
           <cell r="F13" t="str">
             <v>30 Year Fixed Rate Mortgages (%)</v>
@@ -3121,7 +3026,7 @@
         </row>
         <row r="52">
           <cell r="E52">
-            <v>46316.675405092596</v>
+            <v>46323.554456018523</v>
           </cell>
           <cell r="F52" t="str">
             <v>Crude Oil WTI Cushing - Spot USD/BBL Last day of Month</v>
@@ -3129,7 +3034,7 @@
         </row>
         <row r="53">
           <cell r="E53">
-            <v>46316.675416666665</v>
+            <v>46323.554467592592</v>
           </cell>
           <cell r="F53" t="str">
             <v>Crude Oil Brent - Spot USD/BBL Last day of Month</v>
@@ -3137,7 +3042,7 @@
         </row>
         <row r="54">
           <cell r="E54">
-            <v>46316.676724537043</v>
+            <v>46323.564236111109</v>
           </cell>
           <cell r="F54" t="str">
             <v>Henry Hub Natural Gas Spot Price USD/MBTU</v>
@@ -3272,7 +3177,7 @@
         </row>
         <row r="74">
           <cell r="E74">
-            <v>46316.678391203706</v>
+            <v>46321.687152777769</v>
           </cell>
           <cell r="F74" t="str">
             <v>3-Month Treasury Bills, Secondary market (%)</v>
@@ -3280,7 +3185,7 @@
         </row>
         <row r="75">
           <cell r="E75">
-            <v>46316.678148148145</v>
+            <v>46321.678148148145</v>
           </cell>
           <cell r="F75" t="str">
             <v>Bank Prime Rate (%)</v>
@@ -3288,7 +3193,7 @@
         </row>
         <row r="76">
           <cell r="E76">
-            <v>46316.678495370375</v>
+            <v>46321.68712962963</v>
           </cell>
           <cell r="F76" t="str">
             <v>2-yr. Treasury Bond Yield at Constant Maturity (%)</v>
@@ -3296,7 +3201,7 @@
         </row>
         <row r="77">
           <cell r="E77">
-            <v>46316.678310185176</v>
+            <v>46321.687199074076</v>
           </cell>
           <cell r="F77" t="str">
             <v>10-yr. Treasury Bond Yield at Constant Maturity (%)</v>
@@ -3304,7 +3209,7 @@
         </row>
         <row r="78">
           <cell r="E78">
-            <v>46316.710868055554</v>
+            <v>46321.710868055554</v>
           </cell>
           <cell r="F78" t="str">
             <v>10 Yr - 2 Yr Treasury Spread - Const Maturity %</v>
@@ -3312,7 +3217,7 @@
         </row>
         <row r="79">
           <cell r="E79">
-            <v>46316.678263888898</v>
+            <v>46321.687152777769</v>
           </cell>
           <cell r="F79" t="str">
             <v>10-yr. Treasury Bond Yield at Const. Mat. Inflation Indexed (%)</v>
@@ -3320,7 +3225,7 @@
         </row>
         <row r="80">
           <cell r="E80">
-            <v>46316.678472222222</v>
+            <v>46321.687175925923</v>
           </cell>
           <cell r="F80" t="str">
             <v>30-yr. Treasury Bond Yield at Constant Maturity (%)</v>
@@ -3328,7 +3233,7 @@
         </row>
         <row r="81">
           <cell r="E81">
-            <v>46316.710891203693</v>
+            <v>46321.710729166662</v>
           </cell>
           <cell r="F81" t="str">
             <v>10 Yr - 3 Month Treasury Spread - Const Maturity %</v>
@@ -44916,10 +44821,10 @@
             <v>46317</v>
           </cell>
           <cell r="C114" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D114">
-            <v>46317</v>
+            <v>0</v>
           </cell>
           <cell r="E114">
             <v>114</v>
@@ -53450,10 +53355,10 @@
             <v>46316</v>
           </cell>
           <cell r="C616" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D616">
-            <v>46316</v>
+            <v>0</v>
           </cell>
           <cell r="E616">
             <v>616</v>
@@ -53467,10 +53372,10 @@
             <v>46317</v>
           </cell>
           <cell r="C617" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D617">
-            <v>46317</v>
+            <v>0</v>
           </cell>
           <cell r="E617">
             <v>617</v>
@@ -53484,10 +53389,10 @@
             <v>46318</v>
           </cell>
           <cell r="C618" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D618">
-            <v>46318</v>
+            <v>0</v>
           </cell>
           <cell r="E618">
             <v>618</v>
@@ -58975,10 +58880,10 @@
             <v>46316</v>
           </cell>
           <cell r="C941" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D941">
-            <v>46316</v>
+            <v>0</v>
           </cell>
           <cell r="E941">
             <v>941</v>
@@ -58992,10 +58897,10 @@
             <v>46317</v>
           </cell>
           <cell r="C942" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D942">
-            <v>46317</v>
+            <v>0</v>
           </cell>
           <cell r="E942">
             <v>942</v>
@@ -59009,10 +58914,10 @@
             <v>46318</v>
           </cell>
           <cell r="C943" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D943">
-            <v>46318</v>
+            <v>0</v>
           </cell>
           <cell r="E943">
             <v>943</v>
@@ -61661,10 +61566,10 @@
             <v>46316</v>
           </cell>
           <cell r="C1099" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1099">
-            <v>46316</v>
+            <v>0</v>
           </cell>
           <cell r="E1099">
             <v>1099</v>
@@ -62936,10 +62841,10 @@
             <v>46316</v>
           </cell>
           <cell r="C1174" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1174">
-            <v>46316</v>
+            <v>0</v>
           </cell>
           <cell r="E1174">
             <v>1174</v>
@@ -68563,10 +68468,10 @@
             <v>46316</v>
           </cell>
           <cell r="C1505" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1505">
-            <v>46316</v>
+            <v>0</v>
           </cell>
           <cell r="E1505">
             <v>1505</v>
@@ -68580,10 +68485,10 @@
             <v>46317</v>
           </cell>
           <cell r="C1506" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1506">
-            <v>46317</v>
+            <v>0</v>
           </cell>
           <cell r="E1506">
             <v>1506</v>
@@ -68597,10 +68502,10 @@
             <v>46318</v>
           </cell>
           <cell r="C1507" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1507">
-            <v>46318</v>
+            <v>0</v>
           </cell>
           <cell r="E1507">
             <v>1507</v>
@@ -74156,10 +74061,10 @@
             <v>46316</v>
           </cell>
           <cell r="C1834" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1834">
-            <v>46316</v>
+            <v>0</v>
           </cell>
           <cell r="E1834">
             <v>1834</v>
@@ -74173,10 +74078,10 @@
             <v>46317</v>
           </cell>
           <cell r="C1835" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1835">
-            <v>46317</v>
+            <v>0</v>
           </cell>
           <cell r="E1835">
             <v>1835</v>
@@ -74190,10 +74095,10 @@
             <v>46318</v>
           </cell>
           <cell r="C1836" t="b">
-            <v>0</v>
+            <v>1</v>
           </cell>
           <cell r="D1836">
-            <v>46318</v>
+            <v>0</v>
           </cell>
           <cell r="E1836">
             <v>1836</v>
@@ -75384,7 +75289,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8996EBC1-CAA1-4757-AC2A-3D6476573764}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58468F2B-1070-4EDC-8B83-95F0BA3A0A66}">
   <sheetPr codeName="Sheet22">
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
@@ -75411,13 +75316,13 @@
     <col min="34" max="34" width="10.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:34" s="72" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="74"/>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74"/>
+    <row r="1" spans="1:34" s="68" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A1" s="70"/>
+      <c r="B1" s="70"/>
+      <c r="C1" s="70"/>
       <c r="D1" s="37"/>
       <c r="E1" s="37"/>
-      <c r="F1" s="74" t="s">
+      <c r="F1" s="70" t="s">
         <v>190</v>
       </c>
       <c r="G1" s="34">
@@ -75493,7 +75398,7 @@
         <v>2026</v>
       </c>
     </row>
-    <row r="2" spans="1:34" s="72" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:34" s="68" customFormat="1" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A2" s="25"/>
       <c r="B2" s="25"/>
       <c r="C2" s="25" t="s">
@@ -75508,79 +75413,79 @@
       <c r="F2" s="25" t="s">
         <v>186</v>
       </c>
-      <c r="G2" s="73">
+      <c r="G2" s="69">
         <v>45597</v>
       </c>
-      <c r="H2" s="73">
+      <c r="H2" s="69">
         <v>45627</v>
       </c>
-      <c r="I2" s="73">
+      <c r="I2" s="69">
         <v>45658</v>
       </c>
-      <c r="J2" s="73">
+      <c r="J2" s="69">
         <v>45689</v>
       </c>
-      <c r="K2" s="73">
+      <c r="K2" s="69">
         <v>45717</v>
       </c>
-      <c r="L2" s="73">
+      <c r="L2" s="69">
         <v>45748</v>
       </c>
-      <c r="M2" s="73">
+      <c r="M2" s="69">
         <v>45778</v>
       </c>
-      <c r="N2" s="73">
+      <c r="N2" s="69">
         <v>45809</v>
       </c>
-      <c r="O2" s="73">
+      <c r="O2" s="69">
         <v>45839</v>
       </c>
-      <c r="P2" s="73">
+      <c r="P2" s="69">
         <v>45870</v>
       </c>
-      <c r="Q2" s="73">
+      <c r="Q2" s="69">
         <v>45901</v>
       </c>
-      <c r="R2" s="73">
+      <c r="R2" s="69">
         <v>45931</v>
       </c>
-      <c r="S2" s="73">
+      <c r="S2" s="69">
         <v>45962</v>
       </c>
-      <c r="T2" s="73">
+      <c r="T2" s="69">
         <v>45992</v>
       </c>
-      <c r="U2" s="73">
+      <c r="U2" s="69">
         <v>46023</v>
       </c>
-      <c r="V2" s="73">
+      <c r="V2" s="69">
         <v>46054</v>
       </c>
-      <c r="W2" s="73">
+      <c r="W2" s="69">
         <v>46082</v>
       </c>
-      <c r="X2" s="73">
+      <c r="X2" s="69">
         <v>46113</v>
       </c>
-      <c r="Y2" s="73">
+      <c r="Y2" s="69">
         <v>46143</v>
       </c>
-      <c r="Z2" s="73">
+      <c r="Z2" s="69">
         <v>46174</v>
       </c>
-      <c r="AA2" s="73">
+      <c r="AA2" s="69">
         <v>46204</v>
       </c>
-      <c r="AB2" s="73">
+      <c r="AB2" s="69">
         <v>46235</v>
       </c>
-      <c r="AC2" s="73">
+      <c r="AC2" s="69">
         <v>46266</v>
       </c>
-      <c r="AD2" s="73">
+      <c r="AD2" s="69">
         <v>46296</v>
       </c>
-      <c r="AH2" s="72" t="s">
+      <c r="AH2" s="68" t="s">
         <v>185</v>
       </c>
     </row>
@@ -75590,11 +75495,11 @@
         <v>184</v>
       </c>
       <c r="C3" s="10"/>
-      <c r="D3" s="71">
-        <v>46315.356828703705</v>
-      </c>
-      <c r="E3" s="70">
-        <v>46316.675405092596</v>
+      <c r="D3" s="67">
+        <v>46317.501689814817</v>
+      </c>
+      <c r="E3" s="66">
+        <v>46321.678148148145</v>
       </c>
       <c r="F3" s="10" t="s">
         <v>183</v>
@@ -75718,7 +75623,7 @@
       <c r="AD4" s="7" t="e">
         <v>#N/A</v>
       </c>
-      <c r="AE4" s="69" t="s">
+      <c r="AE4" s="65" t="s">
         <v>35</v>
       </c>
       <c r="AH4" t="s">
@@ -76010,7 +75915,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:34" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>9</v>
       </c>
@@ -76105,7 +76010,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A9" s="6">
         <v>7</v>
       </c>
@@ -76184,13 +76089,13 @@
       <c r="Z9" s="18">
         <v>1439</v>
       </c>
-      <c r="AA9" s="68">
+      <c r="AA9" s="17">
         <v>1369</v>
       </c>
-      <c r="AB9" s="67">
+      <c r="AB9" s="17">
         <v>1288</v>
       </c>
-      <c r="AC9" s="67">
+      <c r="AC9" s="17">
         <v>1221</v>
       </c>
       <c r="AD9" s="18" t="e">
@@ -76200,7 +76105,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="10" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A10" s="25"/>
       <c r="B10" s="25"/>
       <c r="C10" s="16" t="s">
@@ -76285,7 +76190,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>131</v>
       </c>
@@ -76367,10 +76272,10 @@
       <c r="AA11" s="62">
         <v>1267</v>
       </c>
-      <c r="AB11" s="66">
+      <c r="AB11" s="62">
         <v>1280</v>
       </c>
-      <c r="AC11" s="65">
+      <c r="AC11" s="62">
         <v>1280</v>
       </c>
       <c r="AD11" s="13" t="e">
@@ -76380,7 +76285,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:34" ht="16.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6">
         <v>133</v>
       </c>
@@ -76465,17 +76370,17 @@
       <c r="AB12" s="59">
         <v>-2.0935100000000002</v>
       </c>
-      <c r="AC12" s="64">
+      <c r="AC12" s="59">
         <v>-0.21382999999999999</v>
       </c>
-      <c r="AD12" s="4" t="e">
+      <c r="AD12" s="7" t="e">
         <v>#N/A</v>
       </c>
       <c r="AH12" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:34" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:34" ht="17.25" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="25">
         <v>13</v>
       </c>
@@ -76486,10 +76391,10 @@
         <v>163</v>
       </c>
       <c r="D13" s="15">
-        <v>46310.501782407409</v>
+        <v>46317.501689814817</v>
       </c>
       <c r="E13" s="52">
-        <v>46317.501782407402</v>
+        <v>46324.501689814817</v>
       </c>
       <c r="F13" s="43" t="s">
         <v>162</v>
@@ -76563,14 +76468,14 @@
       <c r="AC13" s="40">
         <v>6.86</v>
       </c>
-      <c r="AD13" s="40">
-        <v>7.36</v>
+      <c r="AD13" s="64">
+        <v>7.35</v>
       </c>
       <c r="AH13" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:34" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:34" ht="16.5" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A14" s="25"/>
       <c r="B14" s="25"/>
       <c r="C14" s="25"/>
@@ -79492,10 +79397,10 @@
         <v>93</v>
       </c>
       <c r="D52" s="15">
-        <v>46310.675405092596</v>
+        <v>46316.554456018515</v>
       </c>
       <c r="E52" s="14">
-        <v>46316.675405092596</v>
+        <v>46323.554456018523</v>
       </c>
       <c r="F52" s="25" t="s">
         <v>97</v>
@@ -79587,10 +79492,10 @@
         <v>93</v>
       </c>
       <c r="D53" s="21">
-        <v>46310.675416666665</v>
+        <v>46316.554467592592</v>
       </c>
       <c r="E53" s="20">
-        <v>46316.675416666665</v>
+        <v>46323.554467592592</v>
       </c>
       <c r="F53" s="6" t="s">
         <v>95</v>
@@ -79682,10 +79587,10 @@
         <v>93</v>
       </c>
       <c r="D54" s="24">
-        <v>46310.676724537036</v>
+        <v>46316.564236111109</v>
       </c>
       <c r="E54" s="23">
-        <v>46316.676724537043</v>
+        <v>46323.564236111109</v>
       </c>
       <c r="F54" s="57" t="s">
         <v>92</v>
@@ -81384,10 +81289,10 @@
         <v>37</v>
       </c>
       <c r="D74" s="24">
-        <v>46314.678391203706</v>
+        <v>46316.687152777777</v>
       </c>
       <c r="E74" s="49">
-        <v>46316.678391203706</v>
+        <v>46321.687152777769</v>
       </c>
       <c r="F74" s="48" t="s">
         <v>57</v>
@@ -81482,7 +81387,7 @@
         <v>46309.678148148145</v>
       </c>
       <c r="E75" s="52">
-        <v>46316.678148148145</v>
+        <v>46321.678148148145</v>
       </c>
       <c r="F75" s="43" t="s">
         <v>55</v>
@@ -81574,10 +81479,10 @@
         <v>37</v>
       </c>
       <c r="D76" s="21">
-        <v>46314.678495370368</v>
+        <v>46316.68712962963</v>
       </c>
       <c r="E76" s="53">
-        <v>46316.678495370375</v>
+        <v>46321.68712962963</v>
       </c>
       <c r="F76" s="47" t="s">
         <v>53</v>
@@ -81669,10 +81574,10 @@
         <v>37</v>
       </c>
       <c r="D77" s="24">
-        <v>46314.678310185183</v>
+        <v>46316.687199074076</v>
       </c>
       <c r="E77" s="52">
-        <v>46316.678310185176</v>
+        <v>46321.687199074076</v>
       </c>
       <c r="F77" s="48" t="s">
         <v>51</v>
@@ -81767,7 +81672,7 @@
         <v>46296.710868055554</v>
       </c>
       <c r="E78" s="52">
-        <v>46316.710868055554</v>
+        <v>46321.710868055554</v>
       </c>
       <c r="F78" s="43" t="s">
         <v>49</v>
@@ -81860,10 +81765,10 @@
         <v>37</v>
       </c>
       <c r="D79" s="21">
-        <v>46314.678263888891</v>
+        <v>46316.687152777777</v>
       </c>
       <c r="E79" s="50">
-        <v>46316.678263888898</v>
+        <v>46321.687152777769</v>
       </c>
       <c r="F79" s="47" t="s">
         <v>47</v>
@@ -81955,10 +81860,10 @@
         <v>37</v>
       </c>
       <c r="D80" s="24">
-        <v>46314.678472222222</v>
+        <v>46316.687175925923</v>
       </c>
       <c r="E80" s="49">
-        <v>46316.678472222222</v>
+        <v>46321.687175925923</v>
       </c>
       <c r="F80" s="48" t="s">
         <v>45</v>
@@ -82050,10 +81955,10 @@
         <v>42</v>
       </c>
       <c r="D81" s="15">
-        <v>46311.7108912037</v>
+        <v>46316.710729166669</v>
       </c>
       <c r="E81" s="14">
-        <v>46316.710891203693</v>
+        <v>46321.710729166662</v>
       </c>
       <c r="F81" s="43" t="s">
         <v>41</v>
@@ -86129,83 +86034,83 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="AH3:AH96" xr:uid="{88E6C84E-F064-4FC3-A541-ECE5120D7698}">
+    <dataValidation type="list" showInputMessage="1" showErrorMessage="1" sqref="AH3:AH96" xr:uid="{A1E7A28C-F186-4E5E-B020-1A80F6041EDE}">
       <formula1>FormatOptions</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="C4" r:id="rId1" display="https://fred.stlouisfed.org/series/MPCTXXXXS" xr:uid="{7FE01B38-A3AD-4D57-965B-C523DD5E559B}"/>
-    <hyperlink ref="C5" r:id="rId2" display="https://fred.stlouisfed.org/series/TLPRVCONS" xr:uid="{964DA74E-E517-4930-A82D-DCD1F8D115E5}"/>
-    <hyperlink ref="C6" r:id="rId3" display="https://fred.stlouisfed.org/series/TLRESCONS" xr:uid="{5641A39B-6657-4681-9736-4C25135605FB}"/>
-    <hyperlink ref="C7" r:id="rId4" display="https://fred.stlouisfed.org/series/TLHWYCONS" xr:uid="{2A7E7C11-884B-4B9E-A240-9DF70B084BD7}"/>
-    <hyperlink ref="C8" r:id="rId5" display="https://fred.stlouisfed.org/series/HSN1F" xr:uid="{A9D8F207-9447-40D0-8C37-7A13276BC593}"/>
-    <hyperlink ref="C9" r:id="rId6" display="https://fred.stlouisfed.org/series/HOUST" xr:uid="{963A071D-2D6D-4A59-A27E-071FCFCEC865}"/>
-    <hyperlink ref="C11" r:id="rId7" display="https://fred.stlouisfed.org/series/UNDCONTSA" xr:uid="{E383E6F0-7CB8-4B4F-90D4-A04D33B07F45}"/>
-    <hyperlink ref="C12" r:id="rId8" display="https://fred.stlouisfed.org/series/PERMIT" xr:uid="{3B856B7F-91AF-4166-9533-A99C6CF66649}"/>
-    <hyperlink ref="C13" r:id="rId9" display="https://fred.stlouisfed.org/series/MORTGAGE30US" xr:uid="{0A124A9B-8D32-420B-962F-CF7BA73D921D}"/>
-    <hyperlink ref="C16" r:id="rId10" display="https://fred.stlouisfed.org/series/ALTSALES" xr:uid="{3B8E6461-79C0-4F65-96C3-8C95DB9CDF69}"/>
-    <hyperlink ref="C17" r:id="rId11" display="https://fred.stlouisfed.org/series/AISRSA" xr:uid="{98C603F5-3CD7-40ED-83A5-C2BFF4EA9671}"/>
-    <hyperlink ref="C18" r:id="rId12" display="https://fred.stlouisfed.org/series/DAUTOSAAR" xr:uid="{373D6F81-B00A-423A-9D01-BFD93895913B}"/>
-    <hyperlink ref="C19" r:id="rId13" display="https://fred.stlouisfed.org/series/DAUPSA" xr:uid="{D15220AD-AC60-46EB-912E-1EF944F661DB}"/>
-    <hyperlink ref="C23" r:id="rId14" display="https://fred.stlouisfed.org/series/UNEMPLOY" xr:uid="{B5F427E9-38C1-4D6E-BF8F-249E264EC417}"/>
-    <hyperlink ref="C24" r:id="rId15" display="https://fred.stlouisfed.org/series/UNRATE" xr:uid="{77498871-04FE-4760-97FA-0443C59AB29E}"/>
-    <hyperlink ref="C25" r:id="rId16" display="https://fred.stlouisfed.org/series/AWHNONAG" xr:uid="{8532A332-DBB3-4ABF-B0A9-71E35CD31CC8}"/>
-    <hyperlink ref="C26" r:id="rId17" display="https://fred.stlouisfed.org/series/CLF16OV" xr:uid="{BF4A67B3-2B9E-4810-B579-1ADC6ED099E5}"/>
-    <hyperlink ref="C29" r:id="rId18" display="https://fred.stlouisfed.org/series/INDPRO" xr:uid="{31C373F4-8FFF-400C-B3A0-C8759B7ADDD7}"/>
-    <hyperlink ref="C30" r:id="rId19" display="https://fred.stlouisfed.org/series/TCU" xr:uid="{52F33519-107A-4C0C-991B-0D2845F0C384}"/>
-    <hyperlink ref="C31" r:id="rId20" display="https://fred.stlouisfed.org/series/AMTMNO" xr:uid="{0046E6F3-C9C3-4F73-A235-A25E5D49DF8C}"/>
-    <hyperlink ref="C32" r:id="rId21" display="https://fred.stlouisfed.org/series/DGORDER" xr:uid="{03227960-78A4-463A-A845-E22B47327E0C}"/>
-    <hyperlink ref="C33" r:id="rId22" display="https://fred.stlouisfed.org/series/ANXAVS" xr:uid="{5B31B5FC-BDFE-48A6-BA01-F758058970C3}"/>
-    <hyperlink ref="C36" r:id="rId23" display="https://fred.stlouisfed.org/series/BUSINV" xr:uid="{F9D91AD2-94B9-43ED-9548-59AE5387FC68}"/>
-    <hyperlink ref="C37" r:id="rId24" display="https://fred.stlouisfed.org/series/ISRATIO" xr:uid="{FE545E5D-C4B6-46C4-AB9F-5B0CB03E5464}"/>
-    <hyperlink ref="C38" r:id="rId25" display="https://fred.stlouisfed.org/series/RETAILMPCIMSA" xr:uid="{E8027F13-EBE1-4273-8B7E-D7264C848DDB}"/>
-    <hyperlink ref="C39" r:id="rId26" display="https://fred.stlouisfed.org/series/ACNGTI" xr:uid="{42556524-E306-4BFF-BE01-15BDC05D3F94}"/>
-    <hyperlink ref="C42" r:id="rId27" display="https://fred.stlouisfed.org/series/CPIAUCSL" xr:uid="{D6BD34AD-045F-47C5-8468-9E2691214C80}"/>
-    <hyperlink ref="C43" r:id="rId28" display="https://fred.stlouisfed.org/series/CPIFABSL" xr:uid="{25840D65-2EE5-49F1-96FD-A3A83639580D}"/>
-    <hyperlink ref="C44" r:id="rId29" display="https://fred.stlouisfed.org/series/CPIENGSL" xr:uid="{48819B20-1AC4-456B-BABD-FFC1D8811050}"/>
-    <hyperlink ref="C45" r:id="rId30" display="https://fred.stlouisfed.org/series/CPILFESL" xr:uid="{F0D76998-766A-400F-B9F4-C5090E4B4D64}"/>
-    <hyperlink ref="C48" r:id="rId31" display="https://fred.stlouisfed.org/series/WPUFD49207" xr:uid="{F5FA2F6A-7063-4E76-A0AA-752BFB9A2381}"/>
-    <hyperlink ref="C49" r:id="rId32" display="https://fred.stlouisfed.org/series/WPSID61" xr:uid="{3C9EA920-666C-47A6-BD2F-B1B1F394334B}"/>
-    <hyperlink ref="C50" r:id="rId33" display="https://fred.stlouisfed.org/series/PRAWMINDEXM" xr:uid="{755F095A-4FAC-494C-9590-E0A8516EB873}"/>
-    <hyperlink ref="C52" r:id="rId34" display="https://fred.stlouisfed.org/series/DCOILWTICO" xr:uid="{FD90CB8C-6A1F-49DD-ADF1-4FE77EB50725}"/>
-    <hyperlink ref="C53" r:id="rId35" display="https://fred.stlouisfed.org/series/DCOILBRENTEU" xr:uid="{68909A2C-1957-4769-A91C-A290ADA458F6}"/>
-    <hyperlink ref="C54" r:id="rId36" display="https://fred.stlouisfed.org/series/DHHNGSP" xr:uid="{A2538FD1-1EEB-4416-B376-7FC5CA949835}"/>
-    <hyperlink ref="C58" r:id="rId37" display="https://fred.stlouisfed.org/series/DHHNGSP" xr:uid="{E00AB092-68CB-445A-9D48-28908B2BA7B3}"/>
-    <hyperlink ref="C59" r:id="rId38" display="https://fred.stlouisfed.org/series/PI" xr:uid="{DA693AB0-E80C-4F4B-8A89-055240EAB768}"/>
-    <hyperlink ref="C60" r:id="rId39" display="https://fred.stlouisfed.org/series/DSPI" xr:uid="{3FA7B551-F90F-41E7-A525-9CC8DF8A0A16}"/>
-    <hyperlink ref="C61" r:id="rId40" display="https://fred.stlouisfed.org/series/A229RX0" xr:uid="{3AF0D127-26A5-4501-9233-CAF10AB11406}"/>
-    <hyperlink ref="C62" r:id="rId41" display="https://fred.stlouisfed.org/series/PSAVERT" xr:uid="{F8571D3E-8330-4696-A1EE-28C818830989}"/>
-    <hyperlink ref="C63" r:id="rId42" display="https://fred.stlouisfed.org/series/PCE" xr:uid="{03E76F18-EAEB-40C1-8C55-7BD6C0BA8C79}"/>
-    <hyperlink ref="C64" r:id="rId43" display="https://fred.stlouisfed.org/series/PCEC96" xr:uid="{FBA2124B-7C43-40AC-9FDA-6E80AD66FAE7}"/>
-    <hyperlink ref="C65" r:id="rId44" display="https://fred.stlouisfed.org/series/MRTSMPCSM44X72USS" xr:uid="{8D8F07A4-739C-4053-BED1-980B18BB124F}"/>
-    <hyperlink ref="C66" r:id="rId45" display="https://fred.stlouisfed.org/series/TOTALSL" xr:uid="{AF6B8628-BA4E-40E1-9091-461FC44512E5}"/>
-    <hyperlink ref="C67" r:id="rId46" display="https://fred.stlouisfed.org/series/PCEND" xr:uid="{C17F6EEE-A597-4EA5-A5CA-EF6A08DE86F7}"/>
-    <hyperlink ref="C68" r:id="rId47" display="https://fred.stlouisfed.org/series/A22BVS" xr:uid="{9DE336FA-DDEC-41BD-B4A5-F4E9B3201E1D}"/>
-    <hyperlink ref="C71" r:id="rId48" display="https://fred.stlouisfed.org/series/M1SL" xr:uid="{E8092FC1-3BD3-4791-850A-ACF1BBDDA101}"/>
-    <hyperlink ref="C72" r:id="rId49" display="https://fred.stlouisfed.org/series/M2SL" xr:uid="{409F6FEC-3471-4CD1-A095-E451963826BB}"/>
-    <hyperlink ref="C74" r:id="rId50" display="https://fred.stlouisfed.org/series/DTB3" xr:uid="{C282C1F8-9A1E-48C0-9B70-5633368F4EE7}"/>
-    <hyperlink ref="C75" r:id="rId51" display="https://fred.stlouisfed.org/series/DPRIME" xr:uid="{EF653A18-25A3-47DB-9619-6CC165D86CC1}"/>
-    <hyperlink ref="C76" r:id="rId52" display="https://fred.stlouisfed.org/series/DGS10" xr:uid="{0F9B32FC-36CF-4242-B00E-54A99E32D405}"/>
-    <hyperlink ref="C79" r:id="rId53" display="https://fred.stlouisfed.org/series/DFII10" xr:uid="{D8284E1B-44CD-4A99-9920-0A79954597DE}"/>
-    <hyperlink ref="C80" r:id="rId54" display="https://fred.stlouisfed.org/series/DGS30" xr:uid="{76462D74-86DF-4053-91F3-252423DB4A35}"/>
-    <hyperlink ref="C82" r:id="rId55" display="https://fred.stlouisfed.org/series/DEXUSEU" xr:uid="{3C31135F-CF97-49B5-9EBE-47B6BC825FB5}"/>
-    <hyperlink ref="C83" r:id="rId56" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{4EBE0BCB-0013-42BC-8D26-03D99E453B35}"/>
-    <hyperlink ref="C87" r:id="rId57" display="https://fred.stlouisfed.org/series/GDPC1" xr:uid="{BA2A03C1-1A8B-473F-BB60-5416C585C91B}"/>
-    <hyperlink ref="C88" r:id="rId58" display="https://fred.stlouisfed.org/series/GDP" xr:uid="{0D40D6CA-9593-414E-8CEB-A5D591390BB9}"/>
-    <hyperlink ref="C89" r:id="rId59" display="https://fred.stlouisfed.org/series/PCEDG" xr:uid="{887DD5D8-D54A-45F4-AAAA-5B292CFD6730}"/>
-    <hyperlink ref="C90" r:id="rId60" display="https://fred.stlouisfed.org/series/PNFIC1" xr:uid="{2866E896-2C05-463A-9F71-C084426C46A6}"/>
-    <hyperlink ref="C91" r:id="rId61" display="https://fred.stlouisfed.org/series/PRFIC1" xr:uid="{7CEFCBBA-A890-43B2-B8D8-867AD59BF651}"/>
-    <hyperlink ref="C92" r:id="rId62" display="https://fred.stlouisfed.org/series/CBI" xr:uid="{25957A9D-9859-4425-B336-A88CA651DBFE}"/>
-    <hyperlink ref="C93" r:id="rId63" display="https://fred.stlouisfed.org/series/NETEXC" xr:uid="{2A6F419E-109B-4B28-BBFD-1C4307D0445E}"/>
-    <hyperlink ref="C94" r:id="rId64" display="https://fred.stlouisfed.org/series/IEABC" xr:uid="{64987267-8427-4F65-9A0B-9FFF23BB9770}"/>
-    <hyperlink ref="C73" r:id="rId65" display="https://fred.stlouisfed.org/series/BOPGSTB" xr:uid="{5D6B1EFA-5FBA-4914-A6AC-BF0F366D2349}"/>
-    <hyperlink ref="C95" r:id="rId66" display="https://fred.stlouisfed.org/series/GCEC1" xr:uid="{5F9B37BA-8AB3-4DAE-A01C-6F7C5E5C200C}"/>
-    <hyperlink ref="C96" r:id="rId67" display="https://fred.stlouisfed.org/series/EVACANTUSQ176N" xr:uid="{E3C5F381-FD06-488A-8C9F-B3063EF98A32}"/>
-    <hyperlink ref="C81" r:id="rId68" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{CDB27B35-002A-4D8A-BD32-CAD62DF03A98}"/>
-    <hyperlink ref="C78" r:id="rId69" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{99E4FB6A-9CA4-4263-89F8-C482767BDBB0}"/>
-    <hyperlink ref="C77" r:id="rId70" display="https://fred.stlouisfed.org/series/DGS10" xr:uid="{1BC2CE99-09BE-4CB6-8AE5-B826BE2062B3}"/>
-    <hyperlink ref="C51" r:id="rId71" display="https://fred.stlouisfed.org/series/PRAWMINDEXM" xr:uid="{E595BD7B-73BE-4455-A818-237C2E9CACFB}"/>
-    <hyperlink ref="C22" r:id="rId72" display="https://fred.stlouisfed.org/series/PAYEMS" xr:uid="{2FE9D0E0-162F-465E-B85C-F2B30714AB6F}"/>
+    <hyperlink ref="C4" r:id="rId1" display="https://fred.stlouisfed.org/series/MPCTXXXXS" xr:uid="{E098FD44-28F0-4D43-A631-A8BEB7E398A7}"/>
+    <hyperlink ref="C5" r:id="rId2" display="https://fred.stlouisfed.org/series/TLPRVCONS" xr:uid="{2A9C4162-DAB6-42D4-9EB1-98167F36B93E}"/>
+    <hyperlink ref="C6" r:id="rId3" display="https://fred.stlouisfed.org/series/TLRESCONS" xr:uid="{B590A063-ADFB-482F-B11C-D85565F8F20A}"/>
+    <hyperlink ref="C7" r:id="rId4" display="https://fred.stlouisfed.org/series/TLHWYCONS" xr:uid="{F73EEE98-77F7-48EF-B383-884C3510D6C3}"/>
+    <hyperlink ref="C8" r:id="rId5" display="https://fred.stlouisfed.org/series/HSN1F" xr:uid="{A11373A9-59C1-469C-A67B-D2AED8D0157D}"/>
+    <hyperlink ref="C9" r:id="rId6" display="https://fred.stlouisfed.org/series/HOUST" xr:uid="{A99E8ED1-314E-4E98-840C-691D3EE4F89B}"/>
+    <hyperlink ref="C11" r:id="rId7" display="https://fred.stlouisfed.org/series/UNDCONTSA" xr:uid="{DF926F85-CBD6-41A2-9FA9-3E8A33AB90A3}"/>
+    <hyperlink ref="C12" r:id="rId8" display="https://fred.stlouisfed.org/series/PERMIT" xr:uid="{4FBCFE7F-579F-43A1-98BE-29E31166A516}"/>
+    <hyperlink ref="C13" r:id="rId9" display="https://fred.stlouisfed.org/series/MORTGAGE30US" xr:uid="{892D2B13-60FF-44DD-989C-B73BC0E0F57F}"/>
+    <hyperlink ref="C16" r:id="rId10" display="https://fred.stlouisfed.org/series/ALTSALES" xr:uid="{FF0DBFEF-6954-41F6-9D2E-123678F3133C}"/>
+    <hyperlink ref="C17" r:id="rId11" display="https://fred.stlouisfed.org/series/AISRSA" xr:uid="{F8230538-9668-4274-863C-C8DE675D2FD1}"/>
+    <hyperlink ref="C18" r:id="rId12" display="https://fred.stlouisfed.org/series/DAUTOSAAR" xr:uid="{0D18D09E-2F59-436A-9B06-34AAB71FF43F}"/>
+    <hyperlink ref="C19" r:id="rId13" display="https://fred.stlouisfed.org/series/DAUPSA" xr:uid="{B5946E50-D2B7-4088-BA45-721A4B778DE7}"/>
+    <hyperlink ref="C23" r:id="rId14" display="https://fred.stlouisfed.org/series/UNEMPLOY" xr:uid="{CF7700AC-218F-4FD6-B782-4FABF4BD6C69}"/>
+    <hyperlink ref="C24" r:id="rId15" display="https://fred.stlouisfed.org/series/UNRATE" xr:uid="{05C31E23-DD48-44E3-B925-98E0BE8B4F24}"/>
+    <hyperlink ref="C25" r:id="rId16" display="https://fred.stlouisfed.org/series/AWHNONAG" xr:uid="{842F9687-80B9-42DC-8636-66C46BA3D42B}"/>
+    <hyperlink ref="C26" r:id="rId17" display="https://fred.stlouisfed.org/series/CLF16OV" xr:uid="{EC9939A6-5721-4B64-BE42-543873A4B91C}"/>
+    <hyperlink ref="C29" r:id="rId18" display="https://fred.stlouisfed.org/series/INDPRO" xr:uid="{200964CD-A026-480F-B3DC-3FABF2B54363}"/>
+    <hyperlink ref="C30" r:id="rId19" display="https://fred.stlouisfed.org/series/TCU" xr:uid="{1850B0A9-A64A-479A-878E-07A83CB39B79}"/>
+    <hyperlink ref="C31" r:id="rId20" display="https://fred.stlouisfed.org/series/AMTMNO" xr:uid="{0A84041C-7801-4ED2-BA8D-8D3BBD9E853A}"/>
+    <hyperlink ref="C32" r:id="rId21" display="https://fred.stlouisfed.org/series/DGORDER" xr:uid="{C5B9D643-94B7-4DE5-831C-8027D8F34E7C}"/>
+    <hyperlink ref="C33" r:id="rId22" display="https://fred.stlouisfed.org/series/ANXAVS" xr:uid="{25A70503-B5B4-49A0-B4A3-48F6ED39F51B}"/>
+    <hyperlink ref="C36" r:id="rId23" display="https://fred.stlouisfed.org/series/BUSINV" xr:uid="{667495B6-A494-41BF-9FAA-12C3BE78EB49}"/>
+    <hyperlink ref="C37" r:id="rId24" display="https://fred.stlouisfed.org/series/ISRATIO" xr:uid="{7D19DA59-FB1C-41C4-B60C-69B9218A51D1}"/>
+    <hyperlink ref="C38" r:id="rId25" display="https://fred.stlouisfed.org/series/RETAILMPCIMSA" xr:uid="{93CC6739-49C0-4100-A3A1-068E32D89441}"/>
+    <hyperlink ref="C39" r:id="rId26" display="https://fred.stlouisfed.org/series/ACNGTI" xr:uid="{DA068EF5-1CAB-4B5A-A8F6-B2B4FC79655E}"/>
+    <hyperlink ref="C42" r:id="rId27" display="https://fred.stlouisfed.org/series/CPIAUCSL" xr:uid="{4C1176E3-4F88-4381-89A4-F8B921D5D67A}"/>
+    <hyperlink ref="C43" r:id="rId28" display="https://fred.stlouisfed.org/series/CPIFABSL" xr:uid="{5E22767A-0CEF-4519-ABD0-4CC0839D48A5}"/>
+    <hyperlink ref="C44" r:id="rId29" display="https://fred.stlouisfed.org/series/CPIENGSL" xr:uid="{9256F7AC-BB30-40DB-9192-4A119185326D}"/>
+    <hyperlink ref="C45" r:id="rId30" display="https://fred.stlouisfed.org/series/CPILFESL" xr:uid="{E21097E4-8D83-4BF1-9073-13BE42C610B7}"/>
+    <hyperlink ref="C48" r:id="rId31" display="https://fred.stlouisfed.org/series/WPUFD49207" xr:uid="{410CEBD4-3C3F-475B-9553-56A53EF91BB0}"/>
+    <hyperlink ref="C49" r:id="rId32" display="https://fred.stlouisfed.org/series/WPSID61" xr:uid="{B75FCB2A-F435-42D5-8D35-204C532FA536}"/>
+    <hyperlink ref="C50" r:id="rId33" display="https://fred.stlouisfed.org/series/PRAWMINDEXM" xr:uid="{C0E282ED-0899-4B3A-86FF-98C43E5775E9}"/>
+    <hyperlink ref="C52" r:id="rId34" display="https://fred.stlouisfed.org/series/DCOILWTICO" xr:uid="{F1A9156C-0703-4BC3-B39C-517A9B265DD0}"/>
+    <hyperlink ref="C53" r:id="rId35" display="https://fred.stlouisfed.org/series/DCOILBRENTEU" xr:uid="{CF483AD0-D5FB-4A22-9DEF-484D0E95612F}"/>
+    <hyperlink ref="C54" r:id="rId36" display="https://fred.stlouisfed.org/series/DHHNGSP" xr:uid="{88B86E82-5D9B-4776-833C-909F33E6C54B}"/>
+    <hyperlink ref="C58" r:id="rId37" display="https://fred.stlouisfed.org/series/DHHNGSP" xr:uid="{943591D1-1D73-47A1-9A83-0E1AF8AC4439}"/>
+    <hyperlink ref="C59" r:id="rId38" display="https://fred.stlouisfed.org/series/PI" xr:uid="{9DD6436E-886F-4719-B40E-5FD007B13565}"/>
+    <hyperlink ref="C60" r:id="rId39" display="https://fred.stlouisfed.org/series/DSPI" xr:uid="{3B837FDB-F0B3-4586-B17E-E6796B136708}"/>
+    <hyperlink ref="C61" r:id="rId40" display="https://fred.stlouisfed.org/series/A229RX0" xr:uid="{02302EF8-7940-4160-AF62-D47CC30541C2}"/>
+    <hyperlink ref="C62" r:id="rId41" display="https://fred.stlouisfed.org/series/PSAVERT" xr:uid="{8BE68A31-104A-442B-A2B8-A74A6C8EAFDD}"/>
+    <hyperlink ref="C63" r:id="rId42" display="https://fred.stlouisfed.org/series/PCE" xr:uid="{8369BA7B-5662-414B-814E-2E6FD6086F5F}"/>
+    <hyperlink ref="C64" r:id="rId43" display="https://fred.stlouisfed.org/series/PCEC96" xr:uid="{0F0D13D3-863C-493C-90BB-062A829384F6}"/>
+    <hyperlink ref="C65" r:id="rId44" display="https://fred.stlouisfed.org/series/MRTSMPCSM44X72USS" xr:uid="{770DF185-FDDB-49D2-8412-233CFF911217}"/>
+    <hyperlink ref="C66" r:id="rId45" display="https://fred.stlouisfed.org/series/TOTALSL" xr:uid="{A9BF2B53-2BDD-45E3-8330-BDFB8B0732F0}"/>
+    <hyperlink ref="C67" r:id="rId46" display="https://fred.stlouisfed.org/series/PCEND" xr:uid="{85ED2ABD-A4C1-45BB-BC99-97A67F1B88EA}"/>
+    <hyperlink ref="C68" r:id="rId47" display="https://fred.stlouisfed.org/series/A22BVS" xr:uid="{951ABA3E-4094-4785-A558-AE47841707DE}"/>
+    <hyperlink ref="C71" r:id="rId48" display="https://fred.stlouisfed.org/series/M1SL" xr:uid="{34D91CB6-6D99-4449-81F4-0BAA7AD2C92E}"/>
+    <hyperlink ref="C72" r:id="rId49" display="https://fred.stlouisfed.org/series/M2SL" xr:uid="{500DFD36-FB9E-432A-87C7-546A417AF2BF}"/>
+    <hyperlink ref="C74" r:id="rId50" display="https://fred.stlouisfed.org/series/DTB3" xr:uid="{3F885799-5C4E-47E7-B954-67B61E26E1DF}"/>
+    <hyperlink ref="C75" r:id="rId51" display="https://fred.stlouisfed.org/series/DPRIME" xr:uid="{38058022-1D88-484E-BE41-C2FCE98F9918}"/>
+    <hyperlink ref="C76" r:id="rId52" display="https://fred.stlouisfed.org/series/DGS10" xr:uid="{28C15202-5804-415E-8E44-BAE5043F0DBC}"/>
+    <hyperlink ref="C79" r:id="rId53" display="https://fred.stlouisfed.org/series/DFII10" xr:uid="{5CAD2C86-6AF5-4A4B-8CC1-80051976EC1F}"/>
+    <hyperlink ref="C80" r:id="rId54" display="https://fred.stlouisfed.org/series/DGS30" xr:uid="{C04B69CD-E767-46ED-8A1D-D9CF73C5E567}"/>
+    <hyperlink ref="C82" r:id="rId55" display="https://fred.stlouisfed.org/series/DEXUSEU" xr:uid="{BF535801-C907-4FEF-8DD3-5A4FE097DE75}"/>
+    <hyperlink ref="C83" r:id="rId56" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{81EB876B-D4C6-4535-88B4-D7338E172E74}"/>
+    <hyperlink ref="C87" r:id="rId57" display="https://fred.stlouisfed.org/series/GDPC1" xr:uid="{A0E7E155-0622-499E-BB7B-38645B27FBDE}"/>
+    <hyperlink ref="C88" r:id="rId58" display="https://fred.stlouisfed.org/series/GDP" xr:uid="{A1FE3B70-28B7-4A04-A63B-22375805F0A0}"/>
+    <hyperlink ref="C89" r:id="rId59" display="https://fred.stlouisfed.org/series/PCEDG" xr:uid="{A9F276B3-4E19-4BE2-A18B-1C8079316E2A}"/>
+    <hyperlink ref="C90" r:id="rId60" display="https://fred.stlouisfed.org/series/PNFIC1" xr:uid="{738A177B-8D6B-4566-B679-C2D5170B7170}"/>
+    <hyperlink ref="C91" r:id="rId61" display="https://fred.stlouisfed.org/series/PRFIC1" xr:uid="{1012A88A-05D9-4DD4-BE33-968542F85281}"/>
+    <hyperlink ref="C92" r:id="rId62" display="https://fred.stlouisfed.org/series/CBI" xr:uid="{7E9C92B0-D1D9-4377-B1C6-A5F39F32E57E}"/>
+    <hyperlink ref="C93" r:id="rId63" display="https://fred.stlouisfed.org/series/NETEXC" xr:uid="{E1B9CD02-77DD-40C0-BEB1-9B4F8BA40D1C}"/>
+    <hyperlink ref="C94" r:id="rId64" display="https://fred.stlouisfed.org/series/IEABC" xr:uid="{53C4C190-F68D-4F7C-89A6-0A3064276ACF}"/>
+    <hyperlink ref="C73" r:id="rId65" display="https://fred.stlouisfed.org/series/BOPGSTB" xr:uid="{DD2F6DDA-69D5-4A5B-A844-C4BAA6490684}"/>
+    <hyperlink ref="C95" r:id="rId66" display="https://fred.stlouisfed.org/series/GCEC1" xr:uid="{01F44C24-AD61-4799-AD6F-387B8BA25AEC}"/>
+    <hyperlink ref="C96" r:id="rId67" display="https://fred.stlouisfed.org/series/EVACANTUSQ176N" xr:uid="{D7C8DCAB-1190-4CEE-904F-B68AE117241A}"/>
+    <hyperlink ref="C81" r:id="rId68" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{F3BB48CA-0BA3-40B2-9852-CE88BCC44408}"/>
+    <hyperlink ref="C78" r:id="rId69" display="https://fred.stlouisfed.org/series/DTWEXBGS" xr:uid="{31A20F8A-5F02-4AFA-A61C-ED85AA64101F}"/>
+    <hyperlink ref="C77" r:id="rId70" display="https://fred.stlouisfed.org/series/DGS10" xr:uid="{955E2DBE-4D20-4DC6-9E81-BBDC00DF6D5F}"/>
+    <hyperlink ref="C51" r:id="rId71" display="https://fred.stlouisfed.org/series/PRAWMINDEXM" xr:uid="{BD976A13-1C74-42EA-9EBE-2B27FCA2BC44}"/>
+    <hyperlink ref="C22" r:id="rId72" display="https://fred.stlouisfed.org/series/PAYEMS" xr:uid="{E38E0E90-6931-46F7-9FE0-24434F414B18}"/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.25" bottom="0.25" header="0.3" footer="0.3"/>
   <pageSetup scale="64" orientation="landscape" r:id="rId73"/>

</xml_diff>